<commit_message>
Reflect client feedback in Theme 1 workspaces
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="R9f387066fcab4cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="Rfa83b500d1094f25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="R4803b25c07704b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R267cefd24641429e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -237,13 +237,13 @@
     <xdr:ext cx="1905000" cy="1905000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="940fda70-7612-4001-9e8c-c091823a53cc"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4397ac9556174e9b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R04d73fb0ee294a4b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -857,7 +857,7 @@
       </x:c>
       <x:c r="H19" s="15" t="str"/>
     </x:row>
-    <x:row r="20" ht="144" hidden="0" customHeight="1">
+    <x:row r="20" ht="48" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
         <x:v>C09</x:v>
       </x:c>
@@ -871,17 +871,19 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>Review the selected seller and LOI; show award and acceptance status.</x:v>
+        <x:v>Review the selected seller and LOI, plus the required pre-award agreement gate; show agreement, award, and acceptance states.</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>BRD defines LOI as the award step; detailed document fields follow the approved LOI template.</x:v>
+        <x:v>Client requires agreements signed before award and introduction. This conflicts with the BRD LOI/contract order. Clarify agreement types, signatories, and sequence relative to LOI; status depends on that decision.</x:v>
       </x:c>
       <x:c r="G20" s="19" t="str">
-        <x:v>Ready for screen design</x:v>
-      </x:c>
-      <x:c r="H20" s="12" t="str"/>
-    </x:row>
-    <x:row r="21" ht="156" hidden="0" customHeight="1">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H20" s="12" t="str">
+        <x:v>Theme 1 feedback: agreements must be signed before award and introduction. Exact agreement scope/order added to client clarification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" hidden="0" customHeight="1">
       <x:c r="A21" s="15" t="str">
         <x:v>C10</x:v>
       </x:c>
@@ -898,14 +900,14 @@
         <x:v>Schedule and attend the approved introduction meeting after the required gate.</x:v>
       </x:c>
       <x:c r="F21" s="15" t="str">
-        <x:v>Provider choices, meeting-specific recording, consent, and disclosure timing depend on open policy decisions.</x:v>
+        <x:v>Required agreements must precede award and introduction per client feedback; exact agreement types/parties and the relationship to LOI remain open. Provider, recording, consent, and disclosure timing also remain open.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H21" s="15" t="str"/>
     </x:row>
-    <x:row r="22" ht="132" hidden="0" customHeight="1">
+    <x:row r="22" ht="36" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
         <x:v>C11</x:v>
       </x:c>
@@ -919,10 +921,10 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>Track agreement, delivery plan, project milestones, acceptance/rework, and close-out.</x:v>
+        <x:v>Track project agreement status, delivery plan, milestones, acceptance/rework, and close-out; enforce the approved agreement gate before award/introduction.</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>Milestone catalogue and amendment approvals remain open.</x:v>
+        <x:v>Agreement types and sequence relative to LOI need clarification. Milestone catalogue and amendment approvals remain open.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
         <x:v>Needs clarification</x:v>
@@ -953,7 +955,7 @@
       </x:c>
       <x:c r="H23" s="15" t="str"/>
     </x:row>
-    <x:row r="24" ht="108" hidden="0" customHeight="1">
+    <x:row r="24" ht="36" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
         <x:v>C13</x:v>
       </x:c>
@@ -967,10 +969,10 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>Rate the seller and provide feedback after the project.</x:v>
+        <x:v>Collect client feedback for each completed project and link it to the specific consultant or firm engagement.</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>Rating scale, visibility, moderation, and score effects remain open.</x:v>
+        <x:v>Rating scale, visibility, moderation, and whether feedback contributes to the composite/performance score or is displayed separately remain open.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
         <x:v>Needs clarification</x:v>
@@ -1001,7 +1003,7 @@
       </x:c>
       <x:c r="H25" s="15" t="str"/>
     </x:row>
-    <x:row r="26" ht="120" hidden="0" customHeight="1">
+    <x:row r="26" ht="36" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
         <x:v>E01</x:v>
       </x:c>
@@ -1015,16 +1017,16 @@
         <x:v>Consultant, Strategic Advisor, Project Manager</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>Show profile/certification progress, opportunities, active work, and required actions.</x:v>
+        <x:v>Show the role profile, score/certification progress, opportunities, and multiple active project assignments at the same time.</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>Visual hierarchy and summary cards are for client approval.</x:v>
+        <x:v>Visual hierarchy and workload summaries are for client approval; availability/capacity thresholds remain open.</x:v>
       </x:c>
       <x:c r="G26" s="17" t="str">
         <x:v>Pending client approval</x:v>
       </x:c>
       <x:c r="H26" s="12" t="str">
-        <x:v>Review OptimIQ_Consultant_Workspace_Concept.html; record client feedback here.</x:v>
+        <x:v>Theme 1 feedback: consultants may be active on multiple projects concurrently; show each assignment separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="180" hidden="0" customHeight="1">
@@ -1243,7 +1245,7 @@
       </x:c>
       <x:c r="H35" s="15" t="str"/>
     </x:row>
-    <x:row r="36" ht="156" hidden="0" customHeight="1">
+    <x:row r="36" ht="48" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
         <x:v>E11</x:v>
       </x:c>
@@ -1257,17 +1259,19 @@
         <x:v>Selected Expert</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>Review LOI, accept the award, and complete contract/onboarding steps.</x:v>
+        <x:v>Review the required agreements, LOI, award/acceptance status, and contract/onboarding steps.</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>BRD defines LOI acceptance as engagement creation; document contents follow approved templates.</x:v>
+        <x:v>Client requires agreements before award and introduction, while the BRD places LOI at award and contract signature after it. Clarify document types, signatories, and sequencing before finalising this screen.</x:v>
       </x:c>
       <x:c r="G36" s="19" t="str">
-        <x:v>Ready for screen design</x:v>
-      </x:c>
-      <x:c r="H36" s="12" t="str"/>
-    </x:row>
-    <x:row r="37" ht="120" hidden="0" customHeight="1">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H36" s="12" t="str">
+        <x:v>Theme 1 feedback added; sequence relative to BRD LOI/contract workflow remains open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="24" hidden="0" customHeight="1">
       <x:c r="A37" s="15" t="str">
         <x:v>E12</x:v>
       </x:c>
@@ -1281,17 +1285,17 @@
         <x:v>Engaged Expert</x:v>
       </x:c>
       <x:c r="E37" s="15" t="str">
-        <x:v>View delivery plan, assigned milestones, submissions, and payment progress.</x:v>
+        <x:v>View delivery plans, milestones, submissions, payment status, and separate workspaces for concurrent project assignments.</x:v>
       </x:c>
       <x:c r="F37" s="15" t="str">
-        <x:v>Milestone options and changes to agreed schedules remain open.</x:v>
+        <x:v>Milestone options and schedule changes remain open. Capacity thresholds for concurrent assignments remain open.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H37" s="15" t="str"/>
     </x:row>
-    <x:row r="38" ht="144" hidden="0" customHeight="1">
+    <x:row r="38" ht="36" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
         <x:v>E13</x:v>
       </x:c>
@@ -1305,10 +1309,10 @@
         <x:v>Expert account</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>Review ratings, performance history, CPD, and recertification actions.</x:v>
+        <x:v>Review client feedback and performance history separately for each project, alongside the approved composite score and certification state.</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>Performance-score method, rating rules, certificate validity, and renewal method remain open.</x:v>
+        <x:v>Whether client feedback updates the composite/performance score or is displayed as a separate signal remains open, as do rating scales, weights, aggregation, and moderation.</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
         <x:v>Needs clarification</x:v>
@@ -1437,7 +1441,7 @@
       </x:c>
       <x:c r="H43" s="15" t="str"/>
     </x:row>
-    <x:row r="44" ht="144" hidden="0" customHeight="1">
+    <x:row r="44" ht="48" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
         <x:v>F06</x:v>
       </x:c>
@@ -1454,7 +1458,7 @@
         <x:v>Conditionally reserve an Expert with consent; convert to engagement if the firm wins, release if it loses.</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>Reduced fee/linked-engagement rate remains open; reservation is not deployment.</x:v>
+        <x:v>Reduced fee/linked-engagement rate remains open; reservation is not deployment. Client feedback requires agreements before award and introduction; exact agreement scope/order relative to LOI remains open.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
         <x:v>Needs clarification</x:v>
@@ -1727,7 +1731,7 @@
       </x:c>
       <x:c r="H55" s="15" t="str"/>
     </x:row>
-    <x:row r="56" ht="144" hidden="0" customHeight="1">
+    <x:row r="56" ht="36" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
         <x:v>A10</x:v>
       </x:c>
@@ -1741,10 +1745,10 @@
         <x:v>Authorised configuration roles</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>Manage rating scales, visibility/moderation, performance signals, KPIs, and Reward &amp; Recognition.</x:v>
+        <x:v>Manage rating rules, per-project client feedback, performance signals, display/aggregation policy, and rewards through versioned proposals.</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>Rating effects, performance formula, KPI definitions, and reward criteria remain open.</x:v>
+        <x:v>Whether client feedback affects composite/performance scoring or appears separately remains open; rating scales, KPI definitions, and reward criteria also remain open.</x:v>
       </x:c>
       <x:c r="G56" s="14" t="str">
         <x:v>Needs clarification</x:v>
@@ -1838,7 +1842,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b1b5dec29554392"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1506bc6748f4e79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1858,13 +1862,13 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="32" t="str">
-        <x:v>OptimIQ Consultus | Proposed Portal Theme</x:v>
+        <x:v>OptimIQ Consultus | Theme 1 Review</x:v>
       </x:c>
       <x:c r="B1" s="31"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>Visual direction for client screen review; the theme itself is not approved until the client confirms it.</x:v>
+        <x:v>Theme 1 visual direction updated from the client workspace reference; screens remain pending explicit approval.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1875,28 +1879,28 @@
         <x:v>Proposal</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="28" t="str">
         <x:v>Theme name</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>OptimIQ Consultus — brand-led responsive application layout using the logo colors and uploaded portal example.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>Theme 1 — workspace design based on the client reference: deep evergreen sidebar, short OptimIQ mark with wordmark, light content area, and mint accents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="28" t="str">
         <x:v>Navigation</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>Fixed/collapsible deep-green left sidebar; highlight the active page; render menu sections from account type and active role.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>Deep evergreen, role-specific left navigation with the active workspace and page clearly highlighted; collapse to a compact mobile header with scrollable role-aware navigation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="28" t="str">
         <x:v>Main workspace</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
-        <x:v>Pale mint and soft-white canvas with white cards, clear page title and breadcrumbs, concise summaries, tables, and guided workflow panels.</x:v>
+        <x:v>Near-white content canvas, large breadcrumb/page heading, clear review banner, airy cards and project panels; stack content into one column on narrow screens.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1904,7 +1908,7 @@
         <x:v>Top bar</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>Use the supplied OptimIQ Consultus logo, active role/workspace switcher, page-level search where useful, notifications, help, and account menu.</x:v>
+        <x:v>Show the short OptimIQ mark and wordmark in the sidebar; keep active role/workspace, notifications, help, and account controls in the top bar.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1912,7 +1916,7 @@
         <x:v>Primary accent</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>Teal #2B8E79 — primary actions and selected states, sampled from the logo.</x:v>
+        <x:v>Teal #37A78A — primary actions and selection accents from the supplied Theme 1 reference.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1920,7 +1924,7 @@
         <x:v>Sidebar</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>Deep green #0F2E29 — logo-aligned navigation surface.</x:v>
+        <x:v>Deep evergreen #062F29 — sidebar and primary heading color.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1928,7 +1932,7 @@
         <x:v>Brand mint</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>Pale mint #DFF0EA — sampled from the logo background; use as a subtle brand surface.</x:v>
+        <x:v>Pale mint #DFF3EB — brand surface and selected-state support.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1936,7 +1940,7 @@
         <x:v>Canvas and cards</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>Soft white #F7FAF8 canvas; white cards with pale green borders #D5E7E0 and restrained separation.</x:v>
+        <x:v>Soft canvas #F5F8F6 and near-white main area #FBFCFB; white cards with subtle borders #DBE7E2.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1944,7 +1948,7 @@
         <x:v>Text</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
-        <x:v>Deep green #173C35 for primary text; muted green #55756D for secondary labels.</x:v>
+        <x:v>Deep green #092E28 for primary text; muted gray-green #71827D for secondary information.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1955,12 +1959,12 @@
         <x:v>Use restrained semantic colors: green for success, amber for needs attention, red for blocking/error; do not use color as the only signal.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="28" t="str">
         <x:v>Responsive behavior</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>Collapse or overlay the sidebar on narrow screens; keep the current role and page context visible.</x:v>
+        <x:v>At tablet/mobile widths, move the sidebar into a compact top section, allow horizontal navigation scrolling, stack cards and content grids, keep controls readable, and prevent page-level horizontal overflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -2012,7 +2016,7 @@
         <x:v>Approval boundary</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
-        <x:v>The four role workspace shells are concepts for visual review; they do not settle open workflow questions or approve all portal screens. Record feedback in the Screen Inventory tab. Further implementation HTML follows approval of the corresponding screen designs.</x:v>
+        <x:v>The four role workspaces are client-review concepts; screens remain pending explicit approval. Record client feedback in this workbook. Agreement sequencing and feedback scoring details remain clarification items; agreed page layouts can proceed while these flow details are labelled open.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -2020,7 +2024,7 @@
         <x:v>Client review mockups</x:v>
       </x:c>
       <x:c r="B24" s="11" t="str">
-        <x:v>Open OptimIQ_Portal_Demo_Index.html for links to the Client, Consultant, Consulting Firm, and Staff/Admin concepts.</x:v>
+        <x:v>Open index.html for links to the Client, Consultant, Consulting Firm, and Staff/Admin concepts.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -2031,14 +2035,16 @@
         <x:v>Pending client approval across the four role workspace concepts.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="24" hidden="0" customHeight="1">
+    <x:row r="26" ht="36" hidden="0" customHeight="1">
       <x:c r="A26" s="11" t="str">
         <x:v>Client feedback / requested changes</x:v>
       </x:c>
-      <x:c r="B26" s="11" t="str"/>
+      <x:c r="B26" s="11" t="str">
+        <x:v>Client Theme 1 feedback (2026-10-20): required agreements must be signed before award and introduction. Consultant profiles may have multiple concurrent project assignments. Capture feedback per project; whether it contributes to the composite/performance score or appears separately remains open. Agreement type/signatories/sequence conflicts with the BRD LOI and contract order and needs clarification.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf7cbfbf71a64763"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21943529d2244d16"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add portal sign-in review screen
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="R4803b25c07704b18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R267cefd24641429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="R150f23b85354435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R96081ee0edc14075"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -243,7 +243,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R04d73fb0ee294a4b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rece095b6118f4f72"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -495,7 +495,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>Client review tracker — includes four role workspace concepts for review; no screen has client approval yet.</x:v>
+        <x:v>Client review tracker — Theme 1 is approved; the shared sign-in and four role workspaces are tracked for screen-level review.</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -584,12 +584,14 @@
         <x:v>Single entry point for every account type; after authentication, route to authorised workspace and active role.</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Sign-in method, MFA/OTP use, and recovery flow are not defined. Existing website email OTP is verification, not necessarily portal login.</x:v>
+        <x:v>CTA registration performs email verification and password setup; portal sign-in uses those credentials. Account-recovery flow remains open for developer confirmation.</x:v>
       </x:c>
       <x:c r="G8" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H8" s="12" t="str"/>
+      <x:c r="H8" s="12" t="str">
+        <x:v>Sign-in concept created at /login/. Existing CTA registration pages are outside this redesign scope and must not be changed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="108" hidden="0" customHeight="1">
       <x:c r="A9" s="15" t="str">
@@ -1842,7 +1844,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1506bc6748f4e79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88416a6bc2f94f94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2045,6 +2047,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21943529d2244d16"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86af5b69032942cb"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record consultant CTQ scoring clarification
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="R150f23b85354435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R96081ee0edc14075"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="Re9ba93e14fce4487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R742acf56f9fb4aa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -243,7 +243,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rece095b6118f4f72"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R69495489ec644ef6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1042,18 +1042,20 @@
         <x:v>Expert role profile switcher</x:v>
       </x:c>
       <x:c r="D27" s="15" t="str">
-        <x:v>Three Expert role profiles</x:v>
+        <x:v>One candidate with three role-specific scores and project assignments</x:v>
       </x:c>
       <x:c r="E27" s="15" t="str">
-        <x:v>Switch between Consultant, Strategic Advisor, and Project Manager profiles; each has its own score and certification state.</x:v>
+        <x:v>Review role results and active assignments; Consultant, Strategic Advisor, and Project Manager roles can apply to different concurrent projects.</x:v>
       </x:c>
       <x:c r="F27" s="15" t="str">
-        <x:v>The three role profiles are confirmed; interaction treatment is for client approval.</x:v>
+        <x:v>How to add a role after CTA registration remains open for client clarification.</x:v>
       </x:c>
       <x:c r="G27" s="19" t="str">
         <x:v>Ready for screen design</x:v>
       </x:c>
-      <x:c r="H27" s="15" t="str"/>
+      <x:c r="H27" s="15" t="str">
+        <x:v>Client clarification (2026-10-20): the same candidate can be Consultant on Project A and Strategic Advisor on Project B at the same time. Role assignment is per project.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="156" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
@@ -1090,18 +1092,20 @@
         <x:v>CTQ assessment stepper</x:v>
       </x:c>
       <x:c r="D29" s="15" t="str">
-        <x:v>Three role-specific variants</x:v>
+        <x:v>Shared CTQ question set across all three Expert roles</x:v>
       </x:c>
       <x:c r="E29" s="15" t="str">
-        <x:v>Complete the approved eight-step, 36-field CTQ form; all answers remain editable until final submission.</x:v>
+        <x:v>Complete the same eight-step, 36-field CTQ form once. Calculate separate Consultant, Strategic Advisor, and Project Manager scores using each role’s approved weighting; show suitable other-role recommendations.</x:v>
       </x:c>
       <x:c r="F29" s="15" t="str">
-        <x:v>Role-specific data is sourced from the client-approved CTQ workbooks; post-submit reopening is open.</x:v>
+        <x:v>Use the approved role-specific weightings from the client CTQ model. Show scores after final submission; do not ask the candidate to answer duplicate forms.</x:v>
       </x:c>
       <x:c r="G29" s="19" t="str">
-        <x:v>Ready for screen design</x:v>
-      </x:c>
-      <x:c r="H29" s="15" t="str"/>
+        <x:v>Pending client approval</x:v>
+      </x:c>
+      <x:c r="H29" s="15" t="str">
+        <x:v>Client clarification (2026-10-20): identical CTQ fields for all three roles, different weightings and three separate scores per candidate; role-fit recommendations may identify other suitable roles. CTQ stepper updated.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="156" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
@@ -1114,18 +1118,20 @@
         <x:v>Score and tier summary</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>Each Expert role profile</x:v>
+        <x:v>Three role-specific CTQ scores and overall composite/tier</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>Show CTQ component, approved composite components, current score/tier, and progression status.</x:v>
+        <x:v>Show the three separate role CTQ scores and role-fit recommendations. Keep each role CTQ result distinct from the overall composite score and tier.</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>A+B1+B2+C+D+E weights and certification bands are approved; visual presentation is for client approval.</x:v>
+        <x:v>Client feedback treatment within the composite/performance score remains open separately.</x:v>
       </x:c>
       <x:c r="G30" s="19" t="str">
-        <x:v>Ready for screen design</x:v>
-      </x:c>
-      <x:c r="H30" s="12" t="str"/>
+        <x:v>Pending client approval</x:v>
+      </x:c>
+      <x:c r="H30" s="12" t="str">
+        <x:v>Updated consultant workspace to show three CTQ scores and a project-by-project role assignment example.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="132" hidden="0" customHeight="1">
       <x:c r="A31" s="15" t="str">
@@ -1844,7 +1850,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88416a6bc2f94f94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d98fdeae93144b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2026,7 +2032,7 @@
         <x:v>Client review mockups</x:v>
       </x:c>
       <x:c r="B24" s="11" t="str">
-        <x:v>Open index.html for links to the Client, Consultant, Consulting Firm, and Staff/Admin concepts.</x:v>
+        <x:v>Open index.html. Each audience section links to its existing CTA form first, then the shared portal sign-in and relevant workspace screens.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -2034,7 +2040,7 @@
         <x:v>Theme approval status</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
-        <x:v>Pending client approval across the four role workspace concepts.</x:v>
+        <x:v>Theme 1 approved by client. Individual portal screens are reviewed and approved separately; statuses are shown on the review index and Screen Inventory.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="36" hidden="0" customHeight="1">
@@ -2042,11 +2048,12 @@
         <x:v>Client feedback / requested changes</x:v>
       </x:c>
       <x:c r="B26" s="11" t="str">
-        <x:v>Client Theme 1 feedback (2026-10-20): required agreements must be signed before award and introduction. Consultant profiles may have multiple concurrent project assignments. Capture feedback per project; whether it contributes to the composite/performance score or appears separately remains open. Agreement type/signatories/sequence conflicts with the BRD LOI and contract order and needs clarification.</x:v>
+        <x:v>Client Theme 1 feedback (2026-10-20): required agreements must be signed before award and introduction. Consultant profiles may have multiple concurrent project assignments. Capture feedback per project; whether it contributes to the composite/performance score or appears separately remains open. Agreement type/signatories/sequence conflicts with the BRD LOI and contract order and needs clarification.
+Client CTQ and role feedback (2026-10-20): the Consultant, Strategic Advisor, and Project Manager use the same CTQ fields, answered once, with different role-specific weightings producing three separate CTQ scores. The system may recommend other suitable roles. Project role is assigned per engagement, so one candidate may be Consultant on Project A and Strategic Advisor on Project B concurrently. Existing Client, Consultant, and Consulting Firm CTA forms are directly linked in their respective review journeys. Post-registration role addition remains open for client clarification.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86af5b69032942cb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14706378bd304427"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add post-CTQ consultant role fit selection screen
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="Re9ba93e14fce4487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R742acf56f9fb4aa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="Raa80df8488ec4033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="Rc151f921cd434a01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -243,7 +243,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R69495489ec644ef6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd2f7609a3cb34681"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1092,19 +1092,19 @@
         <x:v>CTQ assessment stepper</x:v>
       </x:c>
       <x:c r="D29" s="15" t="str">
-        <x:v>Shared CTQ question set across all three Expert roles</x:v>
+        <x:v>All three consultant roles; shared CTQ form</x:v>
       </x:c>
       <x:c r="E29" s="15" t="str">
-        <x:v>Complete the same eight-step, 36-field CTQ form once. Calculate separate Consultant, Strategic Advisor, and Project Manager scores using each role’s approved weighting; show suitable other-role recommendations.</x:v>
+        <x:v>Complete one eight-step, 36-field form. Do not show scores or weightings. After submission, evaluate the single answer set in the backend for role-fit results.</x:v>
       </x:c>
       <x:c r="F29" s="15" t="str">
-        <x:v>Use the approved role-specific weightings from the client CTQ model. Show scores after final submission; do not ask the candidate to answer duplicate forms.</x:v>
+        <x:v>Exact numeric scores and weightings remain internal. Fit categories appear on the next screen.</x:v>
       </x:c>
       <x:c r="G29" s="19" t="str">
         <x:v>Pending client approval</x:v>
       </x:c>
       <x:c r="H29" s="15" t="str">
-        <x:v>Client clarification (2026-10-20): identical CTQ fields for all three roles, different weightings and three separate scores per candidate; role-fit recommendations may identify other suitable roles. CTQ stepper updated.</x:v>
+        <x:v>Design updated (2026-10-20): one shared CTQ form, no score or weighting shown; backend determines fit categories after submission.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="156" hidden="0" customHeight="1">
@@ -1115,22 +1115,22 @@
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>Score and tier summary</x:v>
+        <x:v>Role-fit results &amp; role selection</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>Three role-specific CTQ scores and overall composite/tier</x:v>
+        <x:v>Consultant, Strategic Advisor, Project Manager</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>Show the three separate role CTQ scores and role-fit recommendations. Keep each role CTQ result distinct from the overall composite score and tier.</x:v>
+        <x:v>After CTQ submission, show a qualitative fit category for each role and let the consultant select one or multiple suitable roles.</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>Client feedback treatment within the composite/performance score remains open separately.</x:v>
+        <x:v>Whether Low-fit roles can be selected and whether confirmed role choices can be changed later remain open for client clarification.</x:v>
       </x:c>
       <x:c r="G30" s="19" t="str">
         <x:v>Pending client approval</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>Updated consultant workspace to show three CTQ scores and a project-by-project role assignment example.</x:v>
+        <x:v>Illustrative results: Best fit Consultant, Moderate fit Strategic Advisor, Low fit Project Manager. Consultant starts selected; low-fit Project Manager is shown but disabled pending clarification. Candidate may keep one role or add a suitable role.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="132" hidden="0" customHeight="1">
@@ -1850,7 +1850,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d98fdeae93144b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e3f50a0463e48bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2054,6 +2054,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14706378bd304427"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8c1adaf0c274e42"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add consultant lifecycle review screens and client feedback
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="Raa80df8488ec4033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="Rc151f921cd434a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen Inventory" sheetId="1" r:id="Re96a55a6293d4818"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="2" r:id="R66bb6c0cf3ba4ec8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +109,16 @@
         <x:fgColor rgb="FFDFF0EA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF5EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border>
@@ -142,7 +152,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -218,6 +228,18 @@
     <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -243,7 +265,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd2f7609a3cb34681"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R40b7cc6d9f7443a9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -258,7 +280,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PortalScreenInventory" displayName="PortalScreenInventory" ref="A7:H59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PortalScreenInventory" displayName="PortalScreenInventory" ref="A7:H66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Screen ID"/>
     <x:tableColumn id="2" name="Workspace"/>
@@ -1147,15 +1169,17 @@
         <x:v>Each Expert role profile</x:v>
       </x:c>
       <x:c r="E31" s="15" t="str">
-        <x:v>Show M1–M7 assessment steps, outcomes, evidence requests, and certification progress.</x:v>
+        <x:v>Show progress across the complete composite assessment: CTQ; domain and behavioral assessments (third party); work-quality evaluation; case studies/client impact; client testimonials/references; and committee interview, once its role is confirmed. Show actions/status, not numeric scores or weights.</x:v>
       </x:c>
       <x:c r="F31" s="15" t="str">
-        <x:v>External certifying organisation identity/role and full recertification process remain open.</x:v>
+        <x:v>Committee interview role is not allocated in the previously approved six-component 100% model. Confirm whether it is evidence in an existing component, a certification gate, or a new weighted component and whether weights change.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H31" s="15" t="str"/>
+      <x:c r="H31" s="15" t="str">
+        <x:v>Client feedback 2026-10-23 incorporated; preserve approved six-component formula pending committee-interview decision.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="108" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
@@ -1213,21 +1237,23 @@
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>Opportunity list</x:v>
+        <x:v>Consultant opportunities and project details</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>Certified Expert</x:v>
+        <x:v>Certified Consultant</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>Review eligible opportunities routed through OptimIQ.</x:v>
+        <x:v>Review masked opportunities matched to selected roles; inspect project details and express interest or submit a bid/quotation before project agreement and award.</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>Matching factors and weights are open; only approved, explainable recommendations should be shown.</x:v>
+        <x:v>Matching/recommendation criteria, bid/quote fields and commercial terms remain open.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H34" s="12" t="str"/>
+      <x:c r="H34" s="12" t="str">
+        <x:v>Consultant opportunities concept added; client review needed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="120" hidden="0" customHeight="1">
       <x:c r="A35" s="15" t="str">
@@ -1237,21 +1263,23 @@
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C35" s="15" t="str">
-        <x:v>Opportunity detail and bid/quote</x:v>
+        <x:v>Opportunity response and bid / quotation</x:v>
       </x:c>
       <x:c r="D35" s="15" t="str">
-        <x:v>Certified Expert</x:v>
+        <x:v>Certified Consultant</x:v>
       </x:c>
       <x:c r="E35" s="15" t="str">
-        <x:v>Review masked client/project details and submit a bid or quotation through OptimIQ.</x:v>
+        <x:v>Prepare a role-specific project response with availability, proposed approach, and configured bid/quotation details.</x:v>
       </x:c>
       <x:c r="F35" s="15" t="str">
-        <x:v>Commercial terms, bid support fees, and exact opportunity details remain open.</x:v>
+        <x:v>Commercial terms, bid support fee, workflow, and identity-release point remain open.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H35" s="15" t="str"/>
+      <x:c r="H35" s="15" t="str">
+        <x:v>Included in the Consultant Opportunities &amp; Project Details screen.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="48" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
@@ -1261,22 +1289,22 @@
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>LOI, contract, and engagement</x:v>
+        <x:v>Project agreement gate before award</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>Selected Expert</x:v>
+        <x:v>Selected Expert / Consultant</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>Review the required agreements, LOI, award/acceptance status, and contract/onboarding steps.</x:v>
+        <x:v>Show required project agreements for review and signature before project award and before Client-Consultant introduction. Award and introduction remain gated until required signatures are recorded.</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>Client requires agreements before award and introduction, while the BRD places LOI at award and contract signature after it. Clarify document types, signatories, and sequencing before finalising this screen.</x:v>
+        <x:v>Agreement types, signatories, and sequence conflict with the BRD LOI/contract workflow; clarify the final order before implementation.</x:v>
       </x:c>
       <x:c r="G36" s="19" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H36" s="12" t="str">
-        <x:v>Theme 1 feedback added; sequence relative to BRD LOI/contract workflow remains open.</x:v>
+        <x:v>Updated to reflect client requirement that agreements are signed before award and introduction; screen concept available for review.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="24" hidden="0" customHeight="1">
@@ -1287,21 +1315,23 @@
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C37" s="15" t="str">
-        <x:v>Delivery and milestone workspace</x:v>
+        <x:v>Engagements and delivery workspace</x:v>
       </x:c>
       <x:c r="D37" s="15" t="str">
-        <x:v>Engaged Expert</x:v>
+        <x:v>Engaged Expert / Consultant</x:v>
       </x:c>
       <x:c r="E37" s="15" t="str">
-        <x:v>View delivery plans, milestones, submissions, payment status, and separate workspaces for concurrent project assignments.</x:v>
+        <x:v>Define an Engagement as an OptimIQ project assignment after applicable award/acceptance steps. Support multiple concurrent assignments, each with its own role, status, milestones, and feedback. Separate active and completed OptimIQ work.</x:v>
       </x:c>
       <x:c r="F37" s="15" t="str">
-        <x:v>Milestone options and schedule changes remain open. Capacity thresholds for concurrent assignments remain open.</x:v>
+        <x:v>Confirm engagement records, project history retention, capacity rules for concurrent work, and milestone changes.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H37" s="15" t="str"/>
+        <x:v>Awaiting client feedback</x:v>
+      </x:c>
+      <x:c r="H37" s="15" t="str">
+        <x:v>Clarified distinction: prior/outside-OptimIQ work belongs to Past Project Experience, not Engagements.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="36" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
@@ -1314,18 +1344,20 @@
         <x:v>Performance, CPD, ratings, renewal</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>Expert account</x:v>
+        <x:v>Expert account / Consultant</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>Review client feedback and performance history separately for each project, alongside the approved composite score and certification state.</x:v>
+        <x:v>Review client feedback separately by engagement and manage Continuing Professional Development (CPD) records. CPD means ongoing learning and professional development activity.</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>Whether client feedback updates the composite/performance score or is displayed as a separate signal remains open, as do rating scales, weights, aggregation, and moderation.</x:v>
+        <x:v>Does feedback affect composite/performance score or remain a separate signal, and how is it aggregated? Confirm CPD units/evidence, validation, and renewal/certification effect.</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H38" s="12" t="str"/>
+      <x:c r="H38" s="12" t="str">
+        <x:v>Client feedback 2026-10-23: added feedback-per-project and CPD definition; scoring and CPD operating rules remain open.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="120" hidden="0" customHeight="1">
       <x:c r="A39" s="15" t="str">
@@ -1834,6 +1866,188 @@
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H59" s="15" t="str"/>
+    </x:row>
+    <x:row r="60" ht="112" customHeight="1">
+      <x:c r="A60" s="33" t="str">
+        <x:v>E14</x:v>
+      </x:c>
+      <x:c r="B60" s="33" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C60" s="33" t="str">
+        <x:v>Profile and assessment progress</x:v>
+      </x:c>
+      <x:c r="D60" s="33" t="str">
+        <x:v>Consultant account</x:v>
+      </x:c>
+      <x:c r="E60" s="33" t="str">
+        <x:v>Allow ongoing profile updates and show status of CTQ and the remaining composite assessment components without showing numeric scores or weights. Score-affecting edits follow evidence and authorised review before recalculation.</x:v>
+      </x:c>
+      <x:c r="F60" s="33" t="str">
+        <x:v>Which changed profile fields are material, what evidence/approvals apply, and what status/score is shown while review is pending?</x:v>
+      </x:c>
+      <x:c r="G60" s="34" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H60" s="33" t="str">
+        <x:v>Consultant can update profile over time; score recalculation follows evidence and review rules in BRD v3.2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="112" customHeight="1">
+      <x:c r="A61" s="35" t="str">
+        <x:v>E15</x:v>
+      </x:c>
+      <x:c r="B61" s="35" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C61" s="35" t="str">
+        <x:v>OptimIQ engagement history</x:v>
+      </x:c>
+      <x:c r="D61" s="35" t="str">
+        <x:v>Consultant account</x:v>
+      </x:c>
+      <x:c r="E61" s="35" t="str">
+        <x:v>View active and completed OptimIQ project assignments separately. A Consultant can work on multiple engagements at the same time. Past Project Experience remains a separate profile section for prior/outside-OptimIQ work.</x:v>
+      </x:c>
+      <x:c r="F61" s="35" t="str">
+        <x:v>Confirm fields, history retention, and concurrent capacity rules.</x:v>
+      </x:c>
+      <x:c r="G61" s="36" t="str">
+        <x:v>Awaiting client feedback</x:v>
+      </x:c>
+      <x:c r="H61" s="35" t="str">
+        <x:v>Terminology clarified from client discussion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="112" customHeight="1">
+      <x:c r="A62" s="33" t="str">
+        <x:v>E16</x:v>
+      </x:c>
+      <x:c r="B62" s="33" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C62" s="33" t="str">
+        <x:v>Payments and invoices</x:v>
+      </x:c>
+      <x:c r="D62" s="33" t="str">
+        <x:v>Consultant account / each engagement</x:v>
+      </x:c>
+      <x:c r="E62" s="33" t="str">
+        <x:v>Show payment and invoice status in the project context with a Consultant-level payout overview. Keep invoices payable to OptimIQ distinct from payouts owed by OptimIQ to the Consultant; hide internal margins/commission.</x:v>
+      </x:c>
+      <x:c r="F62" s="33" t="str">
+        <x:v>Who issues each invoice, who pays whom, whether Consultant invoices or OptimIQ pays by milestone, and visible records/timing.</x:v>
+      </x:c>
+      <x:c r="G62" s="34" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H62" s="33" t="str">
+        <x:v>New Consultant screen concept created.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="112" customHeight="1">
+      <x:c r="A63" s="35" t="str">
+        <x:v>E17</x:v>
+      </x:c>
+      <x:c r="B63" s="35" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C63" s="35" t="str">
+        <x:v>Communications and notifications</x:v>
+      </x:c>
+      <x:c r="D63" s="35" t="str">
+        <x:v>Consultant account</x:v>
+      </x:c>
+      <x:c r="E63" s="35" t="str">
+        <x:v>Provide an OptimIQ-provisioned @optimiqconsultus.com mailbox within the portal, project communications, and in-portal notifications for new emails/messages; support chat and WhatsApp integrations as approved.</x:v>
+      </x:c>
+      <x:c r="F63" s="35" t="str">
+        <x:v>Mailbox provider and lifecycle, inbound/outbound email, messaging/WhatsApp provider, contact masking, retention, notification events and user controls.</x:v>
+      </x:c>
+      <x:c r="G63" s="36" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H63" s="35" t="str">
+        <x:v>New Consultant screen concept created; client requested email, chat, WhatsApp, and notifications.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="112" customHeight="1">
+      <x:c r="A64" s="33" t="str">
+        <x:v>E18</x:v>
+      </x:c>
+      <x:c r="B64" s="33" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C64" s="33" t="str">
+        <x:v>Project calendar</x:v>
+      </x:c>
+      <x:c r="D64" s="33" t="str">
+        <x:v>Consultant account / each engagement</x:v>
+      </x:c>
+      <x:c r="E64" s="33" t="str">
+        <x:v>Show project-related milestones, meetings, and due dates across concurrent engagements.</x:v>
+      </x:c>
+      <x:c r="F64" s="33" t="str">
+        <x:v>Event types, reminders/invitations, and external calendar synchronization/provider.</x:v>
+      </x:c>
+      <x:c r="G64" s="34" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H64" s="33" t="str">
+        <x:v>New Consultant screen concept created.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="112" customHeight="1">
+      <x:c r="A65" s="35" t="str">
+        <x:v>E19</x:v>
+      </x:c>
+      <x:c r="B65" s="35" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C65" s="35" t="str">
+        <x:v>Project documents and knowledge library · Phase 2</x:v>
+      </x:c>
+      <x:c r="D65" s="35" t="str">
+        <x:v>Consultant and authorised Client users</x:v>
+      </x:c>
+      <x:c r="E65" s="35" t="str">
+        <x:v>Provide project folders, documents, Consultant comments, and controlled Client access. Future searchable OptimIQ knowledge resources may include approved project summaries, success stories, and testimonials.</x:v>
+      </x:c>
+      <x:c r="F65" s="35" t="str">
+        <x:v>Folder permissions, versions, downloads, comments, retention/deletion, consent, privacy/anonymisation, and publication/withdrawal approval.</x:v>
+      </x:c>
+      <x:c r="G65" s="36" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H65" s="35" t="str">
+        <x:v>Phase 2 concept only; not an initial release commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="112" customHeight="1">
+      <x:c r="A66" s="33" t="str">
+        <x:v>E20</x:v>
+      </x:c>
+      <x:c r="B66" s="33" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C66" s="33" t="str">
+        <x:v>Performance and Continuing Professional Development</x:v>
+      </x:c>
+      <x:c r="D66" s="33" t="str">
+        <x:v>Consultant account</x:v>
+      </x:c>
+      <x:c r="E66" s="33" t="str">
+        <x:v>Review project feedback separately and record ongoing learning/professional development activity (CPD).</x:v>
+      </x:c>
+      <x:c r="F66" s="33" t="str">
+        <x:v>Whether feedback changes the composite/performance score, feedback aggregation/moderation, CPD evidence/units/validation and certification impact.</x:v>
+      </x:c>
+      <x:c r="G66" s="34" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H66" s="33" t="str">
+        <x:v>New Consultant screen concept created; CPD acronym expanded and operating rules open.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1850,7 +2064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e3f50a0463e48bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac8e63816944264"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1900,7 +2114,7 @@
         <x:v>Navigation</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>Deep evergreen, role-specific left navigation with the active workspace and page clearly highlighted; collapse to a compact mobile header with scrollable role-aware navigation.</x:v>
+        <x:v>Desktop: persistent role-aware left sidebar. Mobile: same vertical navigation in a left-edge drawer with an explicit menu control; avoid horizontal scrolling navigation.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -2049,11 +2263,12 @@
       </x:c>
       <x:c r="B26" s="11" t="str">
         <x:v>Client Theme 1 feedback (2026-10-20): required agreements must be signed before award and introduction. Consultant profiles may have multiple concurrent project assignments. Capture feedback per project; whether it contributes to the composite/performance score or appears separately remains open. Agreement type/signatories/sequence conflicts with the BRD LOI and contract order and needs clarification.
-Client CTQ and role feedback (2026-10-20): the Consultant, Strategic Advisor, and Project Manager use the same CTQ fields, answered once, with different role-specific weightings producing three separate CTQ scores. The system may recommend other suitable roles. Project role is assigned per engagement, so one candidate may be Consultant on Project A and Strategic Advisor on Project B concurrently. Existing Client, Consultant, and Consulting Firm CTA forms are directly linked in their respective review journeys. Post-registration role addition remains open for client clarification.</x:v>
+Client CTQ and role feedback (2026-10-20): the Consultant, Strategic Advisor, and Project Manager use the same CTQ fields, answered once, with different role-specific weightings producing three separate CTQ scores. The system may recommend other suitable roles. Project role is assigned per engagement, so one candidate may be Consultant on Project A and Strategic Advisor on Project B concurrently. Existing Client, Consultant, and Consulting Firm CTA forms are directly linked in their respective review journeys. Post-registration role addition remains open for client clarification.
+Consultant feedback (2026-10-23): standardise typography across Theme 1; define Engagements as OptimIQ project assignments separate from past experience; expand CPD as Continuing Professional Development; show project-linked invoices/payments without internal OptimIQ margins; add the requested OptimIQ mailbox, chat/WhatsApp, and email/message notifications; add a project calendar; mark project folders, Client access, consultant comments, and a future knowledge/success-story library as Phase 2. Preserve the approved six-component composite scoring model. Committee interview scoring role, feedback's effect on score, rescoring triggers, billing flow, mailbox/messaging providers, calendar sync, CPD rules, and Phase 2 access/publication controls remain open. Consultant pages and requirements documents updated together; source BRD in sources remains unchanged.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8c1adaf0c274e42"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae70f1998ef4c29"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add client portal review journey
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6c361a7197fb4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="R523b217a287e477e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="R632d8654190c45f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R675671ee488a4915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="R57edd802f23d461c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="R454c55e724ae4034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R04267e3fa06a48e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R603bccc1c7b64f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra7a0332978874fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="Ra122d669da6b4167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="Rc47f273e17304fd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="Ra04e35f5c0da4968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="R6c20df2caf3e47ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="Rc293edcafd1f4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R908d55a2ba1347eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R99b8de0385fd4a4c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -72,7 +72,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +97,51 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF06352E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F4ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF27836E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF06352E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F4ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF27836E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF06352E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F4ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF27836E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -186,7 +231,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="61">
+  <x:cellXfs count="85">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -296,6 +341,42 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -577,10 +658,10 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="B8" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Preserved for the next streamlined design pass.</x:v>
+        <x:v>Client lifecycle mapped from BRD C1–C8 and the approved categorisation workbook.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -588,7 +669,7 @@
         <x:v>Staff Admin</x:v>
       </x:c>
       <x:c r="B9" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
         <x:v>Existing staff/admin inventory preserved.</x:v>
@@ -602,7 +683,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>17 consulting firm clarification items; other audience questions remain in their own tabs.</x:v>
+        <x:v>17 consulting firm and 18 client clarification items.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2116,66 +2197,66 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="60" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="50" t="str">
+      <x:c r="A1" s="78" t="str">
         <x:v>Client · Screen Approval Inventory</x:v>
       </x:c>
-      <x:c r="B1" s="50"/>
-      <x:c r="C1" s="50"/>
-      <x:c r="D1" s="50"/>
-      <x:c r="E1" s="50"/>
-      <x:c r="F1" s="50"/>
-      <x:c r="G1" s="50"/>
-      <x:c r="H1" s="50"/>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="53" t="str">
-        <x:v>Client journey preserved for the next design pass. Open flow decisions remain flagged; this update does not redesign Client screens.</x:v>
-      </x:c>
-      <x:c r="B2" s="53"/>
-      <x:c r="C2" s="53"/>
-      <x:c r="D2" s="53"/>
-      <x:c r="E2" s="53"/>
-      <x:c r="F2" s="53"/>
-      <x:c r="G2" s="53"/>
-      <x:c r="H2" s="53"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="56" t="str">
+      <x:c r="B1" s="78"/>
+      <x:c r="C1" s="78"/>
+      <x:c r="D1" s="78"/>
+      <x:c r="E1" s="78"/>
+      <x:c r="F1" s="78"/>
+      <x:c r="G1" s="78"/>
+      <x:c r="H1" s="78"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="81" t="str">
+        <x:v>Client lifecycle based on BRD C1–C8 and the approved Client Categorisation workbook. Internal scores/segments remain hidden. Shared Theme 1 components align to Consultant and Consulting Firm.</x:v>
+      </x:c>
+      <x:c r="B2" s="81"/>
+      <x:c r="C2" s="81"/>
+      <x:c r="D2" s="81"/>
+      <x:c r="E2" s="81"/>
+      <x:c r="F2" s="81"/>
+      <x:c r="G2" s="81"/>
+      <x:c r="H2" s="81"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="84" t="str">
         <x:v>Screen ID</x:v>
       </x:c>
-      <x:c r="B4" s="56" t="str">
+      <x:c r="B4" s="84" t="str">
         <x:v>Workspace</x:v>
       </x:c>
-      <x:c r="C4" s="56" t="str">
+      <x:c r="C4" s="84" t="str">
         <x:v>Screen / design unit</x:v>
       </x:c>
-      <x:c r="D4" s="56" t="str">
+      <x:c r="D4" s="84" t="str">
         <x:v>Roles / variants</x:v>
       </x:c>
-      <x:c r="E4" s="56" t="str">
+      <x:c r="E4" s="84" t="str">
         <x:v>Purpose and client review focus</x:v>
       </x:c>
-      <x:c r="F4" s="56" t="str">
+      <x:c r="F4" s="84" t="str">
         <x:v>Clarification to park</x:v>
       </x:c>
-      <x:c r="G4" s="56" t="str">
+      <x:c r="G4" s="84" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H4" s="56" t="str">
+      <x:c r="H4" s="84" t="str">
         <x:v>Client decision / notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="62" customHeight="1">
+    <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>C01</x:v>
       </x:c>
@@ -2183,23 +2264,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Client home dashboard</x:v>
+        <x:v>Client CTA enquiry</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Client account</x:v>
+        <x:v>Client / existing public form</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Overview of active requirements, shortlist actions, engagements, invoices, and next steps.</x:v>
+        <x:v>Existing For Clients form; link as-is and do not redesign.</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>Exact dashboard metrics and client segments are not final.</x:v>
+        <x:v>None for this screen; its relationship to portal account creation is in CL-01.</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6" ht="62" customHeight="1">
+        <x:v>Existing CTA form</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Linked directly from the client review page.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="13" t="str">
         <x:v>C02</x:v>
       </x:c>
@@ -2207,23 +2290,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C6" s="13" t="str">
-        <x:v>Client organisation profile</x:v>
+        <x:v>Optional client details / categorisation enrichment</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
-        <x:v>Client account</x:v>
+        <x:v>Client / optional pre-login step</x:v>
       </x:c>
       <x:c r="E6" s="13" t="str">
-        <x:v>View and maintain organisation details, contacts, categories, and declarations.</x:v>
+        <x:v>Three optional fields: project budget, preferred start timeline, decision-making role. Skip is always available.</x:v>
       </x:c>
       <x:c r="F6" s="13" t="str">
-        <x:v>Client category names/bands and final organisation fields remain open.</x:v>
+        <x:v>Whether the step opens from the confirmation page or email link is a presentation detail; client scoring precision is CL-02.</x:v>
       </x:c>
       <x:c r="G6" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H6" s="13"/>
-    </x:row>
-    <x:row r="7" ht="62" customHeight="1">
+        <x:v>Awaiting screen feedback</x:v>
+      </x:c>
+      <x:c r="H6" s="13" t="str">
+        <x:v>Workbook-approved fields and skippable behavior; no score or segment is displayed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="13" t="str">
         <x:v>C03</x:v>
       </x:c>
@@ -2231,23 +2316,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C7" s="13" t="str">
-        <x:v>Requirement intake / BD capture</x:v>
+        <x:v>Shared portal sign-in</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>Client account and OptimIQ BD staff</x:v>
+        <x:v>Client / shared identity</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
-        <x:v>Screen design depends on the governing flow: client submission from its login or requirement capture by OptimIQ BD/pre-sales in the internal system.</x:v>
+        <x:v>Use the single shared sign-in and route the account to the client journey.</x:v>
       </x:c>
       <x:c r="F7" s="13" t="str">
-        <x:v>Conflict to resolve: the prior discussion says the client enters from its login; BRD v3.2 says OptimIQ BD/pre-sales captures and enters the requirement. Confirm which flow governs before designing this screen.</x:v>
+        <x:v>Account invitation/self-start, OTP, and relation to the existing CTA require reconciliation (CL-01).</x:v>
       </x:c>
       <x:c r="G7" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H7" s="13"/>
-    </x:row>
-    <x:row r="8" ht="62" customHeight="1">
+        <x:v>Already designed · shared screen</x:v>
+      </x:c>
+      <x:c r="H7" s="13" t="str">
+        <x:v>Login after CTA follows the agreed audience sequence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="13" t="str">
         <x:v>C04</x:v>
       </x:c>
@@ -2255,23 +2342,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C8" s="13" t="str">
-        <x:v>Requirement workspace — Track A</x:v>
+        <x:v>Terms &amp; declarations</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
-        <x:v>Client account</x:v>
+        <x:v>Client account holder</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Review a smaller, clear requirement and its managed progress through shortlist and award.</x:v>
+        <x:v>Review and accept client account terms after sign-in if not already accepted.</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
-        <x:v>Routing threshold is open; do not invent a Track A threshold in the screen.</x:v>
+        <x:v>Exact document list, signer authority, payment setup, and legal wording (CL-03).</x:v>
       </x:c>
       <x:c r="G8" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H8" s="13"/>
-    </x:row>
-    <x:row r="9" ht="62" customHeight="1">
+      <x:c r="H8" s="13" t="str">
+        <x:v>Use the same Theme 1 terms structure as Consultant and Consulting Firm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>C05</x:v>
       </x:c>
@@ -2279,23 +2368,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C9" s="13" t="str">
-        <x:v>Masked shortlist comparison</x:v>
+        <x:v>Client dashboard</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>Track A and Track B clients</x:v>
+        <x:v>Client account holder</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>Compare the usual 2–3 masked seller profiles and see why each was recommended.</x:v>
+        <x:v>360° client view, with Phase 1 account/categorisation and Phase 2 requirements/projects views.</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
-        <x:v>Exact masked fields, comparison criteria, and request-more exception workflow need clarification.</x:v>
+        <x:v>Exact dashboard metrics and phase mapping conflict with BRD Phase 1 labels (CL-04).</x:v>
       </x:c>
       <x:c r="G9" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H9" s="13"/>
-    </x:row>
-    <x:row r="10" ht="62" customHeight="1">
+        <x:v>Awaiting screen feedback</x:v>
+      </x:c>
+      <x:c r="H9" s="13" t="str">
+        <x:v>Never expose internal score or CL1–CL4 segment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="13" t="str">
         <x:v>C06</x:v>
       </x:c>
@@ -2303,23 +2394,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>Masked seller profile detail</x:v>
+        <x:v>Client organisation profile</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>Track A and Track B clients</x:v>
+        <x:v>Client account holder</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>Inspect the permitted profile information while identity and contact details remain masked.</x:v>
+        <x:v>Review organisation and contact information in the client account.</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
-        <x:v>Which profile fields are visible before the approved identity-release gate is open.</x:v>
+        <x:v>Editable fields, profile update evidence, approval, and change history (CL-05).</x:v>
       </x:c>
       <x:c r="G10" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H10" s="13"/>
-    </x:row>
-    <x:row r="11" ht="62" customHeight="1">
+      <x:c r="H10" s="13" t="str">
+        <x:v>Do not expose internal OptiMIQ commercial information.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="13" t="str">
         <x:v>C07</x:v>
       </x:c>
@@ -2327,23 +2420,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
-        <x:v>Request additional profiles</x:v>
+        <x:v>Requirement creation &amp; scoping</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
-        <x:v>Client account</x:v>
+        <x:v>Client account; Solution Coordinator</x:v>
       </x:c>
       <x:c r="E11" s="13" t="str">
-        <x:v>Ask OptimIQ for more profiles when the initial shortlist is unsuitable.</x:v>
+        <x:v>Create a client requirement from the portal; OptimIQ scopes and routes it.</x:v>
       </x:c>
       <x:c r="F11" s="13" t="str">
-        <x:v>BRD requires an approved, logged exception beyond 2–3; exact approval path and feedback interaction need clarification.</x:v>
+        <x:v>Exact form fields, required attachments, edit/withdraw states, coordinator assignment, and fee display (CL-06).</x:v>
       </x:c>
       <x:c r="G11" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H11" s="13"/>
-    </x:row>
-    <x:row r="12" ht="62" customHeight="1">
+      <x:c r="H11" s="13" t="str">
+        <x:v>Journey placed after client login, per the agreed audience flow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="13" t="str">
         <x:v>C08</x:v>
       </x:c>
@@ -2351,23 +2446,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C12" s="13" t="str">
-        <x:v>Track B tender and evaluation</x:v>
+        <x:v>Track A masked shortlist</x:v>
       </x:c>
       <x:c r="D12" s="13" t="str">
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E12" s="13" t="str">
-        <x:v>Review a managed procurement event and its technical/financial evaluation stages.</x:v>
+        <x:v>Review the normal 2–3 curated masked profiles and recommendation rationale.</x:v>
       </x:c>
       <x:c r="F12" s="13" t="str">
-        <x:v>Approved evaluation methods, weight limits, scoring view, and Track B routing threshold are open.</x:v>
+        <x:v>Visible profile attributes, comparison criteria, and client decision controls (CL-07).</x:v>
       </x:c>
       <x:c r="G12" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H12" s="13"/>
-    </x:row>
-    <x:row r="13" ht="62" customHeight="1">
+      <x:c r="H12" s="13" t="str">
+        <x:v>No open seller directory or unmasked contact details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="13" t="str">
         <x:v>C09</x:v>
       </x:c>
@@ -2375,25 +2472,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C13" s="13" t="str">
-        <x:v>LOI and award review</x:v>
+        <x:v>Masked seller detail</x:v>
       </x:c>
       <x:c r="D13" s="13" t="str">
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
-        <x:v>Review the selected seller and LOI, plus the required pre-award agreement gate; show agreement, award, and acceptance states.</x:v>
+        <x:v>Inspect permitted experience, fit, and capability details for a shortlisted seller.</x:v>
       </x:c>
       <x:c r="F13" s="13" t="str">
-        <x:v>Client requires agreements signed before award and introduction. This conflicts with the BRD LOI/contract order. Clarify agreement types, signatories, and sequence relative to LOI; status depends on that decision.</x:v>
+        <x:v>Which profile information may be shown before identity-release approval (CL-07).</x:v>
       </x:c>
       <x:c r="G13" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H13" s="13" t="str">
-        <x:v>Theme 1 feedback: agreements must be signed before award and introduction. Exact agreement scope/order added to client clarification.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="62" customHeight="1">
+        <x:v>Mask identity and contact details until approved release.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="13" t="str">
         <x:v>C10</x:v>
       </x:c>
@@ -2401,23 +2498,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C14" s="13" t="str">
-        <x:v>Meeting and controlled introduction</x:v>
+        <x:v>Request additional profiles</x:v>
       </x:c>
       <x:c r="D14" s="13" t="str">
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E14" s="13" t="str">
-        <x:v>Schedule and attend the approved introduction meeting after the required gate.</x:v>
+        <x:v>Ask OptimIQ for more profiles if the initial shortlist is unsuitable.</x:v>
       </x:c>
       <x:c r="F14" s="13" t="str">
-        <x:v>Required agreements must precede award and introduction per client feedback; exact agreement types/parties and the relationship to LOI remain open. Provider, recording, consent, and disclosure timing also remain open.</x:v>
+        <x:v>Exception approval, evidence, reason capture, and number of additional profiles (CL-08).</x:v>
       </x:c>
       <x:c r="G14" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H14" s="13"/>
-    </x:row>
-    <x:row r="15" ht="62" customHeight="1">
+      <x:c r="H14" s="13" t="str">
+        <x:v>BRD requires approved/logged exception beyond the normal shortlist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="13" t="str">
         <x:v>C11</x:v>
       </x:c>
@@ -2425,23 +2524,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C15" s="13" t="str">
-        <x:v>Engagement and delivery workspace</x:v>
+        <x:v>Track B tender &amp; evaluation</x:v>
       </x:c>
       <x:c r="D15" s="13" t="str">
-        <x:v>Client account</x:v>
+        <x:v>Client account; Procurement Desk</x:v>
       </x:c>
       <x:c r="E15" s="13" t="str">
-        <x:v>Track project agreement status, delivery plan, milestones, acceptance/rework, and close-out; enforce the approved agreement gate before award/introduction.</x:v>
+        <x:v>Follow technical evaluation (TER), financial evaluation (FER), decision, and tender status.</x:v>
       </x:c>
       <x:c r="F15" s="13" t="str">
-        <x:v>Agreement types and sequence relative to LOI need clarification. Milestone catalogue and amendment approvals remain open.</x:v>
+        <x:v>Routing threshold, evaluation method, weights, scoring visibility, and client decision rights (CL-09).</x:v>
       </x:c>
       <x:c r="G15" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H15" s="13"/>
-    </x:row>
-    <x:row r="16" ht="62" customHeight="1">
+      <x:c r="H15" s="13" t="str">
+        <x:v>Do not assume the 70:30 example is approved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="13" t="str">
         <x:v>C12</x:v>
       </x:c>
@@ -2449,23 +2550,25 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C16" s="13" t="str">
-        <x:v>Contracts, invoices, payments, refunds</x:v>
+        <x:v>Agreements &amp; award</x:v>
       </x:c>
       <x:c r="D16" s="13" t="str">
-        <x:v>Client account</x:v>
+        <x:v>Client account; selected seller</x:v>
       </x:c>
       <x:c r="E16" s="13" t="str">
-        <x:v>Review commercial documents, invoices, payment status, and applicable credits/refunds.</x:v>
+        <x:v>Show required signature gate before award and introduction, following client feedback.</x:v>
       </x:c>
       <x:c r="F16" s="13" t="str">
-        <x:v>Fee schedules, payment integrations, and refund/credit triggers remain open.</x:v>
+        <x:v>Document types, signatories, and sequence relative to LOI/contract conflict with BRD (CL-10).</x:v>
       </x:c>
       <x:c r="G16" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H16" s="13"/>
-    </x:row>
-    <x:row r="17" ht="62" customHeight="1">
+      <x:c r="H16" s="13" t="str">
+        <x:v>The signature-before-award-and-introduction gate is agreed; exact order remains open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="13" t="str">
         <x:v>C13</x:v>
       </x:c>
@@ -2473,45 +2576,205 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>Project rating and feedback</x:v>
+        <x:v>Meetings &amp; controlled introduction</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
+        <x:v>Client account; OptimIQ staff; seller</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>Coordinate approved scoping, evaluation, and post-award introduction meetings.</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="str">
+        <x:v>Provider, recording, consent, identity disclosure, and timing (CL-11).</x:v>
+      </x:c>
+      <x:c r="G17" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H17" s="13" t="str">
+        <x:v>Controlled interaction; no direct open seller contact before the approved gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="13" t="str">
+        <x:v>C14</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>Engagements &amp; milestones</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>Client account; engagement participants</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>Review mobilisation, milestones, submitted work, acceptance/rework, approved changes, and close-out.</x:v>
+      </x:c>
+      <x:c r="F18" s="13" t="str">
+        <x:v>Milestone catalogue, review window, change approval, and dispute details (CL-12).</x:v>
+      </x:c>
+      <x:c r="G18" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H18" s="13" t="str">
+        <x:v>Per BRD G lifecycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="13" t="str">
+        <x:v>C15</x:v>
+      </x:c>
+      <x:c r="B19" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>Invoices &amp; payments</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="str">
+        <x:v>Client account; Finance</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str">
+        <x:v>Review client invoices, amounts due, payments, and receipts in project context.</x:v>
+      </x:c>
+      <x:c r="F19" s="13" t="str">
+        <x:v>Fees, invoice timing, payment methods, cancellations, refunds, and fee visibility (CL-13).</x:v>
+      </x:c>
+      <x:c r="G19" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H19" s="13" t="str">
+        <x:v>Hide internal OptimIQ margins and commissions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="64" customHeight="1">
+      <x:c r="A20" s="13" t="str">
+        <x:v>C16</x:v>
+      </x:c>
+      <x:c r="B20" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str">
+        <x:v>Feedback &amp; re-engagement</x:v>
+      </x:c>
+      <x:c r="D20" s="13" t="str">
+        <x:v>Client account; per engagement</x:v>
+      </x:c>
+      <x:c r="E20" s="13" t="str">
+        <x:v>Give seller feedback at milestone and project close; return to create repeat requirements.</x:v>
+      </x:c>
+      <x:c r="F20" s="13" t="str">
+        <x:v>Whether client feedback changes composite/performance scores or appears as a separate signal (CL-14).</x:v>
+      </x:c>
+      <x:c r="G20" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H20" s="13" t="str">
+        <x:v>Capture feedback per engagement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="64" customHeight="1">
+      <x:c r="A21" s="13" t="str">
+        <x:v>C17</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>Communications &amp; notifications</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="str">
         <x:v>Client account</x:v>
       </x:c>
-      <x:c r="E17" s="13" t="str">
-        <x:v>Collect client feedback for each completed project and link it to the specific consultant or firm engagement.</x:v>
-      </x:c>
-      <x:c r="F17" s="13" t="str">
-        <x:v>Rating scale, visibility, moderation, and whether feedback contributes to the composite/performance score or is displayed separately remain open.</x:v>
-      </x:c>
-      <x:c r="G17" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H17" s="13"/>
-    </x:row>
-    <x:row r="18" ht="62" customHeight="1">
-      <x:c r="A18" s="14" t="str">
-        <x:v>C14</x:v>
-      </x:c>
-      <x:c r="B18" s="14" t="str">
+      <x:c r="E21" s="13" t="str">
+        <x:v>See OptimIQ messages, project updates, and action notifications.</x:v>
+      </x:c>
+      <x:c r="F21" s="13" t="str">
+        <x:v>Email/chat/WhatsApp, portal mailbox, event triggers, and provider (CL-15).</x:v>
+      </x:c>
+      <x:c r="G21" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H21" s="13" t="str">
+        <x:v>Provider integration is flexible; scope is unconfirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="64" customHeight="1">
+      <x:c r="A22" s="13" t="str">
+        <x:v>C18</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
-      <x:c r="C18" s="14" t="str">
-        <x:v>Post-delivery relationship</x:v>
-      </x:c>
-      <x:c r="D18" s="14" t="str">
+      <x:c r="C22" s="13" t="str">
+        <x:v>Project calendar</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="str">
         <x:v>Client account</x:v>
       </x:c>
-      <x:c r="E18" s="14" t="str">
-        <x:v>Review past work, referrals, repeat requirements, and account follow-up.</x:v>
-      </x:c>
-      <x:c r="F18" s="14" t="str">
-        <x:v>KPIs and referral/repeat-work rules remain open.</x:v>
-      </x:c>
-      <x:c r="G18" s="14" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H18" s="14"/>
+      <x:c r="E22" s="13" t="str">
+        <x:v>Review requirement calls, meetings, milestones, and deadlines.</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="str">
+        <x:v>Event types, calendar sync, invite rules, and meeting-specific recording behavior (CL-16).</x:v>
+      </x:c>
+      <x:c r="G22" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H22" s="13" t="str">
+        <x:v>Use shared layout and role-aware left navigation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="64" customHeight="1">
+      <x:c r="A23" s="13" t="str">
+        <x:v>C19</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>Project documents</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>Client account; approved project participants</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>Access approved project files and consultant comments for the relevant project.</x:v>
+      </x:c>
+      <x:c r="F23" s="13" t="str">
+        <x:v>Folder permissions, retention, upload policy, and knowledge-library/success-story reuse (CL-17).</x:v>
+      </x:c>
+      <x:c r="G23" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H23" s="13" t="str">
+        <x:v>Project folders proposed Phase 2; future reusable library is separate and unapproved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="64" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>C20</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>Support, complaints &amp; account exit</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>Client account; support / grievance staff</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="str">
+        <x:v>Raise and track a grievance/support request and review account status or exit.</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="str">
+        <x:v>Intake categories, escalation, response targets, open-project handling, retention, and settlement (CL-18).</x:v>
+      </x:c>
+      <x:c r="G24" s="14" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H24" s="14" t="str">
+        <x:v>Map to BRD Q and X lifecycle.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2913,85 +3176,61 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="64" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="72" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="2" t="str">
+      <x:c r="A1" s="78" t="str">
         <x:v>Open Clarifications</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>Open Clarifications</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>Open Clarifications</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>Open Clarifications</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>Open Clarifications</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>Open Clarifications</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>Open Clarifications</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="B1" s="78"/>
+      <x:c r="C1" s="78"/>
+      <x:c r="D1" s="78"/>
+      <x:c r="E1" s="78"/>
+      <x:c r="F1" s="78"/>
+      <x:c r="G1" s="78"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="81" t="str">
         <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="str">
-        <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="str">
-        <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
-      </x:c>
-      <x:c r="E2" s="5" t="str">
-        <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="str">
-        <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="str">
-        <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="8" t="str">
+      <x:c r="B2" s="81"/>
+      <x:c r="C2" s="81"/>
+      <x:c r="D2" s="81"/>
+      <x:c r="E2" s="81"/>
+      <x:c r="F2" s="81"/>
+      <x:c r="G2" s="81"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="84" t="str">
         <x:v>Clarification ID</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B4" s="84" t="str">
         <x:v>Audience</x:v>
       </x:c>
-      <x:c r="C4" s="8" t="str">
+      <x:c r="C4" s="84" t="str">
         <x:v>Affected screen</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="str">
+      <x:c r="D4" s="84" t="str">
         <x:v>Question / decision needed</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="str">
+      <x:c r="E4" s="84" t="str">
         <x:v>Source / conflict</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="F4" s="84" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
+      <x:c r="G4" s="84" t="str">
         <x:v>Working assumption shown in wireframe</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="56" customHeight="1">
+    <x:row r="5" ht="65" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>CF-01</x:v>
       </x:c>
@@ -3014,7 +3253,7 @@
         <x:v>Show the shared terms review structure; hold legal text and affiliate-entity interpretation open.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="56" customHeight="1">
+    <x:row r="6" ht="65" customHeight="1">
       <x:c r="A6" s="13" t="str">
         <x:v>CF-02</x:v>
       </x:c>
@@ -3037,7 +3276,7 @@
         <x:v>Keep approved questions and six sections; do not invent boundary inclusivity.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="56" customHeight="1">
+    <x:row r="7" ht="65" customHeight="1">
       <x:c r="A7" s="13" t="str">
         <x:v>CF-03</x:v>
       </x:c>
@@ -3060,7 +3299,7 @@
         <x:v>Assume preliminary status is pending review and show no numeric score until client decides.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="56" customHeight="1">
+    <x:row r="8" ht="65" customHeight="1">
       <x:c r="A8" s="13" t="str">
         <x:v>CF-04</x:v>
       </x:c>
@@ -3083,7 +3322,7 @@
         <x:v>Continue showing current wireframe phase convention, clearly marked provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="56" customHeight="1">
+    <x:row r="9" ht="65" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>CF-05</x:v>
       </x:c>
@@ -3106,7 +3345,7 @@
         <x:v>Wireframe follows the direct user decision: one firm login. Do not show employee invites until the BRD is reconciled.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="56" customHeight="1">
+    <x:row r="10" ht="65" customHeight="1">
       <x:c r="A10" s="13" t="str">
         <x:v>CF-06</x:v>
       </x:c>
@@ -3129,7 +3368,7 @@
         <x:v>Show progress/status placeholders; do not invent a mandatory checklist.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="56" customHeight="1">
+    <x:row r="11" ht="65" customHeight="1">
       <x:c r="A11" s="13" t="str">
         <x:v>CF-07</x:v>
       </x:c>
@@ -3152,7 +3391,7 @@
         <x:v>Model values as Admin-configurable; show no fixed commercial amount.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="56" customHeight="1">
+    <x:row r="12" ht="65" customHeight="1">
       <x:c r="A12" s="13" t="str">
         <x:v>CF-08</x:v>
       </x:c>
@@ -3175,7 +3414,7 @@
         <x:v>Keep technical and commercial bids separate; do not expose competitor bids.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="56" customHeight="1">
+    <x:row r="13" ht="65" customHeight="1">
       <x:c r="A13" s="13" t="str">
         <x:v>CF-09</x:v>
       </x:c>
@@ -3198,7 +3437,7 @@
         <x:v>Keep profiles masked until the approved release gate; exact gate remains open.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="56" customHeight="1">
+    <x:row r="14" ht="65" customHeight="1">
       <x:c r="A14" s="13" t="str">
         <x:v>CF-10</x:v>
       </x:c>
@@ -3221,7 +3460,7 @@
         <x:v>Apply the approved gate that signatures precede award and introduction; resolve document sequence before final flow.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="56" customHeight="1">
+    <x:row r="15" ht="65" customHeight="1">
       <x:c r="A15" s="13" t="str">
         <x:v>CF-11</x:v>
       </x:c>
@@ -3244,7 +3483,7 @@
         <x:v>Reservation is not deployment; release if firm does not win.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="56" customHeight="1">
+    <x:row r="16" ht="65" customHeight="1">
       <x:c r="A16" s="13" t="str">
         <x:v>CF-12</x:v>
       </x:c>
@@ -3267,7 +3506,7 @@
         <x:v>Keep Seller and Buyer money streams distinct; hide internal OptimIQ margin.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="56" customHeight="1">
+    <x:row r="17" ht="65" customHeight="1">
       <x:c r="A17" s="13" t="str">
         <x:v>CF-13</x:v>
       </x:c>
@@ -3290,7 +3529,7 @@
         <x:v>Treat as potential configurable integrations; no provider or SLA commitment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="56" customHeight="1">
+    <x:row r="18" ht="65" customHeight="1">
       <x:c r="A18" s="13" t="str">
         <x:v>CF-14</x:v>
       </x:c>
@@ -3313,7 +3552,7 @@
         <x:v>Show only a proposed module until access policy and rollout are confirmed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="56" customHeight="1">
+    <x:row r="19" ht="65" customHeight="1">
       <x:c r="A19" s="13" t="str">
         <x:v>CF-15</x:v>
       </x:c>
@@ -3336,7 +3575,7 @@
         <x:v>Enforce DR10 separation: Seller performance is not affected by Buyer payment behavior.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="56" customHeight="1">
+    <x:row r="20" ht="65" customHeight="1">
       <x:c r="A20" s="13" t="str">
         <x:v>CF-16</x:v>
       </x:c>
@@ -3359,27 +3598,441 @@
         <x:v>Show request/status concepts only; workflow rules remain open.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="56" customHeight="1">
-      <x:c r="A21" s="14" t="str">
+    <x:row r="21" ht="65" customHeight="1">
+      <x:c r="A21" s="13" t="str">
         <x:v>CF-17</x:v>
       </x:c>
-      <x:c r="B21" s="14" t="str">
+      <x:c r="B21" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
-      <x:c r="C21" s="14" t="str">
+      <x:c r="C21" s="13" t="str">
         <x:v>CTQ and qualification display</x:v>
       </x:c>
-      <x:c r="D21" s="14" t="str">
+      <x:c r="D21" s="13" t="str">
         <x:v>Are proposed firm tier labels and thresholds final for member display after review, and is a numeric composite score ever displayed?</x:v>
       </x:c>
-      <x:c r="E21" s="14" t="str">
+      <x:c r="E21" s="13" t="str">
         <x:v>BRD addendum Table 68; client note</x:v>
       </x:c>
-      <x:c r="F21" s="14" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="G21" s="14" t="str">
+      <x:c r="F21" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G21" s="13" t="str">
         <x:v>Keep scoring internals hidden in the member workspace.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="65" customHeight="1">
+      <x:c r="A22" s="13" t="str">
+        <x:v>CL-01</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str">
+        <x:v>C01–C03 · CTA, enrichment, sign-in</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="str">
+        <x:v>How does the client CTA/enquiry connect to account creation, OTP/password setup, and login? The categorisation workbook specifies soft, non-blocking email confirmation and no login before optional enrichment; prior project direction says CTA then shared portal login; BRD C1/C2 says BD qualification followed by invitation or self-start and OTP.</x:v>
+      </x:c>
+      <x:c r="E22" s="13" t="str">
+        <x:v>Client workbook Read Me / Client Web Form; BRD C1–C2; agreed shared-login journey</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G22" s="13" t="str">
+        <x:v>Keep the existing CTA unchanged, show the optional step skippable, then use shared login. Do not gate enrichment or expose categorisation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="65" customHeight="1">
+      <x:c r="A23" s="13" t="str">
+        <x:v>CL-02</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>C02 · Optional categorisation</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>What score precision/rounding is applied before assigning CL1–CL4? The workbook gives score bands to three decimal places but does not define rounding for scores between the listed boundaries.</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>Client categorisation workbook: Segment Master and Scoring &amp; Follow-up Logic</x:v>
+      </x:c>
+      <x:c r="F23" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G23" s="13" t="str">
+        <x:v>Use the workbook weights and bands as supplied; keep segment assignment internal and do not display numeric score.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="65" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>CL-03</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str">
+        <x:v>C04 · Terms &amp; declarations</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="str">
+        <x:v>Which client terms/declarations are required, who may sign for the organisation, and is payment-method setup part of first-login account setup?</x:v>
+      </x:c>
+      <x:c r="E24" s="13" t="str">
+        <x:v>BRD C2.4–C2.5; exact client documents not specified</x:v>
+      </x:c>
+      <x:c r="F24" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G24" s="13" t="str">
+        <x:v>Show a shared review/acceptance pattern with placeholder document names; do not imply legal copy is final.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="65" customHeight="1">
+      <x:c r="A25" s="13" t="str">
+        <x:v>CL-04</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>C05 / all client screens · phase labels</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
+        <x:v>Which client lifecycle stages belong to each delivery phase? The agreed wireframe convention ends Phase 1 after categorisation/CTQ; BRD Table 60 labels the client lifecycle steps Phase 1.</x:v>
+      </x:c>
+      <x:c r="E25" s="13" t="str">
+        <x:v>BRD Table 60 versus agreed Theme 1 phase convention</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G25" s="13" t="str">
+        <x:v>Show Phase 1 through account/categorisation and Phase 2 from requirements onward, marked as a wireframe assumption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="65" customHeight="1">
+      <x:c r="A26" s="13" t="str">
+        <x:v>CL-05</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C26" s="13" t="str">
+        <x:v>C06 · Organisation profile</x:v>
+      </x:c>
+      <x:c r="D26" s="13" t="str">
+        <x:v>Which organisation and contact fields can the client edit after registration, what evidence is needed, and which changes require OptimIQ approval?</x:v>
+      </x:c>
+      <x:c r="E26" s="13" t="str">
+        <x:v>BRD C3; no client profile field/update rules supplied</x:v>
+      </x:c>
+      <x:c r="F26" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G26" s="13" t="str">
+        <x:v>Show profile review and an edit entry point only; no unsupported approval workflow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="65" customHeight="1">
+      <x:c r="A27" s="13" t="str">
+        <x:v>CL-06</x:v>
+      </x:c>
+      <x:c r="B27" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
+        <x:v>C07 · Requirement creation &amp; scoping</x:v>
+      </x:c>
+      <x:c r="D27" s="13" t="str">
+        <x:v>What requirement fields, evidence, draft/edit/withdraw rules, fee visibility, and Solution Coordinator assignment details should appear?</x:v>
+      </x:c>
+      <x:c r="E27" s="13" t="str">
+        <x:v>BRD C4.1–C4.5; forms F-C04/F-C05; fields not included in source workbook</x:v>
+      </x:c>
+      <x:c r="F27" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G27" s="13" t="str">
+        <x:v>Use the BRD sequence: submit, scope with coordinator, confirm route, then release after applicable fee gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="65" customHeight="1">
+      <x:c r="A28" s="13" t="str">
+        <x:v>CL-07</x:v>
+      </x:c>
+      <x:c r="B28" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C28" s="13" t="str">
+        <x:v>C08–C09 · Track A shortlist / profile</x:v>
+      </x:c>
+      <x:c r="D28" s="13" t="str">
+        <x:v>Which attributes and match rationale can a client see in the normal 2–3 masked profiles, and what comparison or selection actions are allowed before identity release?</x:v>
+      </x:c>
+      <x:c r="E28" s="13" t="str">
+        <x:v>BRD C5 / Track A; approved masking discussion</x:v>
+      </x:c>
+      <x:c r="F28" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G28" s="13" t="str">
+        <x:v>Show masked profiles and rationale; keep direct identity/contact hidden until approved release gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="65" customHeight="1">
+      <x:c r="A29" s="13" t="str">
+        <x:v>CL-08</x:v>
+      </x:c>
+      <x:c r="B29" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C29" s="13" t="str">
+        <x:v>C10 · Request more profiles</x:v>
+      </x:c>
+      <x:c r="D29" s="13" t="str">
+        <x:v>What reason, approval role, and permitted number of additional profiles apply when the normal 2–3 shortlist is not suitable?</x:v>
+      </x:c>
+      <x:c r="E29" s="13" t="str">
+        <x:v>BRD shortlist exception; exact procedure not specified</x:v>
+      </x:c>
+      <x:c r="F29" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G29" s="13" t="str">
+        <x:v>Show request-to-OptimIQ as an exception that is logged; do not auto-generate more profiles.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="65" customHeight="1">
+      <x:c r="A30" s="13" t="str">
+        <x:v>CL-09</x:v>
+      </x:c>
+      <x:c r="B30" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C30" s="13" t="str">
+        <x:v>C11 · Track B evaluation</x:v>
+      </x:c>
+      <x:c r="D30" s="13" t="str">
+        <x:v>What Track B routing thresholds, evaluation methods, weights, technical/financial visibility, and client decision rights apply?</x:v>
+      </x:c>
+      <x:c r="E30" s="13" t="str">
+        <x:v>BRD RB1–RB4 / Table 27; 70:30 is an unapproved example</x:v>
+      </x:c>
+      <x:c r="F30" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G30" s="13" t="str">
+        <x:v>Show TER then FER as a managed sequence; do not publish scores/weights until confirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="65" customHeight="1">
+      <x:c r="A31" s="13" t="str">
+        <x:v>CL-10</x:v>
+      </x:c>
+      <x:c r="B31" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str">
+        <x:v>C12–C13 · Agreements, award, introduction</x:v>
+      </x:c>
+      <x:c r="D31" s="13" t="str">
+        <x:v>Which agreements are signed by which parties, and how do signatures relate to LOI, award, identity disclosure, introduction, and first payment?</x:v>
+      </x:c>
+      <x:c r="E31" s="13" t="str">
+        <x:v>Client feedback requires signatures before award/introduction; BRD C5–C6 / RA3 / G1 order needs reconciliation</x:v>
+      </x:c>
+      <x:c r="F31" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G31" s="13" t="str">
+        <x:v>Enforce the agreed signature-before-award-and-introduction gate; hold exact document sequence and signers open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="65" customHeight="1">
+      <x:c r="A32" s="13" t="str">
+        <x:v>CL-11</x:v>
+      </x:c>
+      <x:c r="B32" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C32" s="13" t="str">
+        <x:v>C13 · Meetings &amp; introduction</x:v>
+      </x:c>
+      <x:c r="D32" s="13" t="str">
+        <x:v>Which meeting provider, recording/consent settings, participant access, and identity-disclosure point apply to each meeting type?</x:v>
+      </x:c>
+      <x:c r="E32" s="13" t="str">
+        <x:v>BRD controlled interaction; prior meeting configuration decisions; client process detail absent</x:v>
+      </x:c>
+      <x:c r="F32" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G32" s="13" t="str">
+        <x:v>Use a provider-flexible meeting concept and meeting-specific recording as a configurable option.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="65" customHeight="1">
+      <x:c r="A33" s="13" t="str">
+        <x:v>CL-12</x:v>
+      </x:c>
+      <x:c r="B33" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str">
+        <x:v>C14 · Engagements &amp; milestones</x:v>
+      </x:c>
+      <x:c r="D33" s="13" t="str">
+        <x:v>What milestone templates, buyer review windows, rework rules, change approvals, and dispute steps should the client see?</x:v>
+      </x:c>
+      <x:c r="E33" s="13" t="str">
+        <x:v>BRD G1–G5; exact client-facing presentation not final</x:v>
+      </x:c>
+      <x:c r="F33" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G33" s="13" t="str">
+        <x:v>Show project-scoped statuses aligned to BRD; use no fixed milestone catalogue.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="65" customHeight="1">
+      <x:c r="A34" s="13" t="str">
+        <x:v>CL-13</x:v>
+      </x:c>
+      <x:c r="B34" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C34" s="13" t="str">
+        <x:v>C15 · Invoices &amp; payments</x:v>
+      </x:c>
+      <x:c r="D34" s="13" t="str">
+        <x:v>Which fees, payment methods, payment dates, cancellation/refund triggers, and client-visible commercial details apply?</x:v>
+      </x:c>
+      <x:c r="E34" s="13" t="str">
+        <x:v>BRD P/G and Table 30; commercial values remain business decisions</x:v>
+      </x:c>
+      <x:c r="F34" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G34" s="13" t="str">
+        <x:v>Use configurable fee values; show only client-facing amounts, never internal OptimIQ margin/commission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="65" customHeight="1">
+      <x:c r="A35" s="13" t="str">
+        <x:v>CL-14</x:v>
+      </x:c>
+      <x:c r="B35" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C35" s="13" t="str">
+        <x:v>C16 · Feedback &amp; re-engagement</x:v>
+      </x:c>
+      <x:c r="D35" s="13" t="str">
+        <x:v>Does client feedback affect seller composite/performance scores, or is it stored and presented as a separate project signal?</x:v>
+      </x:c>
+      <x:c r="E35" s="13" t="str">
+        <x:v>Client feedback per engagement; BRD C8.1 / performance scoring</x:v>
+      </x:c>
+      <x:c r="F35" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G35" s="13" t="str">
+        <x:v>Capture feedback separately per engagement; do not display score impact until approved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="65" customHeight="1">
+      <x:c r="A36" s="13" t="str">
+        <x:v>CL-15</x:v>
+      </x:c>
+      <x:c r="B36" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C36" s="13" t="str">
+        <x:v>C17 · Communications</x:v>
+      </x:c>
+      <x:c r="D36" s="13" t="str">
+        <x:v>Are in-portal email, chat, WhatsApp, and an @optimiqconsultus.com mailbox in scope for clients? Which message types, retention, and providers apply?</x:v>
+      </x:c>
+      <x:c r="E36" s="13" t="str">
+        <x:v>Client feedback on communications; BRD N1; client-specific scope open</x:v>
+      </x:c>
+      <x:c r="F36" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G36" s="13" t="str">
+        <x:v>Show a notification/message centre concept only; integrations and mailbox are not committed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="65" customHeight="1">
+      <x:c r="A37" s="13" t="str">
+        <x:v>CL-16</x:v>
+      </x:c>
+      <x:c r="B37" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C37" s="13" t="str">
+        <x:v>C18 · Project calendar</x:v>
+      </x:c>
+      <x:c r="D37" s="13" t="str">
+        <x:v>Which client event types and calendar integrations are required, and are recording/consent settings global or meeting-specific?</x:v>
+      </x:c>
+      <x:c r="E37" s="13" t="str">
+        <x:v>Client feedback on integrated calendar and meeting configuration</x:v>
+      </x:c>
+      <x:c r="F37" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G37" s="13" t="str">
+        <x:v>Present a project calendar concept; provider and sync rules remain configurable/open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="65" customHeight="1">
+      <x:c r="A38" s="13" t="str">
+        <x:v>CL-17</x:v>
+      </x:c>
+      <x:c r="B38" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C38" s="13" t="str">
+        <x:v>C19 · Project documents</x:v>
+      </x:c>
+      <x:c r="D38" s="13" t="str">
+        <x:v>Which client, consultant, and OptimIQ roles can access project folders and comments, how long are files retained, and can approved summaries become public success stories?</x:v>
+      </x:c>
+      <x:c r="E38" s="13" t="str">
+        <x:v>Client feedback proposed Phase 2 folders/library; BRD access and publication rules incomplete</x:v>
+      </x:c>
+      <x:c r="F38" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G38" s="13" t="str">
+        <x:v>Treat project folders as a Phase 2 concept; keep cross-client reuse/testimonials disabled until explicit consent and policy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="65" customHeight="1">
+      <x:c r="A39" s="14" t="str">
+        <x:v>CL-18</x:v>
+      </x:c>
+      <x:c r="B39" s="14" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="C39" s="14" t="str">
+        <x:v>C20 · Support &amp; account exit</x:v>
+      </x:c>
+      <x:c r="D39" s="14" t="str">
+        <x:v>What complaint routes, escalation targets, account-exit steps, open-project handling, and retention rules apply to client accounts?</x:v>
+      </x:c>
+      <x:c r="E39" s="14" t="str">
+        <x:v>BRD Q/X; client-specific workflow details not provided</x:v>
+      </x:c>
+      <x:c r="F39" s="14" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G39" s="14" t="str">
+        <x:v>Show support and request status only; do not assume account closure is immediate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Unify Phase 1 CTQ journeys across member audiences
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra7a0332978874fcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="Ra122d669da6b4167"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="Rc47f273e17304fd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="Ra04e35f5c0da4968"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="R6c20df2caf3e47ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="Rc293edcafd1f4b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R908d55a2ba1347eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R99b8de0385fd4a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R68135888d47f4999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="R1bf729d1b2734601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="R7bc9fd82a2e246bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R8adc76df65c749bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="Rd9e2ad6211074b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="R044403abbce64888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="Rbc8140e999ec4c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R9922f3a1649a46eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -72,7 +72,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +97,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF06352E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F4ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF27836E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -231,7 +246,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="85">
+  <x:cellXfs count="93">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -377,6 +392,18 @@
     <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -636,10 +663,10 @@
         <x:v>Consultant</x:v>
       </x:c>
       <x:c r="B6" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Existing consultant flow preserved for 1:1 consistency checks.</x:v>
+        <x:v>Phase 1 ends after CTQ and role-fit selection; later screens are Phase 2.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -650,7 +677,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>Full BRD firm lifecycle mapped to one firm workspace and left navigation.</x:v>
+        <x:v>Phase 1 ends at the six-section firm CTQ; later screens are Phase 2.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -661,7 +688,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Client lifecycle mapped from BRD C1–C8 and the approved categorisation workbook.</x:v>
+        <x:v>Phase 1 ends at optional Client CTQ; dashboard and later screens are Phase 2.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -680,10 +707,10 @@
         <x:v>Open Clarifications</x:v>
       </x:c>
       <x:c r="B10" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>17 consulting firm and 18 client clarification items.</x:v>
+        <x:v>16 consulting firm and 17 client clarification items.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -698,7 +725,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="21" t="str">
-        <x:v>The audience tabs use the same screen inventory fields. Approved requirements belong in Purpose/Review focus; unresolved items are written as clarification questions. The firm phase rule remains provisional because the prior client-approved wireframe rule conflicts with the BRD phase tables. No firm employee-invite screen is shown until the BRD’s F-F03 wording is reconciled with the user’s one-firm-login decision.</x:v>
+        <x:v>Phase 1 contains the shared sign-in, post-login terms and audience CTQ journeys for Consultant, Consulting Firm and Client. All dashboards and later operating screens are Phase 2. The Client workbook places its optional CTQ before login; the portal review assumes post-login placement pending confirmation. The firm has one login; employee invitations are not shown.</x:v>
       </x:c>
       <x:c r="B13" s="21"/>
       <x:c r="C13" s="21"/>
@@ -911,142 +938,144 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="60" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="50" t="str">
+      <x:c r="A1" s="86" t="str">
         <x:v>Consultant · Screen Approval Inventory</x:v>
       </x:c>
-      <x:c r="B1" s="50"/>
-      <x:c r="C1" s="50"/>
-      <x:c r="D1" s="50"/>
-      <x:c r="E1" s="50"/>
-      <x:c r="F1" s="50"/>
-      <x:c r="G1" s="50"/>
-      <x:c r="H1" s="50"/>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="53" t="str">
-        <x:v>Consultant journey; latest client decisions are preserved for 1:1 review against shared components.</x:v>
-      </x:c>
-      <x:c r="B2" s="53"/>
-      <x:c r="C2" s="53"/>
-      <x:c r="D2" s="53"/>
-      <x:c r="E2" s="53"/>
-      <x:c r="F2" s="53"/>
-      <x:c r="G2" s="53"/>
-      <x:c r="H2" s="53"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="56" t="str">
+      <x:c r="B1" s="86"/>
+      <x:c r="C1" s="86"/>
+      <x:c r="D1" s="86"/>
+      <x:c r="E1" s="86"/>
+      <x:c r="F1" s="86"/>
+      <x:c r="G1" s="86"/>
+      <x:c r="H1" s="86"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="89" t="str">
+        <x:v>Phase 1: CTA, shared sign-in, terms, CTQ and role fit. Dashboard, assessment and project screens are Phase 2.</x:v>
+      </x:c>
+      <x:c r="B2" s="89"/>
+      <x:c r="C2" s="89"/>
+      <x:c r="D2" s="89"/>
+      <x:c r="E2" s="89"/>
+      <x:c r="F2" s="89"/>
+      <x:c r="G2" s="89"/>
+      <x:c r="H2" s="89"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="92" t="str">
         <x:v>Screen ID</x:v>
       </x:c>
-      <x:c r="B4" s="56" t="str">
+      <x:c r="B4" s="92" t="str">
         <x:v>Workspace</x:v>
       </x:c>
-      <x:c r="C4" s="56" t="str">
+      <x:c r="C4" s="92" t="str">
         <x:v>Screen / design unit</x:v>
       </x:c>
-      <x:c r="D4" s="56" t="str">
+      <x:c r="D4" s="92" t="str">
         <x:v>Roles / variants</x:v>
       </x:c>
-      <x:c r="E4" s="56" t="str">
+      <x:c r="E4" s="92" t="str">
         <x:v>Purpose and client review focus</x:v>
       </x:c>
-      <x:c r="F4" s="56" t="str">
+      <x:c r="F4" s="92" t="str">
         <x:v>Clarification to park</x:v>
       </x:c>
-      <x:c r="G4" s="56" t="str">
+      <x:c r="G4" s="92" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H4" s="56" t="str">
+      <x:c r="H4" s="92" t="str">
         <x:v>Client decision / notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="62" customHeight="1">
+    <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>E01</x:v>
+        <x:v>E-CTA</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Expert</x:v>
+        <x:v>Consultant</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Expert home dashboard</x:v>
+        <x:v>Consultant CTA registration</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Consultant, Strategic Advisor, Project Manager</x:v>
+        <x:v>Consultant / existing public form</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Show the role profile, score/certification progress, opportunities, and multiple active project assignments at the same time.</x:v>
+        <x:v>Phase 1. Existing CTA and role choices; keep the form unchanged.</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>Visual hierarchy and workload summaries are for client approval; availability/capacity thresholds remain open.</x:v>
+        <x:v>None for this existing screen.</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>Pending client approval</x:v>
+        <x:v>Existing CTA form</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
-        <x:v>Theme 1 feedback: consultants may be active on multiple projects concurrently; show each assignment separately.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="62" customHeight="1">
+        <x:v>Linked from the review page.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="13" t="str">
-        <x:v>E02</x:v>
+        <x:v>E-LOGIN</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>Expert</x:v>
+        <x:v>Consultant</x:v>
       </x:c>
       <x:c r="C6" s="13" t="str">
-        <x:v>Expert role profile switcher</x:v>
+        <x:v>Portal sign-in</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
-        <x:v>One candidate with three role-specific scores and project assignments</x:v>
+        <x:v>Consultant / shared identity</x:v>
       </x:c>
       <x:c r="E6" s="13" t="str">
-        <x:v>Review role results and active assignments; Consultant, Strategic Advisor, and Project Manager roles can apply to different concurrent projects.</x:v>
+        <x:v>Phase 1. Use the shared login after public registration.</x:v>
       </x:c>
       <x:c r="F6" s="13" t="str">
-        <x:v>How to add a role after CTA registration remains open for client clarification.</x:v>
+        <x:v>Account recovery implementation remains open.</x:v>
       </x:c>
       <x:c r="G6" s="13" t="str">
-        <x:v>Ready for screen design</x:v>
+        <x:v>Already designed · shared screen</x:v>
       </x:c>
       <x:c r="H6" s="13" t="str">
-        <x:v>Client clarification (2026-10-20): the same candidate can be Consultant on Project A and Strategic Advisor on Project B at the same time. Role assignment is per project.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="62" customHeight="1">
+        <x:v>One login for all audiences.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="13" t="str">
-        <x:v>E03</x:v>
+        <x:v>E-TERMS</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>Expert</x:v>
+        <x:v>Consultant</x:v>
       </x:c>
       <x:c r="C7" s="13" t="str">
-        <x:v>Professional profile editor</x:v>
+        <x:v>Terms &amp; declarations</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>Each Expert role profile</x:v>
+        <x:v>Consultant account holder</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
-        <x:v>View and edit the role-specific professional profile and supporting details.</x:v>
+        <x:v>Phase 1. Review and accept terms before CTQ.</x:v>
       </x:c>
       <x:c r="F7" s="13" t="str">
-        <x:v>The supplied role-specific form content is approved; post-submission material-change review remains open.</x:v>
+        <x:v>Approved legal wording is required.</x:v>
       </x:c>
       <x:c r="G7" s="13" t="str">
-        <x:v>Ready for screen design</x:v>
-      </x:c>
-      <x:c r="H7" s="13"/>
-    </x:row>
-    <x:row r="8" ht="62" customHeight="1">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H7" s="13" t="str">
+        <x:v>Uses the shared Phase 1 terms layout.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="13" t="str">
         <x:v>E04</x:v>
       </x:c>
@@ -1060,7 +1089,7 @@
         <x:v>All three consultant roles; shared CTQ form</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Complete one eight-step, 36-field form. Do not show scores or weightings. After submission, evaluate the single answer set in the backend for role-fit results.</x:v>
+        <x:v>Phase 1. Complete one eight-step, 36-field form. Do not show scores or weightings. After submission, evaluate the single answer set in the backend for role-fit results.</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
         <x:v>Exact numeric scores and weightings remain internal. Fit categories appear on the next screen.</x:v>
@@ -1072,7 +1101,7 @@
         <x:v>Design updated (2026-10-20): one shared CTQ form, no score or weighting shown; backend determines fit categories after submission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="62" customHeight="1">
+    <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>E05</x:v>
       </x:c>
@@ -1086,7 +1115,7 @@
         <x:v>Consultant, Strategic Advisor, Project Manager</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>After CTQ submission, show a qualitative fit category for each role and let the consultant select one or multiple suitable roles.</x:v>
+        <x:v>Phase 1. After CTQ submission, show a qualitative fit category for each role and let the consultant select one or multiple suitable roles.</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
         <x:v>Whether Low-fit roles can be selected and whether confirmed role choices can be changed later remain open for client clarification.</x:v>
@@ -1098,389 +1127,465 @@
         <x:v>Illustrative results: Best fit Consultant, Moderate fit Strategic Advisor, Low fit Project Manager. Consultant starts selected; low-fit Project Manager is shown but disabled pending clarification. Candidate may keep one role or add a suitable role.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="62" customHeight="1">
+    <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="13" t="str">
-        <x:v>E06</x:v>
+        <x:v>E01</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>Assessment and certification progress</x:v>
+        <x:v>Expert home dashboard</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>Each Expert role profile</x:v>
+        <x:v>Consultant, Strategic Advisor, Project Manager</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>Show progress across the complete composite assessment: CTQ; domain and behavioral assessments (third party); work-quality evaluation; case studies/client impact; client testimonials/references; and committee interview, once its role is confirmed. Show actions/status, not numeric scores or weights.</x:v>
+        <x:v>Phase 2. Show the role profile, score/certification progress, opportunities, and multiple active project assignments at the same time.</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
-        <x:v>Committee interview role is not allocated in the previously approved six-component 100% model. Confirm whether it is evidence in an existing component, a certification gate, or a new weighted component and whether weights change.</x:v>
+        <x:v>Visual hierarchy and workload summaries are for client approval; availability/capacity thresholds remain open.</x:v>
       </x:c>
       <x:c r="G10" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Pending client approval</x:v>
       </x:c>
       <x:c r="H10" s="13" t="str">
-        <x:v>Client feedback 2026-10-23 incorporated; preserve approved six-component formula pending committee-interview decision.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="62" customHeight="1">
+        <x:v>Theme 1 feedback: consultants may be active on multiple projects concurrently; show each assignment separately.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="13" t="str">
-        <x:v>E07</x:v>
+        <x:v>E02</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
-        <x:v>Certificate record</x:v>
+        <x:v>Expert role profile switcher</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
-        <x:v>Certified Expert</x:v>
+        <x:v>One candidate with three role-specific scores and project assignments</x:v>
       </x:c>
       <x:c r="E11" s="13" t="str">
-        <x:v>View certificate status, issuer, validity, and renewal information.</x:v>
+        <x:v>Phase 2. Review role results and active assignments; Consultant, Strategic Advisor, and Project Manager roles can apply to different concurrent projects.</x:v>
       </x:c>
       <x:c r="F11" s="13" t="str">
-        <x:v>External issuer and certificate validity period are open.</x:v>
+        <x:v>How to add a role after CTA registration remains open for client clarification.</x:v>
       </x:c>
       <x:c r="G11" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H11" s="13"/>
-    </x:row>
-    <x:row r="12" ht="62" customHeight="1">
+        <x:v>Ready for screen design</x:v>
+      </x:c>
+      <x:c r="H11" s="13" t="str">
+        <x:v>Client clarification (2026-10-20): the same candidate can be Consultant on Project A and Strategic Advisor on Project B at the same time. Role assignment is per project.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>E08</x:v>
+        <x:v>E03</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C12" s="13" t="str">
-        <x:v>Membership and availability</x:v>
+        <x:v>Professional profile editor</x:v>
       </x:c>
       <x:c r="D12" s="13" t="str">
-        <x:v>Expert account</x:v>
+        <x:v>Each Expert role profile</x:v>
       </x:c>
       <x:c r="E12" s="13" t="str">
-        <x:v>Manage membership status and availability for suitable opportunities.</x:v>
+        <x:v>Phase 2. View and edit the role-specific professional profile and supporting details.</x:v>
       </x:c>
       <x:c r="F12" s="13" t="str">
-        <x:v>Membership fee schedule and some availability/risk thresholds remain open.</x:v>
+        <x:v>The supplied role-specific form content is approved; post-submission material-change review remains open.</x:v>
       </x:c>
       <x:c r="G12" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Ready for screen design</x:v>
       </x:c>
       <x:c r="H12" s="13"/>
     </x:row>
-    <x:row r="13" ht="62" customHeight="1">
+    <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="13" t="str">
-        <x:v>E09</x:v>
+        <x:v>E06</x:v>
       </x:c>
       <x:c r="B13" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C13" s="13" t="str">
-        <x:v>Consultant opportunities and project details</x:v>
+        <x:v>Assessment and certification progress</x:v>
       </x:c>
       <x:c r="D13" s="13" t="str">
-        <x:v>Certified Consultant</x:v>
+        <x:v>Each Expert role profile</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
-        <x:v>Review masked opportunities matched to selected roles; inspect project details and express interest or submit a bid/quotation before project agreement and award.</x:v>
+        <x:v>Phase 2. Show progress across the complete composite assessment: CTQ; domain and behavioral assessments (third party); work-quality evaluation; case studies/client impact; client testimonials/references; and committee interview, once its role is confirmed. Show actions/status, not numeric scores or weights.</x:v>
       </x:c>
       <x:c r="F13" s="13" t="str">
-        <x:v>Matching/recommendation criteria, bid/quote fields and commercial terms remain open.</x:v>
+        <x:v>Committee interview role is not allocated in the previously approved six-component 100% model. Confirm whether it is evidence in an existing component, a certification gate, or a new weighted component and whether weights change.</x:v>
       </x:c>
       <x:c r="G13" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H13" s="13" t="str">
-        <x:v>Consultant opportunities concept added; client review needed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="62" customHeight="1">
+        <x:v>Client feedback 2026-10-23 incorporated; preserve approved six-component formula pending committee-interview decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="13" t="str">
-        <x:v>E10</x:v>
+        <x:v>E07</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C14" s="13" t="str">
-        <x:v>Opportunity response and bid / quotation</x:v>
+        <x:v>Certificate record</x:v>
       </x:c>
       <x:c r="D14" s="13" t="str">
-        <x:v>Certified Consultant</x:v>
+        <x:v>Certified Expert</x:v>
       </x:c>
       <x:c r="E14" s="13" t="str">
-        <x:v>Prepare a role-specific project response with availability, proposed approach, and configured bid/quotation details.</x:v>
+        <x:v>Phase 2. View certificate status, issuer, validity, and renewal information.</x:v>
       </x:c>
       <x:c r="F14" s="13" t="str">
-        <x:v>Commercial terms, bid support fee, workflow, and identity-release point remain open.</x:v>
+        <x:v>External issuer and certificate validity period are open.</x:v>
       </x:c>
       <x:c r="G14" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H14" s="13" t="str">
-        <x:v>Included in the Consultant Opportunities &amp; Project Details screen.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="62" customHeight="1">
+      <x:c r="H14" s="13"/>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="13" t="str">
-        <x:v>E11</x:v>
+        <x:v>E08</x:v>
       </x:c>
       <x:c r="B15" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C15" s="13" t="str">
-        <x:v>Project agreement gate before award</x:v>
+        <x:v>Membership and availability</x:v>
       </x:c>
       <x:c r="D15" s="13" t="str">
-        <x:v>Selected Expert / Consultant</x:v>
+        <x:v>Expert account</x:v>
       </x:c>
       <x:c r="E15" s="13" t="str">
-        <x:v>Show required project agreements for review and signature before project award and before Client-Consultant introduction. Award and introduction remain gated until required signatures are recorded.</x:v>
+        <x:v>Phase 2. Manage membership status and availability for suitable opportunities.</x:v>
       </x:c>
       <x:c r="F15" s="13" t="str">
-        <x:v>Agreement types, signatories, and sequence conflict with the BRD LOI/contract workflow; clarify the final order before implementation.</x:v>
+        <x:v>Membership fee schedule and some availability/risk thresholds remain open.</x:v>
       </x:c>
       <x:c r="G15" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
-      <x:c r="H15" s="13" t="str">
-        <x:v>Updated to reflect client requirement that agreements are signed before award and introduction; screen concept available for review.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="62" customHeight="1">
+      <x:c r="H15" s="13"/>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="13" t="str">
-        <x:v>E12</x:v>
+        <x:v>E09</x:v>
       </x:c>
       <x:c r="B16" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C16" s="13" t="str">
-        <x:v>Engagements and delivery workspace</x:v>
+        <x:v>Consultant opportunities and project details</x:v>
       </x:c>
       <x:c r="D16" s="13" t="str">
-        <x:v>Engaged Expert / Consultant</x:v>
+        <x:v>Certified Consultant</x:v>
       </x:c>
       <x:c r="E16" s="13" t="str">
-        <x:v>Define an Engagement as an OptimIQ project assignment after applicable award/acceptance steps. Support multiple concurrent assignments, each with its own role, status, milestones, and feedback. Separate active and completed OptimIQ work.</x:v>
+        <x:v>Phase 2. Review masked opportunities matched to selected roles; inspect project details and express interest or submit a bid/quotation before project agreement and award.</x:v>
       </x:c>
       <x:c r="F16" s="13" t="str">
-        <x:v>Confirm engagement records, project history retention, capacity rules for concurrent work, and milestone changes.</x:v>
+        <x:v>Matching/recommendation criteria, bid/quote fields and commercial terms remain open.</x:v>
       </x:c>
       <x:c r="G16" s="13" t="str">
-        <x:v>Awaiting client feedback</x:v>
+        <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H16" s="13" t="str">
-        <x:v>Clarified distinction: prior/outside-OptimIQ work belongs to Past Project Experience, not Engagements.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="62" customHeight="1">
+        <x:v>Consultant opportunities concept added; client review needed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>E13</x:v>
+        <x:v>E10</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>Performance, CPD, ratings, renewal</x:v>
+        <x:v>Opportunity response and bid / quotation</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>Expert account / Consultant</x:v>
+        <x:v>Certified Consultant</x:v>
       </x:c>
       <x:c r="E17" s="13" t="str">
-        <x:v>Review client feedback separately by engagement and manage Continuing Professional Development (CPD) records. CPD means ongoing learning and professional development activity.</x:v>
+        <x:v>Phase 2. Prepare a role-specific project response with availability, proposed approach, and configured bid/quotation details.</x:v>
       </x:c>
       <x:c r="F17" s="13" t="str">
-        <x:v>Does feedback affect composite/performance score or remain a separate signal, and how is it aggregated? Confirm CPD units/evidence, validation, and renewal/certification effect.</x:v>
+        <x:v>Commercial terms, bid support fee, workflow, and identity-release point remain open.</x:v>
       </x:c>
       <x:c r="G17" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H17" s="13" t="str">
-        <x:v>Client feedback 2026-10-23: added feedback-per-project and CPD definition; scoring and CPD operating rules remain open.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="62" customHeight="1">
+        <x:v>Included in the Consultant Opportunities &amp; Project Details screen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="13" t="str">
-        <x:v>E14</x:v>
+        <x:v>E11</x:v>
       </x:c>
       <x:c r="B18" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C18" s="13" t="str">
-        <x:v>Profile and assessment progress</x:v>
+        <x:v>Project agreement gate before award</x:v>
       </x:c>
       <x:c r="D18" s="13" t="str">
-        <x:v>Consultant account</x:v>
+        <x:v>Selected Expert / Consultant</x:v>
       </x:c>
       <x:c r="E18" s="13" t="str">
-        <x:v>Allow ongoing profile updates and show status of CTQ and the remaining composite assessment components without showing numeric scores or weights. Score-affecting edits follow evidence and authorised review before recalculation.</x:v>
+        <x:v>Phase 2. Show required project agreements for review and signature before project award and before Client-Consultant introduction. Award and introduction remain gated until required signatures are recorded.</x:v>
       </x:c>
       <x:c r="F18" s="13" t="str">
-        <x:v>Which changed profile fields are material, what evidence/approvals apply, and what status/score is shown while review is pending?</x:v>
+        <x:v>Agreement types, signatories, and sequence conflict with the BRD LOI/contract workflow; clarify the final order before implementation.</x:v>
       </x:c>
       <x:c r="G18" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H18" s="13" t="str">
-        <x:v>Consultant can update profile over time; score recalculation follows evidence and review rules in BRD v3.2.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="62" customHeight="1">
+        <x:v>Updated to reflect client requirement that agreements are signed before award and introduction; screen concept available for review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="13" t="str">
-        <x:v>E15</x:v>
+        <x:v>E12</x:v>
       </x:c>
       <x:c r="B19" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C19" s="13" t="str">
-        <x:v>OptimIQ engagement history</x:v>
+        <x:v>Engagements and delivery workspace</x:v>
       </x:c>
       <x:c r="D19" s="13" t="str">
-        <x:v>Consultant account</x:v>
+        <x:v>Engaged Expert / Consultant</x:v>
       </x:c>
       <x:c r="E19" s="13" t="str">
-        <x:v>View active and completed OptimIQ project assignments separately. A Consultant can work on multiple engagements at the same time. Past Project Experience remains a separate profile section for prior/outside-OptimIQ work.</x:v>
+        <x:v>Phase 2. Define an Engagement as an OptimIQ project assignment after applicable award/acceptance steps. Support multiple concurrent assignments, each with its own role, status, milestones, and feedback. Separate active and completed OptimIQ work.</x:v>
       </x:c>
       <x:c r="F19" s="13" t="str">
-        <x:v>Confirm fields, history retention, and concurrent capacity rules.</x:v>
+        <x:v>Confirm engagement records, project history retention, capacity rules for concurrent work, and milestone changes.</x:v>
       </x:c>
       <x:c r="G19" s="13" t="str">
         <x:v>Awaiting client feedback</x:v>
       </x:c>
       <x:c r="H19" s="13" t="str">
-        <x:v>Terminology clarified from client discussion.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="62" customHeight="1">
+        <x:v>Clarified distinction: prior/outside-OptimIQ work belongs to Past Project Experience, not Engagements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="64" customHeight="1">
       <x:c r="A20" s="13" t="str">
-        <x:v>E16</x:v>
+        <x:v>E13</x:v>
       </x:c>
       <x:c r="B20" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C20" s="13" t="str">
-        <x:v>Payments and invoices</x:v>
+        <x:v>Performance, CPD, ratings, renewal</x:v>
       </x:c>
       <x:c r="D20" s="13" t="str">
-        <x:v>Consultant account / each engagement</x:v>
+        <x:v>Expert account / Consultant</x:v>
       </x:c>
       <x:c r="E20" s="13" t="str">
-        <x:v>Show payment and invoice status in the project context with a Consultant-level payout overview. Keep invoices payable to OptimIQ distinct from payouts owed by OptimIQ to the Consultant; hide internal margins/commission.</x:v>
+        <x:v>Phase 2. Review client feedback separately by engagement and manage Continuing Professional Development (CPD) records. CPD means ongoing learning and professional development activity.</x:v>
       </x:c>
       <x:c r="F20" s="13" t="str">
-        <x:v>Who issues each invoice, who pays whom, whether Consultant invoices or OptimIQ pays by milestone, and visible records/timing.</x:v>
+        <x:v>Does feedback affect composite/performance score or remain a separate signal, and how is it aggregated? Confirm CPD units/evidence, validation, and renewal/certification effect.</x:v>
       </x:c>
       <x:c r="G20" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H20" s="13" t="str">
-        <x:v>New Consultant screen concept created.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="62" customHeight="1">
+        <x:v>Client feedback 2026-10-23: added feedback-per-project and CPD definition; scoring and CPD operating rules remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="13" t="str">
-        <x:v>E17</x:v>
+        <x:v>E14</x:v>
       </x:c>
       <x:c r="B21" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>Communications and notifications</x:v>
+        <x:v>Profile and assessment progress</x:v>
       </x:c>
       <x:c r="D21" s="13" t="str">
         <x:v>Consultant account</x:v>
       </x:c>
       <x:c r="E21" s="13" t="str">
-        <x:v>Provide an OptimIQ-provisioned @optimiqconsultus.com mailbox within the portal, project communications, and in-portal notifications for new emails/messages; support chat and WhatsApp integrations as approved.</x:v>
+        <x:v>Phase 2. Allow ongoing profile updates and show status of CTQ and the remaining composite assessment components without showing numeric scores or weights. Score-affecting edits follow evidence and authorised review before recalculation.</x:v>
       </x:c>
       <x:c r="F21" s="13" t="str">
-        <x:v>Mailbox provider and lifecycle, inbound/outbound email, messaging/WhatsApp provider, contact masking, retention, notification events and user controls.</x:v>
+        <x:v>Which changed profile fields are material, what evidence/approvals apply, and what status/score is shown while review is pending?</x:v>
       </x:c>
       <x:c r="G21" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H21" s="13" t="str">
-        <x:v>New Consultant screen concept created; client requested email, chat, WhatsApp, and notifications.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="62" customHeight="1">
+        <x:v>Consultant can update profile over time; score recalculation follows evidence and review rules in BRD v3.2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="64" customHeight="1">
       <x:c r="A22" s="13" t="str">
-        <x:v>E18</x:v>
+        <x:v>E15</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C22" s="13" t="str">
-        <x:v>Project calendar</x:v>
+        <x:v>OptimIQ engagement history</x:v>
       </x:c>
       <x:c r="D22" s="13" t="str">
-        <x:v>Consultant account / each engagement</x:v>
+        <x:v>Consultant account</x:v>
       </x:c>
       <x:c r="E22" s="13" t="str">
-        <x:v>Show project-related milestones, meetings, and due dates across concurrent engagements.</x:v>
+        <x:v>Phase 2. View active and completed OptimIQ project assignments separately. A Consultant can work on multiple engagements at the same time. Past Project Experience remains a separate profile section for prior/outside-OptimIQ work.</x:v>
       </x:c>
       <x:c r="F22" s="13" t="str">
-        <x:v>Event types, reminders/invitations, and external calendar synchronization/provider.</x:v>
+        <x:v>Confirm fields, history retention, and concurrent capacity rules.</x:v>
       </x:c>
       <x:c r="G22" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Awaiting client feedback</x:v>
       </x:c>
       <x:c r="H22" s="13" t="str">
-        <x:v>New Consultant screen concept created.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="62" customHeight="1">
+        <x:v>Terminology clarified from client discussion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="64" customHeight="1">
       <x:c r="A23" s="13" t="str">
-        <x:v>E19</x:v>
+        <x:v>E16</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
         <x:v>Expert</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
+        <x:v>Payments and invoices</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>Consultant account / each engagement</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>Phase 2. Show payment and invoice status in the project context with a Consultant-level payout overview. Keep invoices payable to OptimIQ distinct from payouts owed by OptimIQ to the Consultant; hide internal margins/commission.</x:v>
+      </x:c>
+      <x:c r="F23" s="13" t="str">
+        <x:v>Who issues each invoice, who pays whom, whether Consultant invoices or OptimIQ pays by milestone, and visible records/timing.</x:v>
+      </x:c>
+      <x:c r="G23" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H23" s="13" t="str">
+        <x:v>New Consultant screen concept created.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="64" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>E17</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str">
+        <x:v>Communications and notifications</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="str">
+        <x:v>Consultant account</x:v>
+      </x:c>
+      <x:c r="E24" s="13" t="str">
+        <x:v>Phase 2. Provide an OptimIQ-provisioned @optimiqconsultus.com mailbox within the portal, project communications, and in-portal notifications for new emails/messages; support chat and WhatsApp integrations as approved.</x:v>
+      </x:c>
+      <x:c r="F24" s="13" t="str">
+        <x:v>Mailbox provider and lifecycle, inbound/outbound email, messaging/WhatsApp provider, contact masking, retention, notification events and user controls.</x:v>
+      </x:c>
+      <x:c r="G24" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H24" s="13" t="str">
+        <x:v>New Consultant screen concept created; client requested email, chat, WhatsApp, and notifications.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="64" customHeight="1">
+      <x:c r="A25" s="13" t="str">
+        <x:v>E18</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>Project calendar</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
+        <x:v>Consultant account / each engagement</x:v>
+      </x:c>
+      <x:c r="E25" s="13" t="str">
+        <x:v>Phase 2. Show project-related milestones, meetings, and due dates across concurrent engagements.</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="str">
+        <x:v>Event types, reminders/invitations, and external calendar synchronization/provider.</x:v>
+      </x:c>
+      <x:c r="G25" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H25" s="13" t="str">
+        <x:v>New Consultant screen concept created.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="64" customHeight="1">
+      <x:c r="A26" s="13" t="str">
+        <x:v>E19</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="str">
+        <x:v>Expert</x:v>
+      </x:c>
+      <x:c r="C26" s="13" t="str">
         <x:v>Project documents and knowledge library · Phase 2</x:v>
       </x:c>
-      <x:c r="D23" s="13" t="str">
+      <x:c r="D26" s="13" t="str">
         <x:v>Consultant and authorised Client users</x:v>
       </x:c>
-      <x:c r="E23" s="13" t="str">
-        <x:v>Provide project folders, documents, Consultant comments, and controlled Client access. Future searchable OptimIQ knowledge resources may include approved project summaries, success stories, and testimonials.</x:v>
-      </x:c>
-      <x:c r="F23" s="13" t="str">
+      <x:c r="E26" s="13" t="str">
+        <x:v>Phase 2. Provide project folders, documents, Consultant comments, and controlled Client access. Future searchable OptimIQ knowledge resources may include approved project summaries, success stories, and testimonials.</x:v>
+      </x:c>
+      <x:c r="F26" s="13" t="str">
         <x:v>Folder permissions, versions, downloads, comments, retention/deletion, consent, privacy/anonymisation, and publication/withdrawal approval.</x:v>
       </x:c>
-      <x:c r="G23" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H23" s="13" t="str">
+      <x:c r="G26" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H26" s="13" t="str">
         <x:v>Phase 2 concept only; not an initial release commitment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="62" customHeight="1">
-      <x:c r="A24" s="14" t="str">
+    <x:row r="27" ht="64" customHeight="1">
+      <x:c r="A27" s="14" t="str">
         <x:v>E20</x:v>
       </x:c>
-      <x:c r="B24" s="14" t="str">
+      <x:c r="B27" s="14" t="str">
         <x:v>Expert</x:v>
       </x:c>
-      <x:c r="C24" s="14" t="str">
+      <x:c r="C27" s="14" t="str">
         <x:v>Performance and Continuing Professional Development</x:v>
       </x:c>
-      <x:c r="D24" s="14" t="str">
+      <x:c r="D27" s="14" t="str">
         <x:v>Consultant account</x:v>
       </x:c>
-      <x:c r="E24" s="14" t="str">
-        <x:v>Review project feedback separately and record ongoing learning/professional development activity (CPD).</x:v>
-      </x:c>
-      <x:c r="F24" s="14" t="str">
+      <x:c r="E27" s="14" t="str">
+        <x:v>Phase 2. Review project feedback separately and record ongoing learning/professional development activity (CPD).</x:v>
+      </x:c>
+      <x:c r="F27" s="14" t="str">
         <x:v>Whether feedback changes the composite/performance score, feedback aggregation/moderation, CPD evidence/units/validation and certification impact.</x:v>
       </x:c>
-      <x:c r="G24" s="14" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="H24" s="14" t="str">
+      <x:c r="G27" s="14" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H27" s="14" t="str">
         <x:v>New Consultant screen concept created; CPD acronym expanded and operating rules open.</x:v>
       </x:c>
     </x:row>
@@ -1498,94 +1603,66 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="60" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="2" t="str">
+      <x:c r="A1" s="86" t="str">
         <x:v>Consulting Firm · Screen Approval Inventory</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="str">
-        <x:v>Consulting Firm · Screen Approval Inventory</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="E2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-      <x:c r="H2" s="5" t="str">
-        <x:v>Full firm lifecycle mapped to BRD F1–F8 and firm forms. The single firm account and Theme 1 shell follow the user decisions; unresolved policy is in Open Clarifications.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="8" t="str">
+      <x:c r="B1" s="86"/>
+      <x:c r="C1" s="86"/>
+      <x:c r="D1" s="86"/>
+      <x:c r="E1" s="86"/>
+      <x:c r="F1" s="86"/>
+      <x:c r="G1" s="86"/>
+      <x:c r="H1" s="86"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="89" t="str">
+        <x:v>Phase 1: CTA, shared sign-in, terms and six-section CTQ. Dashboard and all later firm screens are Phase 2.</x:v>
+      </x:c>
+      <x:c r="B2" s="89"/>
+      <x:c r="C2" s="89"/>
+      <x:c r="D2" s="89"/>
+      <x:c r="E2" s="89"/>
+      <x:c r="F2" s="89"/>
+      <x:c r="G2" s="89"/>
+      <x:c r="H2" s="89"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="92" t="str">
         <x:v>Screen ID</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B4" s="92" t="str">
         <x:v>Workspace</x:v>
       </x:c>
-      <x:c r="C4" s="8" t="str">
+      <x:c r="C4" s="92" t="str">
         <x:v>Screen / design unit</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="str">
+      <x:c r="D4" s="92" t="str">
         <x:v>Roles / variants</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="str">
+      <x:c r="E4" s="92" t="str">
         <x:v>Purpose and client review focus</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="F4" s="92" t="str">
         <x:v>Clarification to park</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
+      <x:c r="G4" s="92" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H4" s="8" t="str">
+      <x:c r="H4" s="92" t="str">
         <x:v>Client decision / notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="62" customHeight="1">
+    <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>F01</x:v>
       </x:c>
@@ -1599,7 +1676,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Existing registration form collects company/contact details and handles email verification and password setup before portal sign-in.</x:v>
+        <x:v>Phase 1. Existing registration form collects company/contact details and handles email verification and password setup before portal sign-in.</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>Already-built CTA form; no redesign in this phase.</x:v>
@@ -1611,7 +1688,7 @@
         <x:v>Link to existing client form; do not duplicate registration in the portal.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="62" customHeight="1">
+    <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="13" t="str">
         <x:v>F02</x:v>
       </x:c>
@@ -1625,7 +1702,7 @@
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="E6" s="13" t="str">
-        <x:v>Use the shared portal login; route a registered firm account into its firm workspace.</x:v>
+        <x:v>Phase 1. Use the shared portal login; route a registered firm account into its firm workspace.</x:v>
       </x:c>
       <x:c r="F6" s="13" t="str">
         <x:v>Account recovery and identity routing details remain open for developer confirmation.</x:v>
@@ -1637,7 +1714,7 @@
         <x:v>Same login screen as other audiences; identity setup occurs in CTA.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="62" customHeight="1">
+    <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="13" t="str">
         <x:v>F03</x:v>
       </x:c>
@@ -1651,7 +1728,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
-        <x:v>After first shared sign-in, review and accept required firm terms and declarations when not completed in CTA.</x:v>
+        <x:v>Phase 1. After first shared sign-in, review and accept required firm terms and declarations when not completed in CTA.</x:v>
       </x:c>
       <x:c r="F7" s="13" t="str">
         <x:v>Legal text, affiliate declaration scope, and which agreements apply at registration remain open.</x:v>
@@ -1663,7 +1740,7 @@
         <x:v>Uses the same terms screen structure as Consultant; firm-specific document content needs approval.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="62" customHeight="1">
+    <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="13" t="str">
         <x:v>F04</x:v>
       </x:c>
@@ -1671,13 +1748,13 @@
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C8" s="13" t="str">
-        <x:v>Firm profile &amp; CTQ stepper</x:v>
+        <x:v>Firm CTQ form · six sections</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Complete the approved six-step, 23-question firm CTQ profile; save draft and submit once complete.</x:v>
+        <x:v>Phase 1. Complete the approved six-step, 23-question firm CTQ profile; save draft and submit once complete.</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
         <x:v>Answer-band boundaries for B04/B05/C01/C02, evidence verification rule, and handling of unanswered Good-to-Have/Optional items.</x:v>
@@ -1689,7 +1766,7 @@
         <x:v>CTA is the separate prior registration step; client confirmed the CTQ is six sections. Do not show internal IDs, weights, or raw score.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="62" customHeight="1">
+    <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>F05</x:v>
       </x:c>
@@ -1703,7 +1780,7 @@
         <x:v>One firm account</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>Show qualification status, active work, alerts, and a left navigation listing all firm processes.</x:v>
+        <x:v>Phase 2. Post-CTQ view of firm profile and operating processes.</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
         <x:v>Exact member-facing tier wording and whether a preliminary tier is shown before OptimIQ review; phase mapping conflict with BRD.</x:v>
@@ -1715,7 +1792,7 @@
         <x:v>One login and one workspace; Seller, Buyer, Win-and-Staff are modes/process areas, not separate accounts.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="62" customHeight="1">
+    <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="13" t="str">
         <x:v>F06</x:v>
       </x:c>
@@ -1729,7 +1806,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>Track corporate compliance, evidence/reference review, panel decision, MOU, listing, and onboarding.</x:v>
+        <x:v>Phase 2. Track corporate compliance, evidence/reference review, panel decision, MOU, listing, and onboarding.</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
         <x:v>Document list, evidence standard, reference rules, panel decision states, and appeal/rework workflow.</x:v>
@@ -1741,7 +1818,7 @@
         <x:v>Mapped to BRD F4.1–F4.4. Exact screen waits for client approval of requirements.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="62" customHeight="1">
+    <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="13" t="str">
         <x:v>F07</x:v>
       </x:c>
@@ -1755,7 +1832,7 @@
         <x:v>Firm account · Seller mode</x:v>
       </x:c>
       <x:c r="E11" s="13" t="str">
-        <x:v>Show firm membership status, package, eligibility, and renewal state.</x:v>
+        <x:v>Phase 2. Show firm membership status, package, eligibility, and renewal state.</x:v>
       </x:c>
       <x:c r="F11" s="13" t="str">
         <x:v>Membership packages, fees, benefits, duration, and relationship to Tier qualification.</x:v>
@@ -1767,7 +1844,7 @@
         <x:v>BRD F5S.1. Commercial values should be configurable in Admin after business decisions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="62" customHeight="1">
+    <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="13" t="str">
         <x:v>F08</x:v>
       </x:c>
@@ -1781,7 +1858,7 @@
         <x:v>Firm Seller mode</x:v>
       </x:c>
       <x:c r="E12" s="13" t="str">
-        <x:v>Review eligible client opportunities and manage firm participation without exposing rival bids.</x:v>
+        <x:v>Phase 2. Review eligible client opportunities and manage firm participation without exposing rival bids.</x:v>
       </x:c>
       <x:c r="F12" s="13" t="str">
         <x:v>Opportunity visibility, eligibility, filters, and exception handling.</x:v>
@@ -1793,7 +1870,7 @@
         <x:v>Mapped to BRD F5S.2. A firm may also be Buyer in a project, subject to fairness controls.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="62" customHeight="1">
+    <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="13" t="str">
         <x:v>F09</x:v>
       </x:c>
@@ -1807,7 +1884,7 @@
         <x:v>Firm Seller mode</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
-        <x:v>Request or review OptimIQ bid support for eligible opportunities.</x:v>
+        <x:v>Phase 2. Request or review OptimIQ bid support for eligible opportunities.</x:v>
       </x:c>
       <x:c r="F13" s="13" t="str">
         <x:v>Whether support is optional/charged, fee basis, approval, and status.</x:v>
@@ -1819,7 +1896,7 @@
         <x:v>Mapped to BRD F5S.3. Fees configurable; amount is not specified.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="62" customHeight="1">
+    <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="13" t="str">
         <x:v>F10</x:v>
       </x:c>
@@ -1833,7 +1910,7 @@
         <x:v>Firm Seller mode</x:v>
       </x:c>
       <x:c r="E14" s="13" t="str">
-        <x:v>Create separate technical and commercial bid responses, then track submission, negotiation, opening, and reverse-auction steps if applicable.</x:v>
+        <x:v>Phase 2. Create separate technical and commercial bid responses, then track submission, negotiation, opening, and reverse-auction steps if applicable.</x:v>
       </x:c>
       <x:c r="F14" s="13" t="str">
         <x:v>Required bid fields, commercial model, edit/withdraw rules, evaluation visibility, auction conditions, and sequence with LOI/agreement.</x:v>
@@ -1845,7 +1922,7 @@
         <x:v>Mapped to BRD F5S.4–F5S.6. Keep rival bids private and separate technical and commercial information.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="62" customHeight="1">
+    <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="13" t="str">
         <x:v>F11</x:v>
       </x:c>
@@ -1859,7 +1936,7 @@
         <x:v>Firm Buyer mode</x:v>
       </x:c>
       <x:c r="E15" s="13" t="str">
-        <x:v>Submit a talent requirement for an OptimIQ Expert for the firm’s mandate.</x:v>
+        <x:v>Phase 2. Submit a talent requirement for an OptimIQ Expert for the firm’s mandate.</x:v>
       </x:c>
       <x:c r="F15" s="13" t="str">
         <x:v>Request fields, budget/commercial terms, service levels, and Buyer-to-OptimIQ fee treatment.</x:v>
@@ -1871,7 +1948,7 @@
         <x:v>Mapped to BRD F5B.1. For external mandates, OptimIQ only sources Experts; it does not audit the external contract.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="62" customHeight="1">
+    <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="13" t="str">
         <x:v>F12</x:v>
       </x:c>
@@ -1885,7 +1962,7 @@
         <x:v>Firm Buyer mode</x:v>
       </x:c>
       <x:c r="E16" s="13" t="str">
-        <x:v>Review permitted masked profiles, interview candidates, choose an Expert, and record the LOI state.</x:v>
+        <x:v>Phase 2. Review permitted masked profiles, interview candidates, choose an Expert, and record the LOI state.</x:v>
       </x:c>
       <x:c r="F16" s="13" t="str">
         <x:v>Matching criteria, shortlist size, masking/release gate, interview workflow, and LOI wording.</x:v>
@@ -1897,7 +1974,7 @@
         <x:v>Mapped to BRD F5B.2–F5B.4. Do not expose internal OptimIQ commercial information.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="62" customHeight="1">
+    <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="13" t="str">
         <x:v>F13</x:v>
       </x:c>
@@ -1911,7 +1988,7 @@
         <x:v>Firm Seller + Buyer modes</x:v>
       </x:c>
       <x:c r="E17" s="13" t="str">
-        <x:v>Link a bid team, request Expert reservation with consent, convert after award, or release if the firm loses.</x:v>
+        <x:v>Phase 2. Link a bid team, request Expert reservation with consent, convert after award, or release if the firm loses.</x:v>
       </x:c>
       <x:c r="F17" s="13" t="str">
         <x:v>Reservation period, consent detail, fees, automation phase, and agreement sequence before award/introduction.</x:v>
@@ -1923,7 +2000,7 @@
         <x:v>Mapped to BRD F5W.1–F5W.3. No Expert is deployed before the firm wins.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="62" customHeight="1">
+    <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="13" t="str">
         <x:v>F14</x:v>
       </x:c>
@@ -1937,7 +2014,7 @@
         <x:v>Firm Seller / Buyer project</x:v>
       </x:c>
       <x:c r="E18" s="13" t="str">
-        <x:v>Track required agreement signatures before award and introduction.</x:v>
+        <x:v>Phase 2. Track required agreement signatures before award and introduction.</x:v>
       </x:c>
       <x:c r="F18" s="13" t="str">
         <x:v>Agreement types, parties/signatories, and order relative to LOI; client feedback conflicts with BRD LOI/contract sequence.</x:v>
@@ -1949,7 +2026,7 @@
         <x:v>Client rule is approved: agreements signed before award and introduction. Keep exact document sequence open.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="62" customHeight="1">
+    <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="13" t="str">
         <x:v>F15</x:v>
       </x:c>
@@ -1963,7 +2040,7 @@
         <x:v>Firm account · project-scoped</x:v>
       </x:c>
       <x:c r="E19" s="13" t="str">
-        <x:v>Track mobilisation, delivery milestones, acceptance/rework, and close-out for OptimIQ engagements.</x:v>
+        <x:v>Phase 2. Track mobilisation, delivery milestones, acceptance/rework, and close-out for OptimIQ engagements.</x:v>
       </x:c>
       <x:c r="F19" s="13" t="str">
         <x:v>Milestone catalogue, acceptance rules, amendments, and which firm/Expert activities are visible.</x:v>
@@ -1975,7 +2052,7 @@
         <x:v>Mapped to BRD F6. External projects are not audited by OptimIQ; internal employee deployment remains firm-internal.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="62" customHeight="1">
+    <x:row r="20" ht="64" customHeight="1">
       <x:c r="A20" s="13" t="str">
         <x:v>F16</x:v>
       </x:c>
@@ -1989,7 +2066,7 @@
         <x:v>Firm account · project-scoped</x:v>
       </x:c>
       <x:c r="E20" s="13" t="str">
-        <x:v>Show firm-facing invoices and payment status while separating seller revenue and buyer payments.</x:v>
+        <x:v>Phase 2. Show firm-facing invoices and payment status while separating seller revenue and buyer payments.</x:v>
       </x:c>
       <x:c r="F20" s="13" t="str">
         <x:v>Invoice issuer/payee by flow, fee shares, payment milestones, refunds, and OptimIQ-sourced Expert commercial treatment.</x:v>
@@ -2001,7 +2078,7 @@
         <x:v>BRD separates seller and buyer money. Internal OptimIQ margin/commission is private.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="62" customHeight="1">
+    <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="13" t="str">
         <x:v>F17</x:v>
       </x:c>
@@ -2015,7 +2092,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E21" s="13" t="str">
-        <x:v>Potential inbox for firm/project communications and notification updates.</x:v>
+        <x:v>Phase 2. Potential inbox for firm/project communications and notification updates.</x:v>
       </x:c>
       <x:c r="F21" s="13" t="str">
         <x:v>Whether firm gets portal email/chat/WhatsApp, address lifecycle, provider, notification events, masking, and retention.</x:v>
@@ -2027,7 +2104,7 @@
         <x:v>Consultant feedback requested these integrations; firm-specific use is not defined by BRD.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="62" customHeight="1">
+    <x:row r="22" ht="64" customHeight="1">
       <x:c r="A22" s="13" t="str">
         <x:v>F18</x:v>
       </x:c>
@@ -2041,7 +2118,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E22" s="13" t="str">
-        <x:v>Potential calendar of project meetings, milestones, and due dates.</x:v>
+        <x:v>Phase 2. Potential calendar of project meetings, milestones, and due dates.</x:v>
       </x:c>
       <x:c r="F22" s="13" t="str">
         <x:v>Event types, invitation/RSVP behavior, reminders, external sync, and provider.</x:v>
@@ -2053,7 +2130,7 @@
         <x:v>Keep aligned with shared Theme 1 calendar components if confirmed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="62" customHeight="1">
+    <x:row r="23" ht="64" customHeight="1">
       <x:c r="A23" s="13" t="str">
         <x:v>F19</x:v>
       </x:c>
@@ -2067,7 +2144,7 @@
         <x:v>Firm account · project scoped</x:v>
       </x:c>
       <x:c r="E23" s="13" t="str">
-        <x:v>Potential controlled folder access for firm project files and comments.</x:v>
+        <x:v>Phase 2. Potential controlled folder access for firm project files and comments.</x:v>
       </x:c>
       <x:c r="F23" s="13" t="str">
         <x:v>Firm visibility, Client/Expert sharing, versioning, retention, download, comments, and phase.</x:v>
@@ -2079,7 +2156,7 @@
         <x:v>Client proposed project folders and knowledge library as Phase 2; firm-specific access is not specified.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="62" customHeight="1">
+    <x:row r="24" ht="64" customHeight="1">
       <x:c r="A24" s="13" t="str">
         <x:v>F20</x:v>
       </x:c>
@@ -2093,7 +2170,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E24" s="13" t="str">
-        <x:v>Show approved delivery feedback and periodic relationship review. Keep Seller performance based on Seller work, separate from Buyer payment behavior.</x:v>
+        <x:v>Phase 2. Show approved delivery feedback and periodic relationship review. Keep Seller performance based on Seller work, separate from Buyer payment behavior.</x:v>
       </x:c>
       <x:c r="F24" s="13" t="str">
         <x:v>Firm KPIs, rating scale, visibility, moderation, and any effect on tier/composite score.</x:v>
@@ -2105,7 +2182,7 @@
         <x:v>BRD fairness rule DR10: seller performance is judged on selling only, not buyer payment behavior.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="62" customHeight="1">
+    <x:row r="25" ht="64" customHeight="1">
       <x:c r="A25" s="13" t="str">
         <x:v>F21</x:v>
       </x:c>
@@ -2119,7 +2196,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E25" s="13" t="str">
-        <x:v>Track renewal, periodic tier review, pause, reinstatement, and current membership state.</x:v>
+        <x:v>Phase 2. Track renewal, periodic tier review, pause, reinstatement, and current membership state.</x:v>
       </x:c>
       <x:c r="F25" s="13" t="str">
         <x:v>Renewal cycles, notice periods, triggers, consequences, and appeal/reinstatement rules.</x:v>
@@ -2131,7 +2208,7 @@
         <x:v>Mapped to BRD F8.2–F8.3; tier thresholds are in the BRD but application of updates needs business confirmation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="62" customHeight="1">
+    <x:row r="26" ht="64" customHeight="1">
       <x:c r="A26" s="13" t="str">
         <x:v>F22</x:v>
       </x:c>
@@ -2145,7 +2222,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E26" s="13" t="str">
-        <x:v>Submit and track firm grievances or profile/change requests.</x:v>
+        <x:v>Phase 2. Submit and track firm grievances or profile/change requests.</x:v>
       </x:c>
       <x:c r="F26" s="13" t="str">
         <x:v>Categories, required evidence, review owner, response target, escalation, and appeal flow.</x:v>
@@ -2157,7 +2234,7 @@
         <x:v>BRD F-S01/F-S02; detailed form and status lifecycle not specified.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="62" customHeight="1">
+    <x:row r="27" ht="64" customHeight="1">
       <x:c r="A27" s="14" t="str">
         <x:v>F23</x:v>
       </x:c>
@@ -2171,7 +2248,7 @@
         <x:v>Firm account</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>Submit exit notice and review open-project handling, closure, and settlement status.</x:v>
+        <x:v>Phase 2. Submit exit notice and review open-project handling, closure, and settlement status.</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
         <x:v>Notice period, open engagement treatment, data retention, final settlement, and exit interview flow.</x:v>
@@ -2207,52 +2284,52 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="78" t="str">
+      <x:c r="A1" s="86" t="str">
         <x:v>Client · Screen Approval Inventory</x:v>
       </x:c>
-      <x:c r="B1" s="78"/>
-      <x:c r="C1" s="78"/>
-      <x:c r="D1" s="78"/>
-      <x:c r="E1" s="78"/>
-      <x:c r="F1" s="78"/>
-      <x:c r="G1" s="78"/>
-      <x:c r="H1" s="78"/>
+      <x:c r="B1" s="86"/>
+      <x:c r="C1" s="86"/>
+      <x:c r="D1" s="86"/>
+      <x:c r="E1" s="86"/>
+      <x:c r="F1" s="86"/>
+      <x:c r="G1" s="86"/>
+      <x:c r="H1" s="86"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="81" t="str">
-        <x:v>Client lifecycle based on BRD C1–C8 and the approved Client Categorisation workbook. Internal scores/segments remain hidden. Shared Theme 1 components align to Consultant and Consulting Firm.</x:v>
-      </x:c>
-      <x:c r="B2" s="81"/>
-      <x:c r="C2" s="81"/>
-      <x:c r="D2" s="81"/>
-      <x:c r="E2" s="81"/>
-      <x:c r="F2" s="81"/>
-      <x:c r="G2" s="81"/>
-      <x:c r="H2" s="81"/>
+      <x:c r="A2" s="89" t="str">
+        <x:v>Phase 1: CTA, shared sign-in, terms and optional Client CTQ. Dashboard and all later screens are Phase 2. The CTQ placement needs client confirmation.</x:v>
+      </x:c>
+      <x:c r="B2" s="89"/>
+      <x:c r="C2" s="89"/>
+      <x:c r="D2" s="89"/>
+      <x:c r="E2" s="89"/>
+      <x:c r="F2" s="89"/>
+      <x:c r="G2" s="89"/>
+      <x:c r="H2" s="89"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="84" t="str">
+      <x:c r="A4" s="92" t="str">
         <x:v>Screen ID</x:v>
       </x:c>
-      <x:c r="B4" s="84" t="str">
+      <x:c r="B4" s="92" t="str">
         <x:v>Workspace</x:v>
       </x:c>
-      <x:c r="C4" s="84" t="str">
+      <x:c r="C4" s="92" t="str">
         <x:v>Screen / design unit</x:v>
       </x:c>
-      <x:c r="D4" s="84" t="str">
+      <x:c r="D4" s="92" t="str">
         <x:v>Roles / variants</x:v>
       </x:c>
-      <x:c r="E4" s="84" t="str">
+      <x:c r="E4" s="92" t="str">
         <x:v>Purpose and client review focus</x:v>
       </x:c>
-      <x:c r="F4" s="84" t="str">
+      <x:c r="F4" s="92" t="str">
         <x:v>Clarification to park</x:v>
       </x:c>
-      <x:c r="G4" s="84" t="str">
+      <x:c r="G4" s="92" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H4" s="84" t="str">
+      <x:c r="H4" s="92" t="str">
         <x:v>Client decision / notes</x:v>
       </x:c>
     </x:row>
@@ -2264,13 +2341,13 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Client CTA enquiry</x:v>
+        <x:v>Client CTA registration</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>Client / existing public form</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Existing For Clients form; link as-is and do not redesign.</x:v>
+        <x:v>Phase 1. Existing public registration and enquiry form; keep it unchanged.</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>None for this screen; its relationship to portal account creation is in CL-01.</x:v>
@@ -2290,22 +2367,22 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C6" s="13" t="str">
-        <x:v>Optional client details / categorisation enrichment</x:v>
+        <x:v>Portal sign-in</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
-        <x:v>Client / optional pre-login step</x:v>
+        <x:v>Client / shared identity</x:v>
       </x:c>
       <x:c r="E6" s="13" t="str">
-        <x:v>Three optional fields: project budget, preferred start timeline, decision-making role. Skip is always available.</x:v>
+        <x:v>Phase 1. One shared sign-in routes the client account to its terms and CTQ journey.</x:v>
       </x:c>
       <x:c r="F6" s="13" t="str">
-        <x:v>Whether the step opens from the confirmation page or email link is a presentation detail; client scoring precision is CL-02.</x:v>
+        <x:v>Account invitation/self-start, OTP, and relation to the existing CTA require reconciliation (CL-01).</x:v>
       </x:c>
       <x:c r="G6" s="13" t="str">
-        <x:v>Awaiting screen feedback</x:v>
+        <x:v>Already designed · shared screen</x:v>
       </x:c>
       <x:c r="H6" s="13" t="str">
-        <x:v>Workbook-approved fields and skippable behavior; no score or segment is displayed.</x:v>
+        <x:v>Login after CTA follows the agreed audience sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
@@ -2316,22 +2393,22 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C7" s="13" t="str">
-        <x:v>Shared portal sign-in</x:v>
+        <x:v>Terms &amp; declarations</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>Client / shared identity</x:v>
+        <x:v>Client account holder</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
-        <x:v>Use the single shared sign-in and route the account to the client journey.</x:v>
+        <x:v>Phase 1. Review and accept required account terms before the Client CTQ.</x:v>
       </x:c>
       <x:c r="F7" s="13" t="str">
-        <x:v>Account invitation/self-start, OTP, and relation to the existing CTA require reconciliation (CL-01).</x:v>
+        <x:v>Exact document list, signer authority, payment setup, and legal wording (CL-03).</x:v>
       </x:c>
       <x:c r="G7" s="13" t="str">
-        <x:v>Already designed · shared screen</x:v>
+        <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H7" s="13" t="str">
-        <x:v>Login after CTA follows the agreed audience sequence.</x:v>
+        <x:v>Use the same Theme 1 terms structure as Consultant and Consulting Firm.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
@@ -2342,22 +2419,22 @@
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C8" s="13" t="str">
-        <x:v>Terms &amp; declarations</x:v>
+        <x:v>Client CTQ form · optional</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
-        <x:v>Client account holder</x:v>
+        <x:v>Client / one section after sign-in</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Review and accept client account terms after sign-in if not already accepted.</x:v>
+        <x:v>Phase 1. Three optional questions: budget, preferred start and decision role. Skip remains available. The client sees no score or segment.</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
-        <x:v>Exact document list, signer authority, payment setup, and legal wording (CL-03).</x:v>
+        <x:v>The Client workbook places these questions immediately after CTA without login; the unified portal flow places them after sign-in and terms (CL-01).</x:v>
       </x:c>
       <x:c r="G8" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Awaiting screen feedback</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
-        <x:v>Use the same Theme 1 terms structure as Consultant and Consulting Firm.</x:v>
+        <x:v>Client feedback defines this optional enrichment screen as the Client CTQ.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -2374,7 +2451,7 @@
         <x:v>Client account holder</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>360° client view, with Phase 1 account/categorisation and Phase 2 requirements/projects views.</x:v>
+        <x:v>Phase 2. Post-CTQ client dashboard and account/project overview.</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
         <x:v>Exact dashboard metrics and phase mapping conflict with BRD Phase 1 labels (CL-04).</x:v>
@@ -2400,7 +2477,7 @@
         <x:v>Client account holder</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>Review organisation and contact information in the client account.</x:v>
+        <x:v>Phase 2. Review organisation and contact information in the client account.</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
         <x:v>Editable fields, profile update evidence, approval, and change history (CL-05).</x:v>
@@ -2426,7 +2503,7 @@
         <x:v>Client account; Solution Coordinator</x:v>
       </x:c>
       <x:c r="E11" s="13" t="str">
-        <x:v>Create a client requirement from the portal; OptimIQ scopes and routes it.</x:v>
+        <x:v>Phase 2. Create a client requirement from the portal; OptimIQ scopes and routes it.</x:v>
       </x:c>
       <x:c r="F11" s="13" t="str">
         <x:v>Exact form fields, required attachments, edit/withdraw states, coordinator assignment, and fee display (CL-06).</x:v>
@@ -2452,7 +2529,7 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E12" s="13" t="str">
-        <x:v>Review the normal 2–3 curated masked profiles and recommendation rationale.</x:v>
+        <x:v>Phase 2. Review the normal 2–3 curated masked profiles and recommendation rationale.</x:v>
       </x:c>
       <x:c r="F12" s="13" t="str">
         <x:v>Visible profile attributes, comparison criteria, and client decision controls (CL-07).</x:v>
@@ -2478,7 +2555,7 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
-        <x:v>Inspect permitted experience, fit, and capability details for a shortlisted seller.</x:v>
+        <x:v>Phase 2. Inspect permitted experience, fit, and capability details for a shortlisted seller.</x:v>
       </x:c>
       <x:c r="F13" s="13" t="str">
         <x:v>Which profile information may be shown before identity-release approval (CL-07).</x:v>
@@ -2504,7 +2581,7 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E14" s="13" t="str">
-        <x:v>Ask OptimIQ for more profiles if the initial shortlist is unsuitable.</x:v>
+        <x:v>Phase 2. Ask OptimIQ for more profiles if the initial shortlist is unsuitable.</x:v>
       </x:c>
       <x:c r="F14" s="13" t="str">
         <x:v>Exception approval, evidence, reason capture, and number of additional profiles (CL-08).</x:v>
@@ -2530,7 +2607,7 @@
         <x:v>Client account; Procurement Desk</x:v>
       </x:c>
       <x:c r="E15" s="13" t="str">
-        <x:v>Follow technical evaluation (TER), financial evaluation (FER), decision, and tender status.</x:v>
+        <x:v>Phase 2. Follow technical evaluation (TER), financial evaluation (FER), decision, and tender status.</x:v>
       </x:c>
       <x:c r="F15" s="13" t="str">
         <x:v>Routing threshold, evaluation method, weights, scoring visibility, and client decision rights (CL-09).</x:v>
@@ -2556,7 +2633,7 @@
         <x:v>Client account; selected seller</x:v>
       </x:c>
       <x:c r="E16" s="13" t="str">
-        <x:v>Show required signature gate before award and introduction, following client feedback.</x:v>
+        <x:v>Phase 2. Show required signature gate before award and introduction, following client feedback.</x:v>
       </x:c>
       <x:c r="F16" s="13" t="str">
         <x:v>Document types, signatories, and sequence relative to LOI/contract conflict with BRD (CL-10).</x:v>
@@ -2582,7 +2659,7 @@
         <x:v>Client account; OptimIQ staff; seller</x:v>
       </x:c>
       <x:c r="E17" s="13" t="str">
-        <x:v>Coordinate approved scoping, evaluation, and post-award introduction meetings.</x:v>
+        <x:v>Phase 2. Coordinate approved scoping, evaluation, and post-award introduction meetings.</x:v>
       </x:c>
       <x:c r="F17" s="13" t="str">
         <x:v>Provider, recording, consent, identity disclosure, and timing (CL-11).</x:v>
@@ -2608,7 +2685,7 @@
         <x:v>Client account; engagement participants</x:v>
       </x:c>
       <x:c r="E18" s="13" t="str">
-        <x:v>Review mobilisation, milestones, submitted work, acceptance/rework, approved changes, and close-out.</x:v>
+        <x:v>Phase 2. Review mobilisation, milestones, submitted work, acceptance/rework, approved changes, and close-out.</x:v>
       </x:c>
       <x:c r="F18" s="13" t="str">
         <x:v>Milestone catalogue, review window, change approval, and dispute details (CL-12).</x:v>
@@ -2634,7 +2711,7 @@
         <x:v>Client account; Finance</x:v>
       </x:c>
       <x:c r="E19" s="13" t="str">
-        <x:v>Review client invoices, amounts due, payments, and receipts in project context.</x:v>
+        <x:v>Phase 2. Review client invoices, amounts due, payments, and receipts in project context.</x:v>
       </x:c>
       <x:c r="F19" s="13" t="str">
         <x:v>Fees, invoice timing, payment methods, cancellations, refunds, and fee visibility (CL-13).</x:v>
@@ -2660,7 +2737,7 @@
         <x:v>Client account; per engagement</x:v>
       </x:c>
       <x:c r="E20" s="13" t="str">
-        <x:v>Give seller feedback at milestone and project close; return to create repeat requirements.</x:v>
+        <x:v>Phase 2. Give seller feedback at milestone and project close; return to create repeat requirements.</x:v>
       </x:c>
       <x:c r="F20" s="13" t="str">
         <x:v>Whether client feedback changes composite/performance scores or appears as a separate signal (CL-14).</x:v>
@@ -2686,7 +2763,7 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E21" s="13" t="str">
-        <x:v>See OptimIQ messages, project updates, and action notifications.</x:v>
+        <x:v>Phase 2. See OptimIQ messages, project updates, and action notifications.</x:v>
       </x:c>
       <x:c r="F21" s="13" t="str">
         <x:v>Email/chat/WhatsApp, portal mailbox, event triggers, and provider (CL-15).</x:v>
@@ -2712,7 +2789,7 @@
         <x:v>Client account</x:v>
       </x:c>
       <x:c r="E22" s="13" t="str">
-        <x:v>Review requirement calls, meetings, milestones, and deadlines.</x:v>
+        <x:v>Phase 2. Review requirement calls, meetings, milestones, and deadlines.</x:v>
       </x:c>
       <x:c r="F22" s="13" t="str">
         <x:v>Event types, calendar sync, invite rules, and meeting-specific recording behavior (CL-16).</x:v>
@@ -2738,7 +2815,7 @@
         <x:v>Client account; approved project participants</x:v>
       </x:c>
       <x:c r="E23" s="13" t="str">
-        <x:v>Access approved project files and consultant comments for the relevant project.</x:v>
+        <x:v>Phase 2. Access approved project files and consultant comments for the relevant project.</x:v>
       </x:c>
       <x:c r="F23" s="13" t="str">
         <x:v>Folder permissions, retention, upload policy, and knowledge-library/success-story reuse (CL-17).</x:v>
@@ -2764,7 +2841,7 @@
         <x:v>Client account; support / grievance staff</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>Raise and track a grievance/support request and review account status or exit.</x:v>
+        <x:v>Phase 2. Raise and track a grievance/support request and review account status or exit.</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
         <x:v>Intake categories, escalation, response targets, open-project handling, retention, and settlement (CL-18).</x:v>
@@ -3186,47 +3263,47 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="78" t="str">
+      <x:c r="A1" s="86" t="str">
         <x:v>Open Clarifications</x:v>
       </x:c>
-      <x:c r="B1" s="78"/>
-      <x:c r="C1" s="78"/>
-      <x:c r="D1" s="78"/>
-      <x:c r="E1" s="78"/>
-      <x:c r="F1" s="78"/>
-      <x:c r="G1" s="78"/>
+      <x:c r="B1" s="86"/>
+      <x:c r="C1" s="86"/>
+      <x:c r="D1" s="86"/>
+      <x:c r="E1" s="86"/>
+      <x:c r="F1" s="86"/>
+      <x:c r="G1" s="86"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="81" t="str">
+      <x:c r="A2" s="89" t="str">
         <x:v>Questions that affect screen content, workflow, or architecture. Agreed requirements are recorded on the audience sheet and are not repeated here.</x:v>
       </x:c>
-      <x:c r="B2" s="81"/>
-      <x:c r="C2" s="81"/>
-      <x:c r="D2" s="81"/>
-      <x:c r="E2" s="81"/>
-      <x:c r="F2" s="81"/>
-      <x:c r="G2" s="81"/>
+      <x:c r="B2" s="89"/>
+      <x:c r="C2" s="89"/>
+      <x:c r="D2" s="89"/>
+      <x:c r="E2" s="89"/>
+      <x:c r="F2" s="89"/>
+      <x:c r="G2" s="89"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
-      <x:c r="A4" s="84" t="str">
+      <x:c r="A4" s="92" t="str">
         <x:v>Clarification ID</x:v>
       </x:c>
-      <x:c r="B4" s="84" t="str">
+      <x:c r="B4" s="92" t="str">
         <x:v>Audience</x:v>
       </x:c>
-      <x:c r="C4" s="84" t="str">
+      <x:c r="C4" s="92" t="str">
         <x:v>Affected screen</x:v>
       </x:c>
-      <x:c r="D4" s="84" t="str">
+      <x:c r="D4" s="92" t="str">
         <x:v>Question / decision needed</x:v>
       </x:c>
-      <x:c r="E4" s="84" t="str">
+      <x:c r="E4" s="92" t="str">
         <x:v>Source / conflict</x:v>
       </x:c>
-      <x:c r="F4" s="84" t="str">
+      <x:c r="F4" s="92" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G4" s="84" t="str">
+      <x:c r="G4" s="92" t="str">
         <x:v>Working assumption shown in wireframe</x:v>
       </x:c>
     </x:row>
@@ -3301,739 +3378,711 @@
     </x:row>
     <x:row r="8" ht="65" customHeight="1">
       <x:c r="A8" s="13" t="str">
-        <x:v>CF-04</x:v>
+        <x:v>CF-05</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C8" s="13" t="str">
-        <x:v>F05 / all firm screens</x:v>
+        <x:v>F02 · Shared sign-in / user roles</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
-        <x:v>Which development phase includes F4–F8 firm processes? The previous approved wireframe convention says Phase 1 ends after CTQ; BRD Tables 49/60 put most firm lifecycle activity in Phase 1, with Win-and-Staff automation in Phase 2.</x:v>
+        <x:v>Does each firm remain a single login with no invited employee accounts? BRD F-F03 describes user and role setup, while the user clarified one firm login.</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>BRD Tables 49 and 60; user-approved wireframe phase rule</x:v>
+        <x:v>BRD Table 56 F-F03; direct user decision</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Needs clarification · BRD conflict</x:v>
       </x:c>
       <x:c r="G8" s="13" t="str">
-        <x:v>Continue showing current wireframe phase convention, clearly marked provisional.</x:v>
+        <x:v>Wireframe follows the direct user decision: one firm login. Do not show employee invites until the BRD is reconciled.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="65" customHeight="1">
       <x:c r="A9" s="13" t="str">
-        <x:v>CF-05</x:v>
+        <x:v>CF-06</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C9" s="13" t="str">
-        <x:v>F02 · Shared sign-in / user roles</x:v>
+        <x:v>F06 · Qualification</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>Does each firm remain a single login with no invited employee accounts? BRD F-F03 describes user and role setup, while the user clarified one firm login.</x:v>
+        <x:v>What exact company documents, case-study evidence, references, verification states, and review/appeal outcomes are required?</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>BRD Table 56 F-F03; direct user decision</x:v>
+        <x:v>BRD F4.1–F4.4, F-I07, F-I05</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
-        <x:v>Needs clarification · BRD conflict</x:v>
+        <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G9" s="13" t="str">
-        <x:v>Wireframe follows the direct user decision: one firm login. Do not show employee invites until the BRD is reconciled.</x:v>
+        <x:v>Show progress/status placeholders; do not invent a mandatory checklist.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="65" customHeight="1">
       <x:c r="A10" s="13" t="str">
-        <x:v>CF-06</x:v>
+        <x:v>CF-07</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>F06 · Qualification</x:v>
+        <x:v>F07/F21 · Membership</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>What exact company documents, case-study evidence, references, verification states, and review/appeal outcomes are required?</x:v>
+        <x:v>What membership packages, fees, benefits, duration, and renewal rules apply?</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>BRD F4.1–F4.4, F-I07, F-I05</x:v>
+        <x:v>BRD F5S.1, F8.2–F8.3</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G10" s="13" t="str">
-        <x:v>Show progress/status placeholders; do not invent a mandatory checklist.</x:v>
+        <x:v>Model values as Admin-configurable; show no fixed commercial amount.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="65" customHeight="1">
       <x:c r="A11" s="13" t="str">
-        <x:v>CF-07</x:v>
+        <x:v>CF-08</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
-        <x:v>F07/F21 · Membership</x:v>
+        <x:v>F09/F10 · Seller bids</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
-        <x:v>What membership packages, fees, benefits, duration, and renewal rules apply?</x:v>
+        <x:v>What fields, edit rules, evaluation details, commercial terms, and RM bid-support charges apply?</x:v>
       </x:c>
       <x:c r="E11" s="13" t="str">
-        <x:v>BRD F5S.1, F8.2–F8.3</x:v>
+        <x:v>BRD F5S.3–F5S.6</x:v>
       </x:c>
       <x:c r="F11" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G11" s="13" t="str">
-        <x:v>Model values as Admin-configurable; show no fixed commercial amount.</x:v>
+        <x:v>Keep technical and commercial bids separate; do not expose competitor bids.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="65" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>CF-08</x:v>
+        <x:v>CF-09</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C12" s="13" t="str">
-        <x:v>F09/F10 · Seller bids</x:v>
+        <x:v>F12 · Buyer selection</x:v>
       </x:c>
       <x:c r="D12" s="13" t="str">
-        <x:v>What fields, edit rules, evaluation details, commercial terms, and RM bid-support charges apply?</x:v>
+        <x:v>What matching/shortlist and identity-release rules, interview process, and LOI format apply?</x:v>
       </x:c>
       <x:c r="E12" s="13" t="str">
-        <x:v>BRD F5S.3–F5S.6</x:v>
+        <x:v>BRD F5B.2–F5B.4; masking clarification</x:v>
       </x:c>
       <x:c r="F12" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G12" s="13" t="str">
-        <x:v>Keep technical and commercial bids separate; do not expose competitor bids.</x:v>
+        <x:v>Keep profiles masked until the approved release gate; exact gate remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="65" customHeight="1">
       <x:c r="A13" s="13" t="str">
-        <x:v>CF-09</x:v>
+        <x:v>CF-10</x:v>
       </x:c>
       <x:c r="B13" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C13" s="13" t="str">
-        <x:v>F12 · Buyer selection</x:v>
+        <x:v>F13/F14 · Win-and-Staff and award</x:v>
       </x:c>
       <x:c r="D13" s="13" t="str">
-        <x:v>What matching/shortlist and identity-release rules, interview process, and LOI format apply?</x:v>
+        <x:v>Which agreements must be signed by whom and when relative to LOI, award, and introduction?</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
-        <x:v>BRD F5B.2–F5B.4; masking clarification</x:v>
+        <x:v>Client feedback; BRD F5W.2–F5W.3 and F5B.4</x:v>
       </x:c>
       <x:c r="F13" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Needs clarification · sequence conflict</x:v>
       </x:c>
       <x:c r="G13" s="13" t="str">
-        <x:v>Keep profiles masked until the approved release gate; exact gate remains open.</x:v>
+        <x:v>Apply the approved gate that signatures precede award and introduction; resolve document sequence before final flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="65" customHeight="1">
       <x:c r="A14" s="13" t="str">
-        <x:v>CF-10</x:v>
+        <x:v>CF-11</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C14" s="13" t="str">
-        <x:v>F13/F14 · Win-and-Staff and award</x:v>
+        <x:v>F13 · Reservation</x:v>
       </x:c>
       <x:c r="D14" s="13" t="str">
-        <x:v>Which agreements must be signed by whom and when relative to LOI, award, and introduction?</x:v>
+        <x:v>What reservation period, consent evidence, fee, and automation phase apply?</x:v>
       </x:c>
       <x:c r="E14" s="13" t="str">
-        <x:v>Client feedback; BRD F5W.2–F5W.3 and F5B.4</x:v>
+        <x:v>BRD F5W.1–F5W.3</x:v>
       </x:c>
       <x:c r="F14" s="13" t="str">
-        <x:v>Needs clarification · sequence conflict</x:v>
+        <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G14" s="13" t="str">
-        <x:v>Apply the approved gate that signatures precede award and introduction; resolve document sequence before final flow.</x:v>
+        <x:v>Reservation is not deployment; release if firm does not win.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="65" customHeight="1">
       <x:c r="A15" s="13" t="str">
-        <x:v>CF-11</x:v>
+        <x:v>CF-12</x:v>
       </x:c>
       <x:c r="B15" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C15" s="13" t="str">
-        <x:v>F13 · Reservation</x:v>
+        <x:v>F16 · Payments &amp; invoices</x:v>
       </x:c>
       <x:c r="D15" s="13" t="str">
-        <x:v>What reservation period, consent evidence, fee, and automation phase apply?</x:v>
+        <x:v>Who invoices whom in Seller, Buyer, and OptimIQ-sourced Expert flows, and which milestones trigger payment?</x:v>
       </x:c>
       <x:c r="E15" s="13" t="str">
-        <x:v>BRD F5W.1–F5W.3</x:v>
+        <x:v>BRD financial lifecycle F6/P/G; commercial model open</x:v>
       </x:c>
       <x:c r="F15" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G15" s="13" t="str">
-        <x:v>Reservation is not deployment; release if firm does not win.</x:v>
+        <x:v>Keep Seller and Buyer money streams distinct; hide internal OptimIQ margin.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
       <x:c r="A16" s="13" t="str">
-        <x:v>CF-12</x:v>
+        <x:v>CF-13</x:v>
       </x:c>
       <x:c r="B16" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C16" s="13" t="str">
-        <x:v>F16 · Payments &amp; invoices</x:v>
+        <x:v>F17/F18 · Communications/calendar</x:v>
       </x:c>
       <x:c r="D16" s="13" t="str">
-        <x:v>Who invoices whom in Seller, Buyer, and OptimIQ-sourced Expert flows, and which milestones trigger payment?</x:v>
+        <x:v>Are integrated mailbox, chat, WhatsApp, notifications, and calendar included for firms? Which events/providers/retention apply?</x:v>
       </x:c>
       <x:c r="E16" s="13" t="str">
-        <x:v>BRD financial lifecycle F6/P/G; commercial model open</x:v>
+        <x:v>Consultant client feedback; BRD lacks firm detail</x:v>
       </x:c>
       <x:c r="F16" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G16" s="13" t="str">
-        <x:v>Keep Seller and Buyer money streams distinct; hide internal OptimIQ margin.</x:v>
+        <x:v>Treat as potential configurable integrations; no provider or SLA commitment.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>CF-13</x:v>
+        <x:v>CF-14</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>F17/F18 · Communications/calendar</x:v>
+        <x:v>F19 · Project documents</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>Are integrated mailbox, chat, WhatsApp, notifications, and calendar included for firms? Which events/providers/retention apply?</x:v>
+        <x:v>Does the proposed Phase 2 project folder and knowledge library include consulting firms, and what sharing rights apply?</x:v>
       </x:c>
       <x:c r="E17" s="13" t="str">
-        <x:v>Consultant client feedback; BRD lacks firm detail</x:v>
+        <x:v>Client feedback Phase 2; BRD firm scope not specific</x:v>
       </x:c>
       <x:c r="F17" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G17" s="13" t="str">
-        <x:v>Treat as potential configurable integrations; no provider or SLA commitment.</x:v>
+        <x:v>Show only a proposed module until access policy and rollout are confirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="65" customHeight="1">
       <x:c r="A18" s="13" t="str">
-        <x:v>CF-14</x:v>
+        <x:v>CF-15</x:v>
       </x:c>
       <x:c r="B18" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C18" s="13" t="str">
-        <x:v>F19 · Project documents</x:v>
+        <x:v>F20 · Performance</x:v>
       </x:c>
       <x:c r="D18" s="13" t="str">
-        <x:v>Does the proposed Phase 2 project folder and knowledge library include consulting firms, and what sharing rights apply?</x:v>
+        <x:v>Which firm feedback and KPIs are visible and how do they affect tier?</x:v>
       </x:c>
       <x:c r="E18" s="13" t="str">
-        <x:v>Client feedback Phase 2; BRD firm scope not specific</x:v>
+        <x:v>BRD F8.1; DR10</x:v>
       </x:c>
       <x:c r="F18" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G18" s="13" t="str">
-        <x:v>Show only a proposed module until access policy and rollout are confirmed.</x:v>
+        <x:v>Enforce DR10 separation: Seller performance is not affected by Buyer payment behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="65" customHeight="1">
       <x:c r="A19" s="13" t="str">
-        <x:v>CF-15</x:v>
+        <x:v>CF-16</x:v>
       </x:c>
       <x:c r="B19" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C19" s="13" t="str">
-        <x:v>F20 · Performance</x:v>
+        <x:v>F22/F23 · Grievance and exit</x:v>
       </x:c>
       <x:c r="D19" s="13" t="str">
-        <x:v>Which firm feedback and KPIs are visible and how do they affect tier?</x:v>
+        <x:v>What grievance/change request and exit steps, evidence, review, retention, and final settlement apply?</x:v>
       </x:c>
       <x:c r="E19" s="13" t="str">
-        <x:v>BRD F8.1; DR10</x:v>
+        <x:v>BRD F-S01–F-S04; F8.4</x:v>
       </x:c>
       <x:c r="F19" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G19" s="13" t="str">
-        <x:v>Enforce DR10 separation: Seller performance is not affected by Buyer payment behavior.</x:v>
+        <x:v>Show request/status concepts only; workflow rules remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="65" customHeight="1">
       <x:c r="A20" s="13" t="str">
-        <x:v>CF-16</x:v>
+        <x:v>CF-17</x:v>
       </x:c>
       <x:c r="B20" s="13" t="str">
         <x:v>Consulting Firm</x:v>
       </x:c>
       <x:c r="C20" s="13" t="str">
-        <x:v>F22/F23 · Grievance and exit</x:v>
+        <x:v>CTQ and qualification display</x:v>
       </x:c>
       <x:c r="D20" s="13" t="str">
-        <x:v>What grievance/change request and exit steps, evidence, review, retention, and final settlement apply?</x:v>
+        <x:v>Are proposed firm tier labels and thresholds final for member display after review, and is a numeric composite score ever displayed?</x:v>
       </x:c>
       <x:c r="E20" s="13" t="str">
-        <x:v>BRD F-S01–F-S04; F8.4</x:v>
+        <x:v>BRD addendum Table 68; client note</x:v>
       </x:c>
       <x:c r="F20" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G20" s="13" t="str">
-        <x:v>Show request/status concepts only; workflow rules remain open.</x:v>
+        <x:v>Keep scoring internals hidden in the member workspace.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="65" customHeight="1">
       <x:c r="A21" s="13" t="str">
-        <x:v>CF-17</x:v>
+        <x:v>CL-01</x:v>
       </x:c>
       <x:c r="B21" s="13" t="str">
-        <x:v>Consulting Firm</x:v>
+        <x:v>Client</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>CTQ and qualification display</x:v>
+        <x:v>C01–C04 · CTA through CTQ</x:v>
       </x:c>
       <x:c r="D21" s="13" t="str">
-        <x:v>Are proposed firm tier labels and thresholds final for member display after review, and is a numeric composite score ever displayed?</x:v>
+        <x:v>Confirm where the Client CTQ appears. The approved Client workbook places the optional questions immediately after CTA without login. The agreed shared portal flow places them after sign-in and terms. Also reconcile CTA account creation, OTP/password setup, and BRD invitation/self-start.</x:v>
       </x:c>
       <x:c r="E21" s="13" t="str">
-        <x:v>BRD addendum Table 68; client note</x:v>
+        <x:v>Client workbook Read Me / Optional Enrichment; BRD C1–C2; shared-login decision</x:v>
       </x:c>
       <x:c r="F21" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G21" s="13" t="str">
-        <x:v>Keep scoring internals hidden in the member workspace.</x:v>
+        <x:v>Review flow assumes CTA → shared sign-in → terms → optional Client CTQ. Keep the questions skippable and the existing CTA unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="65" customHeight="1">
       <x:c r="A22" s="13" t="str">
-        <x:v>CL-01</x:v>
+        <x:v>CL-02</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C22" s="13" t="str">
-        <x:v>C01–C03 · CTA, enrichment, sign-in</x:v>
+        <x:v>C04 · Client CTQ scoring</x:v>
       </x:c>
       <x:c r="D22" s="13" t="str">
-        <x:v>How does the client CTA/enquiry connect to account creation, OTP/password setup, and login? The categorisation workbook specifies soft, non-blocking email confirmation and no login before optional enrichment; prior project direction says CTA then shared portal login; BRD C1/C2 says BD qualification followed by invitation or self-start and OTP.</x:v>
+        <x:v>What score precision/rounding is applied before assigning CL1–CL4? The workbook gives score bands to three decimal places but does not define rounding for scores between the listed boundaries.</x:v>
       </x:c>
       <x:c r="E22" s="13" t="str">
-        <x:v>Client workbook Read Me / Client Web Form; BRD C1–C2; agreed shared-login journey</x:v>
+        <x:v>Client categorisation workbook: Segment Master and Scoring &amp; Follow-up Logic</x:v>
       </x:c>
       <x:c r="F22" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G22" s="13" t="str">
-        <x:v>Keep the existing CTA unchanged, show the optional step skippable, then use shared login. Do not gate enrichment or expose categorisation.</x:v>
+        <x:v>Use the workbook weights and bands as supplied; keep segment assignment internal and do not display numeric score.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="65" customHeight="1">
       <x:c r="A23" s="13" t="str">
-        <x:v>CL-02</x:v>
+        <x:v>CL-03</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>C02 · Optional categorisation</x:v>
+        <x:v>C03 · Terms &amp; declarations</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
-        <x:v>What score precision/rounding is applied before assigning CL1–CL4? The workbook gives score bands to three decimal places but does not define rounding for scores between the listed boundaries.</x:v>
+        <x:v>Which client terms/declarations are required, who may sign for the organisation, and is payment-method setup part of first-login account setup?</x:v>
       </x:c>
       <x:c r="E23" s="13" t="str">
-        <x:v>Client categorisation workbook: Segment Master and Scoring &amp; Follow-up Logic</x:v>
+        <x:v>BRD C2.4–C2.5; exact client documents not specified</x:v>
       </x:c>
       <x:c r="F23" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G23" s="13" t="str">
-        <x:v>Use the workbook weights and bands as supplied; keep segment assignment internal and do not display numeric score.</x:v>
+        <x:v>Show a shared review/acceptance pattern with placeholder document names; do not imply legal copy is final.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="65" customHeight="1">
       <x:c r="A24" s="13" t="str">
-        <x:v>CL-03</x:v>
+        <x:v>CL-05</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C24" s="13" t="str">
-        <x:v>C04 · Terms &amp; declarations</x:v>
+        <x:v>C06 · Organisation profile</x:v>
       </x:c>
       <x:c r="D24" s="13" t="str">
-        <x:v>Which client terms/declarations are required, who may sign for the organisation, and is payment-method setup part of first-login account setup?</x:v>
+        <x:v>Which organisation and contact fields can the client edit after registration, what evidence is needed, and which changes require OptimIQ approval?</x:v>
       </x:c>
       <x:c r="E24" s="13" t="str">
-        <x:v>BRD C2.4–C2.5; exact client documents not specified</x:v>
+        <x:v>BRD C3; no client profile field/update rules supplied</x:v>
       </x:c>
       <x:c r="F24" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G24" s="13" t="str">
-        <x:v>Show a shared review/acceptance pattern with placeholder document names; do not imply legal copy is final.</x:v>
+        <x:v>Show profile review and an edit entry point only; no unsupported approval workflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="65" customHeight="1">
       <x:c r="A25" s="13" t="str">
-        <x:v>CL-04</x:v>
+        <x:v>CL-06</x:v>
       </x:c>
       <x:c r="B25" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C25" s="13" t="str">
-        <x:v>C05 / all client screens · phase labels</x:v>
+        <x:v>C07 · Requirement creation &amp; scoping</x:v>
       </x:c>
       <x:c r="D25" s="13" t="str">
-        <x:v>Which client lifecycle stages belong to each delivery phase? The agreed wireframe convention ends Phase 1 after categorisation/CTQ; BRD Table 60 labels the client lifecycle steps Phase 1.</x:v>
+        <x:v>What requirement fields, evidence, draft/edit/withdraw rules, fee visibility, and Solution Coordinator assignment details should appear?</x:v>
       </x:c>
       <x:c r="E25" s="13" t="str">
-        <x:v>BRD Table 60 versus agreed Theme 1 phase convention</x:v>
+        <x:v>BRD C4.1–C4.5; forms F-C04/F-C05; fields not included in source workbook</x:v>
       </x:c>
       <x:c r="F25" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G25" s="13" t="str">
-        <x:v>Show Phase 1 through account/categorisation and Phase 2 from requirements onward, marked as a wireframe assumption.</x:v>
+        <x:v>Use the BRD sequence: submit, scope with coordinator, confirm route, then release after applicable fee gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="65" customHeight="1">
       <x:c r="A26" s="13" t="str">
-        <x:v>CL-05</x:v>
+        <x:v>CL-07</x:v>
       </x:c>
       <x:c r="B26" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C26" s="13" t="str">
-        <x:v>C06 · Organisation profile</x:v>
+        <x:v>C08–C09 · Track A shortlist / profile</x:v>
       </x:c>
       <x:c r="D26" s="13" t="str">
-        <x:v>Which organisation and contact fields can the client edit after registration, what evidence is needed, and which changes require OptimIQ approval?</x:v>
+        <x:v>Which attributes and match rationale can a client see in the normal 2–3 masked profiles, and what comparison or selection actions are allowed before identity release?</x:v>
       </x:c>
       <x:c r="E26" s="13" t="str">
-        <x:v>BRD C3; no client profile field/update rules supplied</x:v>
+        <x:v>BRD C5 / Track A; approved masking discussion</x:v>
       </x:c>
       <x:c r="F26" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G26" s="13" t="str">
-        <x:v>Show profile review and an edit entry point only; no unsupported approval workflow.</x:v>
+        <x:v>Show masked profiles and rationale; keep direct identity/contact hidden until approved release gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="65" customHeight="1">
       <x:c r="A27" s="13" t="str">
-        <x:v>CL-06</x:v>
+        <x:v>CL-08</x:v>
       </x:c>
       <x:c r="B27" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C27" s="13" t="str">
-        <x:v>C07 · Requirement creation &amp; scoping</x:v>
+        <x:v>C10 · Request more profiles</x:v>
       </x:c>
       <x:c r="D27" s="13" t="str">
-        <x:v>What requirement fields, evidence, draft/edit/withdraw rules, fee visibility, and Solution Coordinator assignment details should appear?</x:v>
+        <x:v>What reason, approval role, and permitted number of additional profiles apply when the normal 2–3 shortlist is not suitable?</x:v>
       </x:c>
       <x:c r="E27" s="13" t="str">
-        <x:v>BRD C4.1–C4.5; forms F-C04/F-C05; fields not included in source workbook</x:v>
+        <x:v>BRD shortlist exception; exact procedure not specified</x:v>
       </x:c>
       <x:c r="F27" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G27" s="13" t="str">
-        <x:v>Use the BRD sequence: submit, scope with coordinator, confirm route, then release after applicable fee gate.</x:v>
+        <x:v>Show request-to-OptimIQ as an exception that is logged; do not auto-generate more profiles.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="65" customHeight="1">
       <x:c r="A28" s="13" t="str">
-        <x:v>CL-07</x:v>
+        <x:v>CL-09</x:v>
       </x:c>
       <x:c r="B28" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C28" s="13" t="str">
-        <x:v>C08–C09 · Track A shortlist / profile</x:v>
+        <x:v>C11 · Track B evaluation</x:v>
       </x:c>
       <x:c r="D28" s="13" t="str">
-        <x:v>Which attributes and match rationale can a client see in the normal 2–3 masked profiles, and what comparison or selection actions are allowed before identity release?</x:v>
+        <x:v>What Track B routing thresholds, evaluation methods, weights, technical/financial visibility, and client decision rights apply?</x:v>
       </x:c>
       <x:c r="E28" s="13" t="str">
-        <x:v>BRD C5 / Track A; approved masking discussion</x:v>
+        <x:v>BRD RB1–RB4 / Table 27; 70:30 is an unapproved example</x:v>
       </x:c>
       <x:c r="F28" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G28" s="13" t="str">
-        <x:v>Show masked profiles and rationale; keep direct identity/contact hidden until approved release gate.</x:v>
+        <x:v>Show TER then FER as a managed sequence; do not publish scores/weights until confirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="65" customHeight="1">
       <x:c r="A29" s="13" t="str">
-        <x:v>CL-08</x:v>
+        <x:v>CL-10</x:v>
       </x:c>
       <x:c r="B29" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C29" s="13" t="str">
-        <x:v>C10 · Request more profiles</x:v>
+        <x:v>C12–C13 · Agreements, award, introduction</x:v>
       </x:c>
       <x:c r="D29" s="13" t="str">
-        <x:v>What reason, approval role, and permitted number of additional profiles apply when the normal 2–3 shortlist is not suitable?</x:v>
+        <x:v>Which agreements are signed by which parties, and how do signatures relate to LOI, award, identity disclosure, introduction, and first payment?</x:v>
       </x:c>
       <x:c r="E29" s="13" t="str">
-        <x:v>BRD shortlist exception; exact procedure not specified</x:v>
+        <x:v>Client feedback requires signatures before award/introduction; BRD C5–C6 / RA3 / G1 order needs reconciliation</x:v>
       </x:c>
       <x:c r="F29" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G29" s="13" t="str">
-        <x:v>Show request-to-OptimIQ as an exception that is logged; do not auto-generate more profiles.</x:v>
+        <x:v>Enforce the agreed signature-before-award-and-introduction gate; hold exact document sequence and signers open.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="65" customHeight="1">
       <x:c r="A30" s="13" t="str">
-        <x:v>CL-09</x:v>
+        <x:v>CL-11</x:v>
       </x:c>
       <x:c r="B30" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C30" s="13" t="str">
-        <x:v>C11 · Track B evaluation</x:v>
+        <x:v>C13 · Meetings &amp; introduction</x:v>
       </x:c>
       <x:c r="D30" s="13" t="str">
-        <x:v>What Track B routing thresholds, evaluation methods, weights, technical/financial visibility, and client decision rights apply?</x:v>
+        <x:v>Which meeting provider, recording/consent settings, participant access, and identity-disclosure point apply to each meeting type?</x:v>
       </x:c>
       <x:c r="E30" s="13" t="str">
-        <x:v>BRD RB1–RB4 / Table 27; 70:30 is an unapproved example</x:v>
+        <x:v>BRD controlled interaction; prior meeting configuration decisions; client process detail absent</x:v>
       </x:c>
       <x:c r="F30" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G30" s="13" t="str">
-        <x:v>Show TER then FER as a managed sequence; do not publish scores/weights until confirmed.</x:v>
+        <x:v>Use a provider-flexible meeting concept and meeting-specific recording as a configurable option.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="65" customHeight="1">
       <x:c r="A31" s="13" t="str">
-        <x:v>CL-10</x:v>
+        <x:v>CL-12</x:v>
       </x:c>
       <x:c r="B31" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C31" s="13" t="str">
-        <x:v>C12–C13 · Agreements, award, introduction</x:v>
+        <x:v>C14 · Engagements &amp; milestones</x:v>
       </x:c>
       <x:c r="D31" s="13" t="str">
-        <x:v>Which agreements are signed by which parties, and how do signatures relate to LOI, award, identity disclosure, introduction, and first payment?</x:v>
+        <x:v>What milestone templates, buyer review windows, rework rules, change approvals, and dispute steps should the client see?</x:v>
       </x:c>
       <x:c r="E31" s="13" t="str">
-        <x:v>Client feedback requires signatures before award/introduction; BRD C5–C6 / RA3 / G1 order needs reconciliation</x:v>
+        <x:v>BRD G1–G5; exact client-facing presentation not final</x:v>
       </x:c>
       <x:c r="F31" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G31" s="13" t="str">
-        <x:v>Enforce the agreed signature-before-award-and-introduction gate; hold exact document sequence and signers open.</x:v>
+        <x:v>Show project-scoped statuses aligned to BRD; use no fixed milestone catalogue.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="65" customHeight="1">
       <x:c r="A32" s="13" t="str">
-        <x:v>CL-11</x:v>
+        <x:v>CL-13</x:v>
       </x:c>
       <x:c r="B32" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C32" s="13" t="str">
-        <x:v>C13 · Meetings &amp; introduction</x:v>
+        <x:v>C15 · Invoices &amp; payments</x:v>
       </x:c>
       <x:c r="D32" s="13" t="str">
-        <x:v>Which meeting provider, recording/consent settings, participant access, and identity-disclosure point apply to each meeting type?</x:v>
+        <x:v>Which fees, payment methods, payment dates, cancellation/refund triggers, and client-visible commercial details apply?</x:v>
       </x:c>
       <x:c r="E32" s="13" t="str">
-        <x:v>BRD controlled interaction; prior meeting configuration decisions; client process detail absent</x:v>
+        <x:v>BRD P/G and Table 30; commercial values remain business decisions</x:v>
       </x:c>
       <x:c r="F32" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G32" s="13" t="str">
-        <x:v>Use a provider-flexible meeting concept and meeting-specific recording as a configurable option.</x:v>
+        <x:v>Use configurable fee values; show only client-facing amounts, never internal OptimIQ margin/commission.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="65" customHeight="1">
       <x:c r="A33" s="13" t="str">
-        <x:v>CL-12</x:v>
+        <x:v>CL-14</x:v>
       </x:c>
       <x:c r="B33" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C33" s="13" t="str">
-        <x:v>C14 · Engagements &amp; milestones</x:v>
+        <x:v>C16 · Feedback &amp; re-engagement</x:v>
       </x:c>
       <x:c r="D33" s="13" t="str">
-        <x:v>What milestone templates, buyer review windows, rework rules, change approvals, and dispute steps should the client see?</x:v>
+        <x:v>Does client feedback affect seller composite/performance scores, or is it stored and presented as a separate project signal?</x:v>
       </x:c>
       <x:c r="E33" s="13" t="str">
-        <x:v>BRD G1–G5; exact client-facing presentation not final</x:v>
+        <x:v>Client feedback per engagement; BRD C8.1 / performance scoring</x:v>
       </x:c>
       <x:c r="F33" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G33" s="13" t="str">
-        <x:v>Show project-scoped statuses aligned to BRD; use no fixed milestone catalogue.</x:v>
+        <x:v>Capture feedback separately per engagement; do not display score impact until approved.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="65" customHeight="1">
       <x:c r="A34" s="13" t="str">
-        <x:v>CL-13</x:v>
+        <x:v>CL-15</x:v>
       </x:c>
       <x:c r="B34" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C34" s="13" t="str">
-        <x:v>C15 · Invoices &amp; payments</x:v>
+        <x:v>C17 · Communications</x:v>
       </x:c>
       <x:c r="D34" s="13" t="str">
-        <x:v>Which fees, payment methods, payment dates, cancellation/refund triggers, and client-visible commercial details apply?</x:v>
+        <x:v>Are in-portal email, chat, WhatsApp, and an @optimiqconsultus.com mailbox in scope for clients? Which message types, retention, and providers apply?</x:v>
       </x:c>
       <x:c r="E34" s="13" t="str">
-        <x:v>BRD P/G and Table 30; commercial values remain business decisions</x:v>
+        <x:v>Client feedback on communications; BRD N1; client-specific scope open</x:v>
       </x:c>
       <x:c r="F34" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G34" s="13" t="str">
-        <x:v>Use configurable fee values; show only client-facing amounts, never internal OptimIQ margin/commission.</x:v>
+        <x:v>Show a notification/message centre concept only; integrations and mailbox are not committed.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="65" customHeight="1">
       <x:c r="A35" s="13" t="str">
-        <x:v>CL-14</x:v>
+        <x:v>CL-16</x:v>
       </x:c>
       <x:c r="B35" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C35" s="13" t="str">
-        <x:v>C16 · Feedback &amp; re-engagement</x:v>
+        <x:v>C18 · Project calendar</x:v>
       </x:c>
       <x:c r="D35" s="13" t="str">
-        <x:v>Does client feedback affect seller composite/performance scores, or is it stored and presented as a separate project signal?</x:v>
+        <x:v>Which client event types and calendar integrations are required, and are recording/consent settings global or meeting-specific?</x:v>
       </x:c>
       <x:c r="E35" s="13" t="str">
-        <x:v>Client feedback per engagement; BRD C8.1 / performance scoring</x:v>
+        <x:v>Client feedback on integrated calendar and meeting configuration</x:v>
       </x:c>
       <x:c r="F35" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G35" s="13" t="str">
-        <x:v>Capture feedback separately per engagement; do not display score impact until approved.</x:v>
+        <x:v>Present a project calendar concept; provider and sync rules remain configurable/open.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="65" customHeight="1">
       <x:c r="A36" s="13" t="str">
-        <x:v>CL-15</x:v>
+        <x:v>CL-17</x:v>
       </x:c>
       <x:c r="B36" s="13" t="str">
         <x:v>Client</x:v>
       </x:c>
       <x:c r="C36" s="13" t="str">
-        <x:v>C17 · Communications</x:v>
+        <x:v>C19 · Project documents</x:v>
       </x:c>
       <x:c r="D36" s="13" t="str">
-        <x:v>Are in-portal email, chat, WhatsApp, and an @optimiqconsultus.com mailbox in scope for clients? Which message types, retention, and providers apply?</x:v>
+        <x:v>Which client, consultant, and OptimIQ roles can access project folders and comments, how long are files retained, and can approved summaries become public success stories?</x:v>
       </x:c>
       <x:c r="E36" s="13" t="str">
-        <x:v>Client feedback on communications; BRD N1; client-specific scope open</x:v>
+        <x:v>Client feedback proposed Phase 2 folders/library; BRD access and publication rules incomplete</x:v>
       </x:c>
       <x:c r="F36" s="13" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="G36" s="13" t="str">
-        <x:v>Show a notification/message centre concept only; integrations and mailbox are not committed.</x:v>
+        <x:v>Treat project folders as a Phase 2 concept; keep cross-client reuse/testimonials disabled until explicit consent and policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="65" customHeight="1">
-      <x:c r="A37" s="13" t="str">
-        <x:v>CL-16</x:v>
-      </x:c>
-      <x:c r="B37" s="13" t="str">
+      <x:c r="A37" s="14" t="str">
+        <x:v>CL-18</x:v>
+      </x:c>
+      <x:c r="B37" s="14" t="str">
         <x:v>Client</x:v>
       </x:c>
-      <x:c r="C37" s="13" t="str">
-        <x:v>C18 · Project calendar</x:v>
-      </x:c>
-      <x:c r="D37" s="13" t="str">
-        <x:v>Which client event types and calendar integrations are required, and are recording/consent settings global or meeting-specific?</x:v>
-      </x:c>
-      <x:c r="E37" s="13" t="str">
-        <x:v>Client feedback on integrated calendar and meeting configuration</x:v>
-      </x:c>
-      <x:c r="F37" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="G37" s="13" t="str">
-        <x:v>Present a project calendar concept; provider and sync rules remain configurable/open.</x:v>
+      <x:c r="C37" s="14" t="str">
+        <x:v>C20 · Support &amp; account exit</x:v>
+      </x:c>
+      <x:c r="D37" s="14" t="str">
+        <x:v>What complaint routes, escalation targets, account-exit steps, open-project handling, and retention rules apply to client accounts?</x:v>
+      </x:c>
+      <x:c r="E37" s="14" t="str">
+        <x:v>BRD Q/X; client-specific workflow details not provided</x:v>
+      </x:c>
+      <x:c r="F37" s="14" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G37" s="14" t="str">
+        <x:v>Show support and request status only; do not assume account closure is immediate.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="65" customHeight="1">
-      <x:c r="A38" s="13" t="str">
-        <x:v>CL-17</x:v>
-      </x:c>
-      <x:c r="B38" s="13" t="str">
-        <x:v>Client</x:v>
-      </x:c>
-      <x:c r="C38" s="13" t="str">
-        <x:v>C19 · Project documents</x:v>
-      </x:c>
-      <x:c r="D38" s="13" t="str">
-        <x:v>Which client, consultant, and OptimIQ roles can access project folders and comments, how long are files retained, and can approved summaries become public success stories?</x:v>
-      </x:c>
-      <x:c r="E38" s="13" t="str">
-        <x:v>Client feedback proposed Phase 2 folders/library; BRD access and publication rules incomplete</x:v>
-      </x:c>
-      <x:c r="F38" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="G38" s="13" t="str">
-        <x:v>Treat project folders as a Phase 2 concept; keep cross-client reuse/testimonials disabled until explicit consent and policy.</x:v>
-      </x:c>
+      <x:c r="A38"/>
+      <x:c r="B38"/>
+      <x:c r="C38"/>
+      <x:c r="D38"/>
+      <x:c r="E38"/>
+      <x:c r="F38"/>
+      <x:c r="G38"/>
     </x:row>
     <x:row r="39" ht="65" customHeight="1">
-      <x:c r="A39" s="14" t="str">
-        <x:v>CL-18</x:v>
-      </x:c>
-      <x:c r="B39" s="14" t="str">
-        <x:v>Client</x:v>
-      </x:c>
-      <x:c r="C39" s="14" t="str">
-        <x:v>C20 · Support &amp; account exit</x:v>
-      </x:c>
-      <x:c r="D39" s="14" t="str">
-        <x:v>What complaint routes, escalation targets, account-exit steps, open-project handling, and retention rules apply to client accounts?</x:v>
-      </x:c>
-      <x:c r="E39" s="14" t="str">
-        <x:v>BRD Q/X; client-specific workflow details not provided</x:v>
-      </x:c>
-      <x:c r="F39" s="14" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-      <x:c r="G39" s="14" t="str">
-        <x:v>Show support and request status only; do not assume account closure is immediate.</x:v>
-      </x:c>
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Add enterprise phase plan and mind map screen placeholders
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R68135888d47f4999"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="R1bf729d1b2734601"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="R7bc9fd82a2e246bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R8adc76df65c749bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="Rd9e2ad6211074b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="R044403abbce64888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="Rbc8140e999ec4c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R9922f3a1649a46eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8d4700642f6a4b03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="R9d04dd42821b4d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="Re59cfd16140141c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R0ce3fc12a1194ebb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="Rb34a105410914d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="R32d94a27eb964eb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R11d87014811746f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R8e1174f52edb4977"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="9" r:id="R2933d994e5f84439"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -72,7 +73,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +98,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF06352E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F4ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF27836E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -246,7 +262,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="93">
+  <x:cellXfs count="100">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -406,6 +422,15 @@
     <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -4066,23 +4091,143 @@
         <x:v>Show support and request status only; do not assume account closure is immediate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="65" customHeight="1">
-      <x:c r="A38"/>
-      <x:c r="B38"/>
-      <x:c r="C38"/>
-      <x:c r="D38"/>
-      <x:c r="E38"/>
-      <x:c r="F38"/>
-      <x:c r="G38"/>
-    </x:row>
-    <x:row r="39" ht="65" customHeight="1">
-      <x:c r="A39"/>
-      <x:c r="B39"/>
-      <x:c r="C39"/>
-      <x:c r="D39"/>
-      <x:c r="E39"/>
-      <x:c r="F39"/>
-      <x:c r="G39"/>
+    <x:row r="38" ht="70" customHeight="1">
+      <x:c r="A38" s="12" t="str">
+        <x:v>MM-Q1</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>Client / Staff</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str">
+        <x:v>Client categorisation and routing</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="str">
+        <x:v>How do Type A/B/C and Strategic/Priority/Standard map to internal CL1–CL4 and Track A/B?</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="str">
+        <x:v>Client mind map vs approved client categorisation workbook</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G38" s="12" t="str">
+        <x:v>Keep classifications separate and hidden from the client.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="70" customHeight="1">
+      <x:c r="A39" s="13" t="str">
+        <x:v>MM-Q2</x:v>
+      </x:c>
+      <x:c r="B39" s="13" t="str">
+        <x:v>Consulting Firm</x:v>
+      </x:c>
+      <x:c r="C39" s="13" t="str">
+        <x:v>Firm assessment progress</x:v>
+      </x:c>
+      <x:c r="D39" s="13" t="str">
+        <x:v>What does the mind map 0–3 / 4–7 / &gt;7 Consultant CTQ branch measure and what action follows?</x:v>
+      </x:c>
+      <x:c r="E39" s="13" t="str">
+        <x:v>Client mind map; one-firm-login rule</x:v>
+      </x:c>
+      <x:c r="F39" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G39" s="13" t="str">
+        <x:v>Do not create employee logins or derive eligibility from the bands.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="70" customHeight="1">
+      <x:c r="A40" s="13" t="str">
+        <x:v>MM-Q3</x:v>
+      </x:c>
+      <x:c r="B40" s="13" t="str">
+        <x:v>Consultant / Firm</x:v>
+      </x:c>
+      <x:c r="C40" s="13" t="str">
+        <x:v>Composite assessment</x:v>
+      </x:c>
+      <x:c r="D40" s="13" t="str">
+        <x:v>Which components, weights, evidence, providers and committee-interview rule define each composite?</x:v>
+      </x:c>
+      <x:c r="E40" s="13" t="str">
+        <x:v>Client mind map vs existing consultant component model</x:v>
+      </x:c>
+      <x:c r="F40" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G40" s="13" t="str">
+        <x:v>Show progress only and keep weights and scores private.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="70" customHeight="1">
+      <x:c r="A41" s="13" t="str">
+        <x:v>MM-Q4</x:v>
+      </x:c>
+      <x:c r="B41" s="13" t="str">
+        <x:v>Client / Firm / Staff</x:v>
+      </x:c>
+      <x:c r="C41" s="13" t="str">
+        <x:v>Tender and e-evaluation</x:v>
+      </x:c>
+      <x:c r="D41" s="13" t="str">
+        <x:v>What TOR fields, technical/financial parameters, QCBS method, disclosure and decision rights apply?</x:v>
+      </x:c>
+      <x:c r="E41" s="13" t="str">
+        <x:v>Client mind map tender branch; BRD Track B</x:v>
+      </x:c>
+      <x:c r="F41" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G41" s="13" t="str">
+        <x:v>Present a managed tender sequence without an invented formula.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="70" customHeight="1">
+      <x:c r="A42" s="13" t="str">
+        <x:v>MM-Q5</x:v>
+      </x:c>
+      <x:c r="B42" s="13" t="str">
+        <x:v>Consultant / Firm</x:v>
+      </x:c>
+      <x:c r="C42" s="13" t="str">
+        <x:v>Project performance and feedback</x:v>
+      </x:c>
+      <x:c r="D42" s="13" t="str">
+        <x:v>Does project-specific client and relationship-team feedback alter the composite or remain a separate signal?</x:v>
+      </x:c>
+      <x:c r="E42" s="13" t="str">
+        <x:v>Client mind map and prior client feedback</x:v>
+      </x:c>
+      <x:c r="F42" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G42" s="13" t="str">
+        <x:v>Store feedback per engagement and display it separately for now.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="70" customHeight="1">
+      <x:c r="A43" s="14" t="str">
+        <x:v>MM-Q6</x:v>
+      </x:c>
+      <x:c r="B43" s="14" t="str">
+        <x:v>All audiences / Staff</x:v>
+      </x:c>
+      <x:c r="C43" s="14" t="str">
+        <x:v>Communications and integrations</x:v>
+      </x:c>
+      <x:c r="D43" s="14" t="str">
+        <x:v>Which chatbot, WhatsApp, email, AI calling, Calendly and meeting-provider features are required in which release, with what consent and provider?</x:v>
+      </x:c>
+      <x:c r="E43" s="14" t="str">
+        <x:v>Client mind map integration branches</x:v>
+      </x:c>
+      <x:c r="F43" s="14" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="G43" s="14" t="str">
+        <x:v>Treat them as replaceable Phase 2 candidates until scope is confirmed.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4357,4 +4502,305 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="35" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="65" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="94" t="str">
+        <x:v>OptimIQ Consultus · Enterprise Phase Plan</x:v>
+      </x:c>
+      <x:c r="B1" s="94"/>
+      <x:c r="C1" s="94"/>
+      <x:c r="D1" s="94"/>
+      <x:c r="E1" s="94"/>
+      <x:c r="F1" s="94"/>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="97" t="str">
+        <x:v>Phase 1 boundary is approved. Phase 2 increments are a proposed sequence for client review, not committed dates. Mind map phases describe process stages, not these release phases.</x:v>
+      </x:c>
+      <x:c r="B2" s="97"/>
+      <x:c r="C2" s="97"/>
+      <x:c r="D2" s="97"/>
+      <x:c r="E2" s="97"/>
+      <x:c r="F2" s="97"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="99" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="B4" s="99" t="str">
+        <x:v>Screen family</x:v>
+      </x:c>
+      <x:c r="C4" s="99" t="str">
+        <x:v>Audience</x:v>
+      </x:c>
+      <x:c r="D4" s="99" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="E4" s="99" t="str">
+        <x:v>Clarification needed</x:v>
+      </x:c>
+      <x:c r="F4" s="99" t="str">
+        <x:v>Review status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="58" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Phase 1</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Shared sign-in + identity</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>All audiences</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>One account route to the correct audience journey</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Confirm client CTQ placement after CTA vs post-login</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Approved release boundary; screen review in progress</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="58" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>Phase 1</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="str">
+        <x:v>Consultant terms + CTQ + role fit</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="str">
+        <x:v>Consultant</x:v>
+      </x:c>
+      <x:c r="D6" s="13" t="str">
+        <x:v>Eight CTQ sections, private scoring, then role choice</x:v>
+      </x:c>
+      <x:c r="E6" s="13" t="str">
+        <x:v>Final legal copy and exact scoring/role rules as tracked</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="str">
+        <x:v>Screen review in progress</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="58" customHeight="1">
+      <x:c r="A7" s="13" t="str">
+        <x:v>Phase 1</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="str">
+        <x:v>Firm terms + CTQ</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="str">
+        <x:v>Consulting Firm</x:v>
+      </x:c>
+      <x:c r="D7" s="13" t="str">
+        <x:v>Six CTQ sections using the same shell</x:v>
+      </x:c>
+      <x:c r="E7" s="13" t="str">
+        <x:v>Band inclusivity and member-facing tier wording</x:v>
+      </x:c>
+      <x:c r="F7" s="13" t="str">
+        <x:v>Screen review in progress</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="13" t="str">
+        <x:v>Phase 1</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="str">
+        <x:v>Client terms + optional CTQ</x:v>
+      </x:c>
+      <x:c r="C8" s="13" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="D8" s="13" t="str">
+        <x:v>Optional three-question CTQ; private categorisation</x:v>
+      </x:c>
+      <x:c r="E8" s="13" t="str">
+        <x:v>Placement and legal signer/documents</x:v>
+      </x:c>
+      <x:c r="F8" s="13" t="str">
+        <x:v>Screen review in progress</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="13" t="str">
+        <x:v>Phase 2A</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="str">
+        <x:v>Composite assessment + qualification</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="str">
+        <x:v>Consultant / Firm</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="str">
+        <x:v>Track evidence, third-party assessments and qualification</x:v>
+      </x:c>
+      <x:c r="E9" s="13" t="str">
+        <x:v>Weights, modalities, committee role, firm 0–3 / 4–7 / &gt;7 meaning</x:v>
+      </x:c>
+      <x:c r="F9" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="13" t="str">
+        <x:v>Phase 2A</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="str">
+        <x:v>Client categorisation operations</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="str">
+        <x:v>Staff Admin</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="str">
+        <x:v>Route accounts internally without showing labels to clients</x:v>
+      </x:c>
+      <x:c r="E10" s="13" t="str">
+        <x:v>Type A/B/C and account-label mapping to CL1–CL4 / Track A/B</x:v>
+      </x:c>
+      <x:c r="F10" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="13" t="str">
+        <x:v>Phase 2B</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>Requirements, opportunities and matching</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>Client / Consultant / Firm</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="str">
+        <x:v>Client demand, masked profiles, Firm Seller/Buyer/Win-and-Staff</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="str">
+        <x:v>Search access, matching, masking, shortlist and reservation rules</x:v>
+      </x:c>
+      <x:c r="F11" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="13" t="str">
+        <x:v>Phase 2C</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>Tender and e-evaluation</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>Client / Firm / Staff</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>TOR, bids, technical and financial review, QCBS decision</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>TOR fields, weights, formula, evaluator and decision rights</x:v>
+      </x:c>
+      <x:c r="F12" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
+      <x:c r="A13" s="13" t="str">
+        <x:v>Phase 2C</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>Agreements, award and introduction</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>All audiences</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>Signed agreement gate before award and introduction</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>Document types, signers, LOI order, payment and identity release</x:v>
+      </x:c>
+      <x:c r="F13" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
+      <x:c r="A14" s="13" t="str">
+        <x:v>Phase 2D</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>Engagement and performance</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>All audiences</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>Concurrent assignments, milestones and project-specific feedback</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>Feedback impact on composite versus separate performance signal</x:v>
+      </x:c>
+      <x:c r="F14" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="13" t="str">
+        <x:v>Phase 2D</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>Finance, communication and knowledge</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>All audiences / Staff</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>Billing, notifications, calendar, files and controlled reuse</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>Fees, providers, consent, rights, retention and case-study approval</x:v>
+      </x:c>
+      <x:c r="F15" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>Phase 2D</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>Staff team work queues</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>Staff Admin</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Role-based operations and Master Admin final approval</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>Team queue items, authority and record visibility</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show Phase 1 CTQ administration dependency
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8d4700642f6a4b03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="R9d04dd42821b4d32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="Re59cfd16140141c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R0ce3fc12a1194ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="Rb34a105410914d5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="R32d94a27eb964eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R11d87014811746f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R8e1174f52edb4977"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="9" r:id="R2933d994e5f84439"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra5bc95f2ca5d4d03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="Ra1545dc3659e4b98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="R2abca8c2fa0744f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R1fa49e33182441f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="R0a23948743144d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="Rf64f82d086404297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R0ee9d5779f584264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R2b3311059ea34a6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="9" r:id="Re49ddab2e5264cd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,7 +73,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="30">
+  <x:fills count="33">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +98,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF06352E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F4ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF27836E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -262,7 +277,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="100">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -431,6 +446,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2915,7 +2939,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="53" t="str">
-        <x:v>OptimIQ staff and admin screens preserved.</x:v>
+        <x:v>Phase 1 includes staff provisioning and CTQ publication controls. Full relationship, tender, finance and platform operations are Phase 2.</x:v>
       </x:c>
       <x:c r="B2" s="53"/>
       <x:c r="C2" s="53"/>
@@ -3015,7 +3039,7 @@
         <x:v>Admin, Super Admin, Master Admin</x:v>
       </x:c>
       <x:c r="E7" s="13" t="str">
-        <x:v>Assign one or more approved roles to staff; one role can be assigned to multiple staff members.</x:v>
+        <x:v>Phase 1. Provision staff access and assign one or more approved roles.</x:v>
       </x:c>
       <x:c r="F7" s="13" t="str">
         <x:v>Client will define the fixed permission/separation matrix; role assignments must obey it.</x:v>
@@ -3039,7 +3063,7 @@
         <x:v>Master Admin approver; lower-level submitters</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Review proposed decisions/configuration changes with clear before/after details, impact, rationale, and audit trail.</x:v>
+        <x:v>Phase 1 CTQ publication control; extended to all configuration changes in Phase 2. Show before/after values, impact, rationale and audit trail for Master Admin approval.</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str">
         <x:v>Master Admin final approval is confirmed; detailed layout awaits client screen approval.</x:v>
@@ -3063,7 +3087,7 @@
         <x:v>Authorised configuration roles</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>Manage approved Expert CTQ fields, role mappings, score weights, bands, and gate settings through versioned proposals.</x:v>
+        <x:v>Phase 1 Consultant CTQ questions, role weights, private scoring and fit rules; composite assessment settings follow in Phase 2.</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
         <x:v>Expert model is approved; exact configuration page controls and approval presentation need visual review.</x:v>
@@ -3087,7 +3111,7 @@
         <x:v>Authorised configuration roles</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>Manage firm CTQ questions, evidence rules, weights, scales, and tiers.</x:v>
+        <x:v>Phase 1 Firm CTQ questions, weights, bands and versioned publication. Wider firm assessment settings follow in Phase 2.</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
         <x:v>Final Firm CTQ business rules remain open.</x:v>
@@ -3264,6 +3288,54 @@
         <x:v>Needs clarification</x:v>
       </x:c>
       <x:c r="H17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>A14</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>Staff/Admin</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>Client CTQ settings</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>Authorised configuration roles</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="str">
+        <x:v>Phase 1. Maintain optional Client CTQ questions, private categorisation rules and versioned publication.</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="str">
+        <x:v>Client CTQ location and score rounding remain open.</x:v>
+      </x:c>
+      <x:c r="G18" s="12" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+      <x:c r="H18" s="12" t="str"/>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>A15</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>Staff/Admin</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>CTQ priority colour settings</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Authorised configuration roles</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="str">
+        <x:v>Phase 1. Configure and preview accessible Must Have, Good to Have and Optional indicators across all three CTQs.</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>Colour changes affect presentation only; client screen review pending.</x:v>
+      </x:c>
+      <x:c r="G19" s="14" t="str">
+        <x:v>Needs detailed screen review</x:v>
+      </x:c>
+      <x:c r="H19" s="14" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4517,42 +4589,42 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="94" t="str">
+      <x:c r="A1" s="101" t="str">
         <x:v>OptimIQ Consultus · Enterprise Phase Plan</x:v>
       </x:c>
-      <x:c r="B1" s="94"/>
-      <x:c r="C1" s="94"/>
-      <x:c r="D1" s="94"/>
-      <x:c r="E1" s="94"/>
-      <x:c r="F1" s="94"/>
+      <x:c r="B1" s="101"/>
+      <x:c r="C1" s="101"/>
+      <x:c r="D1" s="101"/>
+      <x:c r="E1" s="101"/>
+      <x:c r="F1" s="101"/>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="97" t="str">
+      <x:c r="A2" s="104" t="str">
         <x:v>Phase 1 boundary is approved. Phase 2 increments are a proposed sequence for client review, not committed dates. Mind map phases describe process stages, not these release phases.</x:v>
       </x:c>
-      <x:c r="B2" s="97"/>
-      <x:c r="C2" s="97"/>
-      <x:c r="D2" s="97"/>
-      <x:c r="E2" s="97"/>
-      <x:c r="F2" s="97"/>
+      <x:c r="B2" s="104"/>
+      <x:c r="C2" s="104"/>
+      <x:c r="D2" s="104"/>
+      <x:c r="E2" s="104"/>
+      <x:c r="F2" s="104"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="99" t="str">
+      <x:c r="A4" s="106" t="str">
         <x:v>Release</x:v>
       </x:c>
-      <x:c r="B4" s="99" t="str">
+      <x:c r="B4" s="106" t="str">
         <x:v>Screen family</x:v>
       </x:c>
-      <x:c r="C4" s="99" t="str">
+      <x:c r="C4" s="106" t="str">
         <x:v>Audience</x:v>
       </x:c>
-      <x:c r="D4" s="99" t="str">
+      <x:c r="D4" s="106" t="str">
         <x:v>Purpose</x:v>
       </x:c>
-      <x:c r="E4" s="99" t="str">
+      <x:c r="E4" s="106" t="str">
         <x:v>Clarification needed</x:v>
       </x:c>
-      <x:c r="F4" s="99" t="str">
+      <x:c r="F4" s="106" t="str">
         <x:v>Review status</x:v>
       </x:c>
     </x:row>
@@ -4638,22 +4710,22 @@
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="13" t="str">
-        <x:v>Phase 2A</x:v>
+        <x:v>Phase 1</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>Composite assessment + qualification</x:v>
+        <x:v>CTQ publication controls</x:v>
       </x:c>
       <x:c r="C9" s="13" t="str">
-        <x:v>Consultant / Firm</x:v>
+        <x:v>Staff Admin</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>Track evidence, third-party assessments and qualification</x:v>
+        <x:v>Provision staff and publish versioned CTQ/scoring changes with Master Admin approval</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
-        <x:v>Weights, modalities, committee role, firm 0–3 / 4–7 / &gt;7 meaning</x:v>
+        <x:v>Detailed configuration and approval screen review</x:v>
       </x:c>
       <x:c r="F9" s="13" t="str">
-        <x:v>Needs clarification</x:v>
+        <x:v>Needs detailed screen review</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
@@ -4661,16 +4733,16 @@
         <x:v>Phase 2A</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>Client categorisation operations</x:v>
+        <x:v>Composite assessment + qualification</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>Staff Admin</x:v>
+        <x:v>Consultant / Firm</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>Route accounts internally without showing labels to clients</x:v>
+        <x:v>Track evidence, third-party assessments and qualification</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
-        <x:v>Type A/B/C and account-label mapping to CL1–CL4 / Track A/B</x:v>
+        <x:v>Weights, modalities, committee role, firm 0–3 / 4–7 / &gt;7 meaning</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
         <x:v>Needs clarification</x:v>
@@ -4678,19 +4750,19 @@
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" s="13" t="str">
-        <x:v>Phase 2B</x:v>
+        <x:v>Phase 2A</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
-        <x:v>Requirements, opportunities and matching</x:v>
+        <x:v>Client categorisation operations</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
-        <x:v>Client / Consultant / Firm</x:v>
+        <x:v>Staff Admin</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
-        <x:v>Client demand, masked profiles, Firm Seller/Buyer/Win-and-Staff</x:v>
+        <x:v>Route accounts internally without showing labels to clients</x:v>
       </x:c>
       <x:c r="E11" s="13" t="str">
-        <x:v>Search access, matching, masking, shortlist and reservation rules</x:v>
+        <x:v>Type A/B/C and account-label mapping to CL1–CL4 / Track A/B</x:v>
       </x:c>
       <x:c r="F11" s="13" t="str">
         <x:v>Needs clarification</x:v>
@@ -4698,19 +4770,19 @@
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>Phase 2C</x:v>
+        <x:v>Phase 2B</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
-        <x:v>Tender and e-evaluation</x:v>
+        <x:v>Requirements, opportunities and matching</x:v>
       </x:c>
       <x:c r="C12" s="13" t="str">
-        <x:v>Client / Firm / Staff</x:v>
+        <x:v>Client / Consultant / Firm</x:v>
       </x:c>
       <x:c r="D12" s="13" t="str">
-        <x:v>TOR, bids, technical and financial review, QCBS decision</x:v>
+        <x:v>Client demand, masked profiles, Firm Seller/Buyer/Win-and-Staff</x:v>
       </x:c>
       <x:c r="E12" s="13" t="str">
-        <x:v>TOR fields, weights, formula, evaluator and decision rights</x:v>
+        <x:v>Search access, matching, masking, shortlist and reservation rules</x:v>
       </x:c>
       <x:c r="F12" s="13" t="str">
         <x:v>Needs clarification</x:v>
@@ -4721,16 +4793,16 @@
         <x:v>Phase 2C</x:v>
       </x:c>
       <x:c r="B13" s="13" t="str">
-        <x:v>Agreements, award and introduction</x:v>
+        <x:v>Tender and e-evaluation</x:v>
       </x:c>
       <x:c r="C13" s="13" t="str">
-        <x:v>All audiences</x:v>
+        <x:v>Client / Firm / Staff</x:v>
       </x:c>
       <x:c r="D13" s="13" t="str">
-        <x:v>Signed agreement gate before award and introduction</x:v>
+        <x:v>TOR, bids, technical and financial review, QCBS decision</x:v>
       </x:c>
       <x:c r="E13" s="13" t="str">
-        <x:v>Document types, signers, LOI order, payment and identity release</x:v>
+        <x:v>TOR fields, weights, formula, evaluator and decision rights</x:v>
       </x:c>
       <x:c r="F13" s="13" t="str">
         <x:v>Needs clarification</x:v>
@@ -4738,19 +4810,19 @@
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="13" t="str">
-        <x:v>Phase 2D</x:v>
+        <x:v>Phase 2C</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
-        <x:v>Engagement and performance</x:v>
+        <x:v>Agreements, award and introduction</x:v>
       </x:c>
       <x:c r="C14" s="13" t="str">
         <x:v>All audiences</x:v>
       </x:c>
       <x:c r="D14" s="13" t="str">
-        <x:v>Concurrent assignments, milestones and project-specific feedback</x:v>
+        <x:v>Signed agreement gate before award and introduction</x:v>
       </x:c>
       <x:c r="E14" s="13" t="str">
-        <x:v>Feedback impact on composite versus separate performance signal</x:v>
+        <x:v>Document types, signers, LOI order, payment and identity release</x:v>
       </x:c>
       <x:c r="F14" s="13" t="str">
         <x:v>Needs clarification</x:v>
@@ -4761,38 +4833,58 @@
         <x:v>Phase 2D</x:v>
       </x:c>
       <x:c r="B15" s="13" t="str">
+        <x:v>Engagement and performance</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>All audiences</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>Concurrent assignments, milestones and project-specific feedback</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>Feedback impact on composite versus separate performance signal</x:v>
+      </x:c>
+      <x:c r="F15" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="13" t="str">
+        <x:v>Phase 2D</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
         <x:v>Finance, communication and knowledge</x:v>
       </x:c>
-      <x:c r="C15" s="13" t="str">
+      <x:c r="C16" s="13" t="str">
         <x:v>All audiences / Staff</x:v>
       </x:c>
-      <x:c r="D15" s="13" t="str">
+      <x:c r="D16" s="13" t="str">
         <x:v>Billing, notifications, calendar, files and controlled reuse</x:v>
       </x:c>
-      <x:c r="E15" s="13" t="str">
+      <x:c r="E16" s="13" t="str">
         <x:v>Fees, providers, consent, rights, retention and case-study approval</x:v>
       </x:c>
-      <x:c r="F15" s="13" t="str">
-        <x:v>Needs clarification</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="58" customHeight="1">
-      <x:c r="A16" s="14" t="str">
+      <x:c r="F16" s="13" t="str">
+        <x:v>Needs clarification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="14" t="str">
         <x:v>Phase 2D</x:v>
       </x:c>
-      <x:c r="B16" s="14" t="str">
+      <x:c r="B17" s="14" t="str">
         <x:v>Staff team work queues</x:v>
       </x:c>
-      <x:c r="C16" s="14" t="str">
+      <x:c r="C17" s="14" t="str">
         <x:v>Staff Admin</x:v>
       </x:c>
-      <x:c r="D16" s="14" t="str">
+      <x:c r="D17" s="14" t="str">
         <x:v>Role-based operations and Master Admin final approval</x:v>
       </x:c>
-      <x:c r="E16" s="14" t="str">
+      <x:c r="E17" s="14" t="str">
         <x:v>Team queue items, authority and record visibility</x:v>
       </x:c>
-      <x:c r="F16" s="14" t="str">
+      <x:c r="F17" s="14" t="str">
         <x:v>Needs clarification</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Use neutral step labels across CTQ forms
</commit_message>
<xml_diff>
--- a/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
+++ b/OptimIQ_Portal_Screen_Approval_Inventory.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra5bc95f2ca5d4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="Ra1545dc3659e4b98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="R2abca8c2fa0744f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="R1fa49e33182441f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="R0a23948743144d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="Rf64f82d086404297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R0ee9d5779f584264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="R2b3311059ea34a6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="9" r:id="Re49ddab2e5264cd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6defbca9c9b648a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Access" sheetId="2" r:id="R075330b62c2048f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consultant" sheetId="3" r:id="R1045ad6a4533435c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Firm" sheetId="4" r:id="Re3fef7dfb9d94e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="5" r:id="R392daf8c5f0e41ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Admin" sheetId="6" r:id="R4d8c13fe3a644d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Clarifications" sheetId="7" r:id="R84ed0a4c03b24c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme &amp; Review" sheetId="8" r:id="Ra809add163ff45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="9" r:id="R77e230f7ffa34800"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1147,7 +1147,8 @@
         <x:v>Pending client approval</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
-        <x:v>Design updated (2026-10-20): one shared CTQ form, no score or weighting shown; backend determines fit categories after submission.</x:v>
+        <x:v>Design updated (2026-10-20): one shared CTQ form, no score or weighting shown; backend determines fit categories after submission.
+UX update (2026-10-26): CTQ navigation, progress and question-group headings use neutral Step 1, Step 2, etc. Process-category titles and descriptions are hidden on the member form. Question wording and rules are unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -1812,7 +1813,8 @@
         <x:v>Awaiting client feedback</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
-        <x:v>CTA is the separate prior registration step; client confirmed the CTQ is six sections. Do not show internal IDs, weights, or raw score.</x:v>
+        <x:v>CTA is the separate prior registration step; client confirmed the CTQ is six sections. Do not show internal IDs, weights, or raw score.
+UX update (2026-10-26): CTQ navigation, progress and question-group headings use neutral Step 1, Step 2, etc. Process-category titles and descriptions are hidden on the member form. Question wording and rules are unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -2483,7 +2485,8 @@
         <x:v>Awaiting screen feedback</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
-        <x:v>Client feedback defines this optional enrichment screen as the Client CTQ.</x:v>
+        <x:v>Client feedback defines this optional enrichment screen as the Client CTQ.
+UX update (2026-10-26): CTQ navigation, progress and question-group headings use neutral Step 1, Step 2, etc. Process-category titles and descriptions are hidden on the member form. Question wording and rules are unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">

</xml_diff>